<commit_message>
[PowerPoint] (Shape) Add snippet that gets Base64 image
</commit_message>
<xml_diff>
--- a/snippet-extractor-metadata/powerpoint.xlsx
+++ b/snippet-extractor-metadata/powerpoint.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{995B1E0C-ED6E-4740-AEB3-BEC61464CEDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7C414EC-35C0-4625-9957-123F9D615DF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{CB5595D7-4492-4192-A1C1-2583BA1957AA}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25180" windowHeight="16140" xr2:uid="{CB5595D7-4492-4192-A1C1-2583BA1957AA}"/>
   </bookViews>
   <sheets>
     <sheet name="Snippets" sheetId="2" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="816" uniqueCount="210">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="831" uniqueCount="215">
   <si>
     <t>Class</t>
   </si>
@@ -650,6 +650,21 @@
   </si>
   <si>
     <t>updateHyperlinkOnShape</t>
+  </si>
+  <si>
+    <t>ShapeGetImageOptions</t>
+  </si>
+  <si>
+    <t>powerpoint-shapes-get-shape-as-image</t>
+  </si>
+  <si>
+    <t>getImageWithAllOptions</t>
+  </si>
+  <si>
+    <t>getImageDefault</t>
+  </si>
+  <si>
+    <t>ShapeGetImageFormatType</t>
   </si>
 </sst>
 </file>
@@ -730,10 +745,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{78C585A5-D505-49C6-9CA1-8E6558948317}" name="Snippets" displayName="Snippets" ref="A1:F163" totalsRowShown="0" headerRowDxfId="4">
-  <autoFilter ref="A1:F163" xr:uid="{EAC65D03-FDD2-4352-A5F3-1CDEDE6251B2}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F159">
-    <sortCondition ref="B1:B159"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{78C585A5-D505-49C6-9CA1-8E6558948317}" name="Snippets" displayName="Snippets" ref="A1:F166" totalsRowShown="0" headerRowDxfId="4">
+  <autoFilter ref="A1:F166" xr:uid="{EAC65D03-FDD2-4352-A5F3-1CDEDE6251B2}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F162">
+    <sortCondition ref="B1:B162"/>
   </sortState>
   <tableColumns count="6">
     <tableColumn id="6" xr3:uid="{408888B8-C1DD-4B51-B1EB-5663F091D142}" name="Package"/>
@@ -1044,19 +1059,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{809930CD-A227-47DC-AAA4-BB816AEDEB59}">
-  <dimension ref="A1:F163"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:F166"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="26.5546875" customWidth="1"/>
-    <col min="3" max="3" width="26.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.54296875" customWidth="1"/>
+    <col min="3" max="3" width="26.54296875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="23" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="42.77734375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="42.81640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="55" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="31" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>31</v>
       </c>
@@ -1076,7 +1091,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>32</v>
       </c>
@@ -1093,7 +1108,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>32</v>
       </c>
@@ -1110,7 +1125,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>32</v>
       </c>
@@ -1130,7 +1145,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>32</v>
       </c>
@@ -1147,7 +1162,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>32</v>
       </c>
@@ -1167,7 +1182,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>32</v>
       </c>
@@ -1187,7 +1202,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>32</v>
       </c>
@@ -1204,7 +1219,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>32</v>
       </c>
@@ -1221,7 +1236,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>32</v>
       </c>
@@ -1238,7 +1253,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>32</v>
       </c>
@@ -1255,7 +1270,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>32</v>
       </c>
@@ -1272,7 +1287,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>32</v>
       </c>
@@ -1289,7 +1304,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>32</v>
       </c>
@@ -1306,7 +1321,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>32</v>
       </c>
@@ -1323,7 +1338,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>32</v>
       </c>
@@ -1340,7 +1355,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>32</v>
       </c>
@@ -1357,7 +1372,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>32</v>
       </c>
@@ -1374,7 +1389,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>32</v>
       </c>
@@ -1391,7 +1406,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>32</v>
       </c>
@@ -1408,7 +1423,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>32</v>
       </c>
@@ -1425,7 +1440,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>32</v>
       </c>
@@ -1442,7 +1457,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>32</v>
       </c>
@@ -1459,7 +1474,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>32</v>
       </c>
@@ -1476,7 +1491,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>32</v>
       </c>
@@ -1493,14 +1508,14 @@
         <v>102</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>32</v>
       </c>
       <c r="B26" t="s">
         <v>100</v>
       </c>
-      <c r="C26" s="2" t="s">
+      <c r="C26" t="s">
         <v>20</v>
       </c>
       <c r="D26">
@@ -1509,11 +1524,11 @@
       <c r="E26" t="s">
         <v>103</v>
       </c>
-      <c r="F26" s="2" t="s">
+      <c r="F26" t="s">
         <v>207</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>32</v>
       </c>
@@ -1530,7 +1545,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>32</v>
       </c>
@@ -1547,7 +1562,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>32</v>
       </c>
@@ -1564,7 +1579,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>32</v>
       </c>
@@ -1581,7 +1596,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>32</v>
       </c>
@@ -1598,7 +1613,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>32</v>
       </c>
@@ -1615,7 +1630,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>32</v>
       </c>
@@ -1632,7 +1647,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>32</v>
       </c>
@@ -1649,7 +1664,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>32</v>
       </c>
@@ -1666,7 +1681,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>32</v>
       </c>
@@ -1686,7 +1701,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>32</v>
       </c>
@@ -1706,7 +1721,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>32</v>
       </c>
@@ -1726,7 +1741,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>32</v>
       </c>
@@ -1746,7 +1761,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>32</v>
       </c>
@@ -1766,7 +1781,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>32</v>
       </c>
@@ -1786,7 +1801,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>32</v>
       </c>
@@ -1806,7 +1821,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>32</v>
       </c>
@@ -1826,7 +1841,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>32</v>
       </c>
@@ -1846,7 +1861,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>32</v>
       </c>
@@ -1866,7 +1881,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>32</v>
       </c>
@@ -1886,7 +1901,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>32</v>
       </c>
@@ -1903,7 +1918,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>32</v>
       </c>
@@ -1920,7 +1935,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>32</v>
       </c>
@@ -1940,47 +1955,47 @@
         <v>96</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>32</v>
       </c>
       <c r="B50" t="s">
         <v>45</v>
       </c>
-      <c r="C50" t="s">
-        <v>161</v>
+      <c r="C50" s="2" t="s">
+        <v>106</v>
       </c>
       <c r="D50">
         <v>1</v>
       </c>
-      <c r="E50" t="s">
-        <v>116</v>
-      </c>
-      <c r="F50" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E50" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="F50" s="2" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>32</v>
       </c>
       <c r="B51" t="s">
         <v>45</v>
       </c>
-      <c r="C51" s="2" t="s">
-        <v>208</v>
+      <c r="C51" t="s">
+        <v>161</v>
       </c>
       <c r="D51">
         <v>1</v>
       </c>
-      <c r="E51" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="F51" s="2" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E51" t="s">
+        <v>116</v>
+      </c>
+      <c r="F51" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>32</v>
       </c>
@@ -1988,19 +2003,19 @@
         <v>45</v>
       </c>
       <c r="C52" t="s">
-        <v>176</v>
+        <v>208</v>
       </c>
       <c r="D52">
         <v>1</v>
       </c>
       <c r="E52" t="s">
-        <v>168</v>
+        <v>103</v>
       </c>
       <c r="F52" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>32</v>
       </c>
@@ -2008,16 +2023,19 @@
         <v>45</v>
       </c>
       <c r="C53" t="s">
-        <v>58</v>
+        <v>176</v>
+      </c>
+      <c r="D53">
+        <v>1</v>
       </c>
       <c r="E53" t="s">
-        <v>53</v>
+        <v>168</v>
       </c>
       <c r="F53" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>32</v>
       </c>
@@ -2025,16 +2043,16 @@
         <v>45</v>
       </c>
       <c r="C54" t="s">
-        <v>108</v>
+        <v>58</v>
       </c>
       <c r="E54" t="s">
-        <v>109</v>
+        <v>53</v>
       </c>
       <c r="F54" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>32</v>
       </c>
@@ -2042,16 +2060,16 @@
         <v>45</v>
       </c>
       <c r="C55" t="s">
-        <v>52</v>
+        <v>108</v>
       </c>
       <c r="E55" t="s">
-        <v>53</v>
+        <v>109</v>
       </c>
       <c r="F55" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>32</v>
       </c>
@@ -2059,7 +2077,7 @@
         <v>45</v>
       </c>
       <c r="C56" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="E56" t="s">
         <v>53</v>
@@ -2068,7 +2086,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>32</v>
       </c>
@@ -2076,16 +2094,16 @@
         <v>45</v>
       </c>
       <c r="C57" t="s">
-        <v>196</v>
+        <v>49</v>
       </c>
       <c r="E57" t="s">
-        <v>85</v>
+        <v>53</v>
       </c>
       <c r="F57" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>32</v>
       </c>
@@ -2093,16 +2111,16 @@
         <v>45</v>
       </c>
       <c r="C58" t="s">
-        <v>50</v>
+        <v>196</v>
       </c>
       <c r="E58" t="s">
-        <v>53</v>
+        <v>85</v>
       </c>
       <c r="F58" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.3">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>32</v>
       </c>
@@ -2110,16 +2128,16 @@
         <v>45</v>
       </c>
       <c r="C59" t="s">
-        <v>86</v>
+        <v>50</v>
       </c>
       <c r="E59" t="s">
-        <v>85</v>
+        <v>53</v>
       </c>
       <c r="F59" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.3">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>32</v>
       </c>
@@ -2127,16 +2145,16 @@
         <v>45</v>
       </c>
       <c r="C60" t="s">
-        <v>51</v>
+        <v>86</v>
       </c>
       <c r="E60" t="s">
-        <v>53</v>
+        <v>85</v>
       </c>
       <c r="F60" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.3">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>32</v>
       </c>
@@ -2144,87 +2162,84 @@
         <v>45</v>
       </c>
       <c r="C61" t="s">
+        <v>51</v>
+      </c>
+      <c r="E61" t="s">
+        <v>53</v>
+      </c>
+      <c r="F61" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A62" t="s">
+        <v>32</v>
+      </c>
+      <c r="B62" t="s">
+        <v>45</v>
+      </c>
+      <c r="C62" t="s">
         <v>178</v>
       </c>
-      <c r="E61" t="s">
+      <c r="E62" t="s">
         <v>168</v>
       </c>
-      <c r="F61" t="s">
+      <c r="F62" t="s">
         <v>177</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A62" t="s">
-        <v>32</v>
-      </c>
-      <c r="B62" t="s">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A63" t="s">
+        <v>32</v>
+      </c>
+      <c r="B63" t="s">
         <v>95</v>
       </c>
-      <c r="D62" t="s">
+      <c r="D63" t="s">
         <v>68</v>
-      </c>
-      <c r="E62" t="s">
-        <v>24</v>
-      </c>
-      <c r="F62" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A63" t="s">
-        <v>32</v>
-      </c>
-      <c r="B63" t="s">
-        <v>187</v>
-      </c>
-      <c r="D63" t="s">
-        <v>65</v>
       </c>
       <c r="E63" t="s">
         <v>24</v>
       </c>
       <c r="F63" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A64" t="s">
+        <v>32</v>
+      </c>
+      <c r="B64" t="s">
+        <v>187</v>
+      </c>
+      <c r="D64" t="s">
+        <v>65</v>
+      </c>
+      <c r="E64" t="s">
+        <v>24</v>
+      </c>
+      <c r="F64" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A64" t="s">
-        <v>32</v>
-      </c>
-      <c r="B64" t="s">
-        <v>21</v>
-      </c>
-      <c r="D64" t="s">
-        <v>87</v>
-      </c>
-      <c r="E64" t="s">
-        <v>85</v>
-      </c>
-      <c r="F64" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>32</v>
       </c>
       <c r="B65" t="s">
         <v>21</v>
       </c>
-      <c r="C65" t="s">
-        <v>25</v>
-      </c>
-      <c r="D65">
-        <v>1</v>
+      <c r="D65" t="s">
+        <v>87</v>
       </c>
       <c r="E65" t="s">
-        <v>24</v>
+        <v>85</v>
       </c>
       <c r="F65" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.3">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>32</v>
       </c>
@@ -2232,19 +2247,19 @@
         <v>21</v>
       </c>
       <c r="C66" t="s">
-        <v>111</v>
+        <v>25</v>
       </c>
       <c r="D66">
         <v>1</v>
       </c>
       <c r="E66" t="s">
-        <v>109</v>
+        <v>24</v>
       </c>
       <c r="F66" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>32</v>
       </c>
@@ -2252,19 +2267,19 @@
         <v>21</v>
       </c>
       <c r="C67" t="s">
-        <v>27</v>
+        <v>111</v>
       </c>
       <c r="D67">
         <v>1</v>
       </c>
       <c r="E67" t="s">
-        <v>24</v>
+        <v>109</v>
       </c>
       <c r="F67" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>32</v>
       </c>
@@ -2272,19 +2287,19 @@
         <v>21</v>
       </c>
       <c r="C68" t="s">
-        <v>115</v>
+        <v>27</v>
       </c>
       <c r="D68">
         <v>1</v>
       </c>
       <c r="E68" t="s">
-        <v>116</v>
+        <v>24</v>
       </c>
       <c r="F68" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.3">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>32</v>
       </c>
@@ -2292,19 +2307,19 @@
         <v>21</v>
       </c>
       <c r="C69" t="s">
-        <v>29</v>
+        <v>115</v>
       </c>
       <c r="D69">
         <v>1</v>
       </c>
       <c r="E69" t="s">
-        <v>24</v>
+        <v>116</v>
       </c>
       <c r="F69" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.3">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>32</v>
       </c>
@@ -2312,19 +2327,19 @@
         <v>21</v>
       </c>
       <c r="C70" t="s">
-        <v>91</v>
+        <v>29</v>
       </c>
       <c r="D70">
         <v>1</v>
       </c>
       <c r="E70" t="s">
-        <v>116</v>
+        <v>24</v>
       </c>
       <c r="F70" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>32</v>
       </c>
@@ -2332,19 +2347,19 @@
         <v>21</v>
       </c>
       <c r="C71" t="s">
-        <v>16</v>
+        <v>91</v>
       </c>
       <c r="D71">
         <v>1</v>
       </c>
       <c r="E71" t="s">
-        <v>14</v>
+        <v>116</v>
       </c>
       <c r="F71" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.3">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>32</v>
       </c>
@@ -2352,27 +2367,30 @@
         <v>21</v>
       </c>
       <c r="C72" t="s">
+        <v>16</v>
+      </c>
+      <c r="D72">
+        <v>1</v>
+      </c>
+      <c r="E72" t="s">
+        <v>14</v>
+      </c>
+      <c r="F72" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A73" t="s">
+        <v>32</v>
+      </c>
+      <c r="B73" t="s">
+        <v>21</v>
+      </c>
+      <c r="C73" t="s">
         <v>70</v>
       </c>
-      <c r="D72">
+      <c r="D73">
         <v>2</v>
-      </c>
-      <c r="E72" t="s">
-        <v>85</v>
-      </c>
-      <c r="F72" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A73" t="s">
-        <v>32</v>
-      </c>
-      <c r="B73" t="s">
-        <v>59</v>
-      </c>
-      <c r="D73" t="s">
-        <v>87</v>
       </c>
       <c r="E73" t="s">
         <v>85</v>
@@ -2381,27 +2399,24 @@
         <v>81</v>
       </c>
     </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>32</v>
       </c>
       <c r="B74" t="s">
         <v>59</v>
       </c>
-      <c r="C74" t="s">
-        <v>179</v>
-      </c>
-      <c r="D74">
-        <v>1</v>
+      <c r="D74" t="s">
+        <v>87</v>
       </c>
       <c r="E74" t="s">
-        <v>168</v>
+        <v>85</v>
       </c>
       <c r="F74" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.3">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>32</v>
       </c>
@@ -2409,19 +2424,19 @@
         <v>59</v>
       </c>
       <c r="C75" t="s">
-        <v>60</v>
+        <v>179</v>
       </c>
       <c r="D75">
         <v>1</v>
       </c>
       <c r="E75" t="s">
-        <v>53</v>
+        <v>168</v>
       </c>
       <c r="F75" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.3">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>32</v>
       </c>
@@ -2429,16 +2444,19 @@
         <v>59</v>
       </c>
       <c r="C76" t="s">
-        <v>93</v>
+        <v>60</v>
+      </c>
+      <c r="D76">
+        <v>1</v>
       </c>
       <c r="E76" t="s">
         <v>53</v>
       </c>
       <c r="F76" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.3">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>32</v>
       </c>
@@ -2446,16 +2464,16 @@
         <v>59</v>
       </c>
       <c r="C77" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="E77" t="s">
-        <v>85</v>
+        <v>53</v>
       </c>
       <c r="F77" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.3">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
         <v>32</v>
       </c>
@@ -2463,24 +2481,24 @@
         <v>59</v>
       </c>
       <c r="C78" t="s">
+        <v>82</v>
+      </c>
+      <c r="E78" t="s">
+        <v>85</v>
+      </c>
+      <c r="F78" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A79" t="s">
+        <v>32</v>
+      </c>
+      <c r="B79" t="s">
+        <v>59</v>
+      </c>
+      <c r="C79" t="s">
         <v>86</v>
-      </c>
-      <c r="E78" t="s">
-        <v>53</v>
-      </c>
-      <c r="F78" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A79" t="s">
-        <v>32</v>
-      </c>
-      <c r="B79" t="s">
-        <v>189</v>
-      </c>
-      <c r="D79" t="s">
-        <v>65</v>
       </c>
       <c r="E79" t="s">
         <v>53</v>
@@ -2489,41 +2507,41 @@
         <v>44</v>
       </c>
     </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
         <v>32</v>
       </c>
       <c r="B80" t="s">
-        <v>61</v>
+        <v>189</v>
       </c>
       <c r="D80" t="s">
-        <v>87</v>
+        <v>65</v>
       </c>
       <c r="E80" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F80" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.3">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
         <v>32</v>
       </c>
       <c r="B81" t="s">
         <v>61</v>
       </c>
-      <c r="C81" t="s">
-        <v>62</v>
+      <c r="D81" t="s">
+        <v>87</v>
       </c>
       <c r="E81" t="s">
         <v>54</v>
       </c>
       <c r="F81" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.3">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
         <v>32</v>
       </c>
@@ -2531,24 +2549,24 @@
         <v>61</v>
       </c>
       <c r="C82" t="s">
+        <v>62</v>
+      </c>
+      <c r="E82" t="s">
+        <v>54</v>
+      </c>
+      <c r="F82" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A83" t="s">
+        <v>32</v>
+      </c>
+      <c r="B83" t="s">
+        <v>61</v>
+      </c>
+      <c r="C83" t="s">
         <v>190</v>
-      </c>
-      <c r="E82" t="s">
-        <v>24</v>
-      </c>
-      <c r="F82" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A83" t="s">
-        <v>32</v>
-      </c>
-      <c r="B83" t="s">
-        <v>188</v>
-      </c>
-      <c r="D83" t="s">
-        <v>65</v>
       </c>
       <c r="E83" t="s">
         <v>24</v>
@@ -2557,140 +2575,139 @@
         <v>89</v>
       </c>
     </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
         <v>32</v>
       </c>
       <c r="B84" t="s">
+        <v>188</v>
+      </c>
+      <c r="D84" t="s">
+        <v>65</v>
+      </c>
+      <c r="E84" t="s">
+        <v>24</v>
+      </c>
+      <c r="F84" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A85" t="s">
+        <v>32</v>
+      </c>
+      <c r="B85" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="C85" s="2"/>
+      <c r="D85" t="s">
+        <v>65</v>
+      </c>
+      <c r="E85" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="F85" s="2" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A86" t="s">
+        <v>32</v>
+      </c>
+      <c r="B86" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="C86" s="2"/>
+      <c r="D86" t="s">
+        <v>68</v>
+      </c>
+      <c r="E86" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="F86" s="2" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A87" t="s">
+        <v>32</v>
+      </c>
+      <c r="B87" t="s">
         <v>113</v>
-      </c>
-      <c r="D84" t="s">
-        <v>87</v>
-      </c>
-      <c r="E84" t="s">
-        <v>109</v>
-      </c>
-      <c r="F84" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A85" t="s">
-        <v>32</v>
-      </c>
-      <c r="B85" t="s">
-        <v>113</v>
-      </c>
-      <c r="C85" t="s">
-        <v>114</v>
-      </c>
-      <c r="D85">
-        <v>1</v>
-      </c>
-      <c r="E85" t="s">
-        <v>109</v>
-      </c>
-      <c r="F85" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A86" t="s">
-        <v>32</v>
-      </c>
-      <c r="B86" t="s">
-        <v>80</v>
-      </c>
-      <c r="D86" t="s">
-        <v>65</v>
-      </c>
-      <c r="E86" t="s">
-        <v>85</v>
-      </c>
-      <c r="F86" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A87" t="s">
-        <v>32</v>
-      </c>
-      <c r="B87" t="s">
-        <v>83</v>
       </c>
       <c r="D87" t="s">
         <v>87</v>
       </c>
       <c r="E87" t="s">
+        <v>109</v>
+      </c>
+      <c r="F87" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A88" t="s">
+        <v>32</v>
+      </c>
+      <c r="B88" t="s">
+        <v>113</v>
+      </c>
+      <c r="C88" t="s">
+        <v>114</v>
+      </c>
+      <c r="D88">
+        <v>1</v>
+      </c>
+      <c r="E88" t="s">
+        <v>109</v>
+      </c>
+      <c r="F88" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A89" t="s">
+        <v>32</v>
+      </c>
+      <c r="B89" t="s">
+        <v>80</v>
+      </c>
+      <c r="D89" t="s">
+        <v>65</v>
+      </c>
+      <c r="E89" t="s">
         <v>85</v>
       </c>
-      <c r="F87" t="s">
+      <c r="F89" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A88" t="s">
-        <v>32</v>
-      </c>
-      <c r="B88" t="s">
+    <row r="90" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A90" t="s">
+        <v>32</v>
+      </c>
+      <c r="B90" t="s">
         <v>83</v>
       </c>
-      <c r="C88" t="s">
+      <c r="D90" t="s">
+        <v>87</v>
+      </c>
+      <c r="E90" t="s">
+        <v>85</v>
+      </c>
+      <c r="F90" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A91" t="s">
+        <v>32</v>
+      </c>
+      <c r="B91" t="s">
+        <v>83</v>
+      </c>
+      <c r="C91" t="s">
         <v>84</v>
-      </c>
-      <c r="E88" t="s">
-        <v>85</v>
-      </c>
-      <c r="F88" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A89" t="s">
-        <v>32</v>
-      </c>
-      <c r="B89" t="s">
-        <v>90</v>
-      </c>
-      <c r="D89" t="s">
-        <v>87</v>
-      </c>
-      <c r="E89" t="s">
-        <v>53</v>
-      </c>
-      <c r="F89" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A90" t="s">
-        <v>32</v>
-      </c>
-      <c r="B90" t="s">
-        <v>90</v>
-      </c>
-      <c r="C90" t="s">
-        <v>91</v>
-      </c>
-      <c r="D90">
-        <v>1</v>
-      </c>
-      <c r="E90" t="s">
-        <v>53</v>
-      </c>
-      <c r="F90" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A91" t="s">
-        <v>32</v>
-      </c>
-      <c r="B91" t="s">
-        <v>78</v>
-      </c>
-      <c r="D91" t="s">
-        <v>65</v>
       </c>
       <c r="E91" t="s">
         <v>85</v>
@@ -2699,118 +2716,112 @@
         <v>79</v>
       </c>
     </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
         <v>32</v>
       </c>
       <c r="B92" t="s">
+        <v>90</v>
+      </c>
+      <c r="D92" t="s">
+        <v>87</v>
+      </c>
+      <c r="E92" t="s">
+        <v>53</v>
+      </c>
+      <c r="F92" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A93" t="s">
+        <v>32</v>
+      </c>
+      <c r="B93" t="s">
+        <v>90</v>
+      </c>
+      <c r="C93" t="s">
+        <v>91</v>
+      </c>
+      <c r="D93">
+        <v>1</v>
+      </c>
+      <c r="E93" t="s">
+        <v>53</v>
+      </c>
+      <c r="F93" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A94" t="s">
+        <v>32</v>
+      </c>
+      <c r="B94" t="s">
+        <v>78</v>
+      </c>
+      <c r="D94" t="s">
+        <v>65</v>
+      </c>
+      <c r="E94" t="s">
+        <v>85</v>
+      </c>
+      <c r="F94" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A95" t="s">
+        <v>32</v>
+      </c>
+      <c r="B95" t="s">
         <v>180</v>
       </c>
-      <c r="D92" t="s">
+      <c r="D95" t="s">
         <v>65</v>
       </c>
-      <c r="E92" t="s">
+      <c r="E95" t="s">
         <v>168</v>
       </c>
-      <c r="F92" t="s">
+      <c r="F95" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A93" t="s">
-        <v>32</v>
-      </c>
-      <c r="B93" t="s">
+    <row r="96" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A96" t="s">
+        <v>32</v>
+      </c>
+      <c r="B96" t="s">
         <v>180</v>
       </c>
-      <c r="D93" t="s">
+      <c r="D96" t="s">
         <v>65</v>
       </c>
-      <c r="E93" t="s">
+      <c r="E96" t="s">
         <v>168</v>
       </c>
-      <c r="F93" t="s">
+      <c r="F96" t="s">
         <v>177</v>
       </c>
     </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A94" t="s">
-        <v>32</v>
-      </c>
-      <c r="B94" t="s">
-        <v>19</v>
-      </c>
-      <c r="D94" t="s">
-        <v>87</v>
-      </c>
-      <c r="E94" t="s">
-        <v>53</v>
-      </c>
-      <c r="F94" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A95" t="s">
-        <v>32</v>
-      </c>
-      <c r="B95" t="s">
-        <v>19</v>
-      </c>
-      <c r="C95" t="s">
-        <v>20</v>
-      </c>
-      <c r="D95">
-        <v>1</v>
-      </c>
-      <c r="E95" t="s">
-        <v>40</v>
-      </c>
-      <c r="F95" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A96" t="s">
-        <v>32</v>
-      </c>
-      <c r="B96" t="s">
-        <v>19</v>
-      </c>
-      <c r="C96" t="s">
-        <v>104</v>
-      </c>
-      <c r="D96">
-        <v>1</v>
-      </c>
-      <c r="E96" t="s">
-        <v>105</v>
-      </c>
-      <c r="F96" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
         <v>32</v>
       </c>
       <c r="B97" t="s">
         <v>19</v>
       </c>
-      <c r="C97" t="s">
-        <v>106</v>
-      </c>
-      <c r="D97">
-        <v>1</v>
+      <c r="D97" t="s">
+        <v>87</v>
       </c>
       <c r="E97" t="s">
-        <v>105</v>
+        <v>53</v>
       </c>
       <c r="F97" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.3">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A98" t="s">
         <v>32</v>
       </c>
@@ -2818,19 +2829,19 @@
         <v>19</v>
       </c>
       <c r="C98" t="s">
-        <v>38</v>
+        <v>20</v>
       </c>
       <c r="D98">
         <v>1</v>
       </c>
       <c r="E98" t="s">
-        <v>53</v>
+        <v>40</v>
       </c>
       <c r="F98" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.3">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A99" t="s">
         <v>32</v>
       </c>
@@ -2838,19 +2849,19 @@
         <v>19</v>
       </c>
       <c r="C99" t="s">
-        <v>38</v>
+        <v>104</v>
       </c>
       <c r="D99">
         <v>1</v>
       </c>
       <c r="E99" t="s">
-        <v>53</v>
+        <v>105</v>
       </c>
       <c r="F99" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.3">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A100" t="s">
         <v>32</v>
       </c>
@@ -2858,152 +2869,158 @@
         <v>19</v>
       </c>
       <c r="C100" t="s">
+        <v>106</v>
+      </c>
+      <c r="D100">
+        <v>1</v>
+      </c>
+      <c r="E100" t="s">
+        <v>105</v>
+      </c>
+      <c r="F100" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A101" t="s">
+        <v>32</v>
+      </c>
+      <c r="B101" t="s">
+        <v>19</v>
+      </c>
+      <c r="C101" t="s">
+        <v>38</v>
+      </c>
+      <c r="D101">
+        <v>1</v>
+      </c>
+      <c r="E101" t="s">
+        <v>53</v>
+      </c>
+      <c r="F101" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A102" t="s">
+        <v>32</v>
+      </c>
+      <c r="B102" t="s">
+        <v>19</v>
+      </c>
+      <c r="C102" t="s">
+        <v>38</v>
+      </c>
+      <c r="D102">
+        <v>1</v>
+      </c>
+      <c r="E102" t="s">
+        <v>53</v>
+      </c>
+      <c r="F102" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A103" t="s">
+        <v>32</v>
+      </c>
+      <c r="B103" t="s">
+        <v>19</v>
+      </c>
+      <c r="C103" t="s">
         <v>206</v>
       </c>
-      <c r="E100" t="s">
+      <c r="E103" t="s">
         <v>103</v>
       </c>
-      <c r="F100" t="s">
+      <c r="F103" t="s">
         <v>204</v>
       </c>
     </row>
-    <row r="101" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A101" t="s">
-        <v>32</v>
-      </c>
-      <c r="B101" t="s">
+    <row r="104" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A104" t="s">
+        <v>32</v>
+      </c>
+      <c r="B104" t="s">
         <v>9</v>
       </c>
-      <c r="D101" t="s">
+      <c r="D104" t="s">
         <v>87</v>
       </c>
-      <c r="E101" t="s">
+      <c r="E104" t="s">
         <v>11</v>
       </c>
-      <c r="F101" t="s">
+      <c r="F104" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="102" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A102" t="s">
-        <v>32</v>
-      </c>
-      <c r="B102" t="s">
+    <row r="105" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A105" t="s">
+        <v>32</v>
+      </c>
+      <c r="B105" t="s">
         <v>9</v>
       </c>
-      <c r="C102" t="s">
+      <c r="C105" t="s">
         <v>10</v>
       </c>
-      <c r="D102">
-        <v>1</v>
-      </c>
-      <c r="E102" t="s">
-        <v>11</v>
-      </c>
-      <c r="F102" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="103" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A103" t="s">
-        <v>32</v>
-      </c>
-      <c r="B103" t="s">
-        <v>9</v>
-      </c>
-      <c r="C103" t="s">
-        <v>16</v>
-      </c>
-      <c r="D103">
-        <v>1</v>
-      </c>
-      <c r="E103" t="s">
-        <v>40</v>
-      </c>
-      <c r="F103" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="104" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A104" t="s">
-        <v>32</v>
-      </c>
-      <c r="B104" t="s">
-        <v>185</v>
-      </c>
-      <c r="D104" t="s">
-        <v>68</v>
-      </c>
-      <c r="E104" t="s">
-        <v>105</v>
-      </c>
-      <c r="F104" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="105" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A105" t="s">
-        <v>32</v>
-      </c>
-      <c r="B105" t="s">
-        <v>75</v>
-      </c>
-      <c r="D105" t="s">
-        <v>87</v>
+      <c r="D105">
+        <v>1</v>
       </c>
       <c r="E105" t="s">
         <v>11</v>
       </c>
       <c r="F105" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="106" spans="1:6" x14ac:dyDescent="0.3">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A106" t="s">
         <v>32</v>
       </c>
       <c r="B106" t="s">
+        <v>9</v>
+      </c>
+      <c r="C106" t="s">
+        <v>16</v>
+      </c>
+      <c r="D106">
+        <v>1</v>
+      </c>
+      <c r="E106" t="s">
+        <v>40</v>
+      </c>
+      <c r="F106" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A107" t="s">
+        <v>32</v>
+      </c>
+      <c r="B107" t="s">
+        <v>185</v>
+      </c>
+      <c r="D107" t="s">
+        <v>68</v>
+      </c>
+      <c r="E107" t="s">
+        <v>105</v>
+      </c>
+      <c r="F107" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A108" t="s">
+        <v>32</v>
+      </c>
+      <c r="B108" t="s">
         <v>75</v>
       </c>
-      <c r="C106" t="s">
-        <v>74</v>
-      </c>
-      <c r="E106" t="s">
-        <v>11</v>
-      </c>
-      <c r="F106" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="107" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A107" t="s">
-        <v>32</v>
-      </c>
-      <c r="B107" t="s">
-        <v>72</v>
-      </c>
-      <c r="D107" t="s">
+      <c r="D108" t="s">
         <v>87</v>
-      </c>
-      <c r="E107" t="s">
-        <v>11</v>
-      </c>
-      <c r="F107" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="108" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A108" t="s">
-        <v>32</v>
-      </c>
-      <c r="B108" t="s">
-        <v>72</v>
-      </c>
-      <c r="C108" t="s">
-        <v>70</v>
-      </c>
-      <c r="D108">
-        <v>2</v>
       </c>
       <c r="E108" t="s">
         <v>11</v>
@@ -3012,29 +3029,29 @@
         <v>71</v>
       </c>
     </row>
-    <row r="109" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A109" t="s">
         <v>32</v>
       </c>
       <c r="B109" t="s">
-        <v>186</v>
-      </c>
-      <c r="D109" t="s">
-        <v>65</v>
+        <v>75</v>
+      </c>
+      <c r="C109" t="s">
+        <v>74</v>
       </c>
       <c r="E109" t="s">
-        <v>85</v>
+        <v>11</v>
       </c>
       <c r="F109" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="110" spans="1:6" x14ac:dyDescent="0.3">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A110" t="s">
         <v>32</v>
       </c>
       <c r="B110" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D110" t="s">
         <v>87</v>
@@ -3046,15 +3063,18 @@
         <v>71</v>
       </c>
     </row>
-    <row r="111" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A111" t="s">
         <v>32</v>
       </c>
       <c r="B111" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C111" t="s">
-        <v>74</v>
+        <v>70</v>
+      </c>
+      <c r="D111">
+        <v>2</v>
       </c>
       <c r="E111" t="s">
         <v>11</v>
@@ -3063,35 +3083,32 @@
         <v>71</v>
       </c>
     </row>
-    <row r="112" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A112" t="s">
         <v>32</v>
       </c>
       <c r="B112" t="s">
-        <v>69</v>
+        <v>186</v>
       </c>
       <c r="D112" t="s">
+        <v>65</v>
+      </c>
+      <c r="E112" t="s">
+        <v>85</v>
+      </c>
+      <c r="F112" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A113" t="s">
+        <v>32</v>
+      </c>
+      <c r="B113" t="s">
+        <v>73</v>
+      </c>
+      <c r="D113" t="s">
         <v>87</v>
-      </c>
-      <c r="E112" t="s">
-        <v>11</v>
-      </c>
-      <c r="F112" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="113" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A113" t="s">
-        <v>32</v>
-      </c>
-      <c r="B113" t="s">
-        <v>69</v>
-      </c>
-      <c r="C113" t="s">
-        <v>70</v>
-      </c>
-      <c r="D113">
-        <v>2</v>
       </c>
       <c r="E113" t="s">
         <v>11</v>
@@ -3100,129 +3117,132 @@
         <v>71</v>
       </c>
     </row>
-    <row r="114" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A114" t="s">
         <v>32</v>
       </c>
       <c r="B114" t="s">
-        <v>92</v>
-      </c>
-      <c r="D114" t="s">
-        <v>87</v>
+        <v>73</v>
+      </c>
+      <c r="C114" t="s">
+        <v>74</v>
       </c>
       <c r="E114" t="s">
-        <v>53</v>
+        <v>11</v>
       </c>
       <c r="F114" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="115" spans="1:6" x14ac:dyDescent="0.3">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A115" t="s">
         <v>32</v>
       </c>
       <c r="B115" t="s">
-        <v>162</v>
+        <v>69</v>
       </c>
       <c r="D115" t="s">
         <v>87</v>
       </c>
       <c r="E115" t="s">
-        <v>116</v>
+        <v>11</v>
       </c>
       <c r="F115" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A116" t="s">
+        <v>32</v>
+      </c>
+      <c r="B116" t="s">
+        <v>69</v>
+      </c>
+      <c r="C116" t="s">
+        <v>70</v>
+      </c>
+      <c r="D116">
+        <v>2</v>
+      </c>
+      <c r="E116" t="s">
+        <v>11</v>
+      </c>
+      <c r="F116" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A117" t="s">
+        <v>32</v>
+      </c>
+      <c r="B117" t="s">
+        <v>92</v>
+      </c>
+      <c r="D117" t="s">
+        <v>87</v>
+      </c>
+      <c r="E117" t="s">
+        <v>53</v>
+      </c>
+      <c r="F117" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A118" t="s">
+        <v>32</v>
+      </c>
+      <c r="B118" t="s">
+        <v>162</v>
+      </c>
+      <c r="D118" t="s">
+        <v>87</v>
+      </c>
+      <c r="E118" t="s">
+        <v>116</v>
+      </c>
+      <c r="F118" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="116" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A116" t="s">
-        <v>32</v>
-      </c>
-      <c r="B116" t="s">
+    <row r="119" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A119" t="s">
+        <v>32</v>
+      </c>
+      <c r="B119" t="s">
         <v>162</v>
       </c>
-      <c r="C116" t="s">
+      <c r="C119" t="s">
         <v>164</v>
       </c>
-      <c r="D116">
-        <v>1</v>
-      </c>
-      <c r="E116" t="s">
-        <v>116</v>
-      </c>
-      <c r="F116" t="s">
+      <c r="D119">
+        <v>1</v>
+      </c>
+      <c r="E119" t="s">
+        <v>116</v>
+      </c>
+      <c r="F119" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="117" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A117" t="s">
-        <v>32</v>
-      </c>
-      <c r="B117" t="s">
-        <v>118</v>
-      </c>
-      <c r="D117" t="s">
-        <v>68</v>
-      </c>
-      <c r="E117" t="s">
-        <v>116</v>
-      </c>
-      <c r="F117" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="118" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A118" t="s">
-        <v>32</v>
-      </c>
-      <c r="B118" t="s">
-        <v>118</v>
-      </c>
-      <c r="C118" t="s">
-        <v>124</v>
-      </c>
-      <c r="E118" t="s">
-        <v>116</v>
-      </c>
-      <c r="F118" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="119" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A119" t="s">
-        <v>32</v>
-      </c>
-      <c r="B119" t="s">
-        <v>118</v>
-      </c>
-      <c r="C119" t="s">
-        <v>52</v>
-      </c>
-      <c r="E119" t="s">
-        <v>116</v>
-      </c>
-      <c r="F119" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="120" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A120" t="s">
         <v>32</v>
       </c>
       <c r="B120" t="s">
         <v>118</v>
       </c>
-      <c r="C120" t="s">
-        <v>129</v>
+      <c r="D120" t="s">
+        <v>68</v>
       </c>
       <c r="E120" t="s">
         <v>116</v>
       </c>
       <c r="F120" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="121" spans="1:6" x14ac:dyDescent="0.3">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A121" t="s">
         <v>32</v>
       </c>
@@ -3230,7 +3250,7 @@
         <v>118</v>
       </c>
       <c r="C121" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="E121" t="s">
         <v>116</v>
@@ -3239,7 +3259,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="122" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A122" t="s">
         <v>32</v>
       </c>
@@ -3247,16 +3267,16 @@
         <v>118</v>
       </c>
       <c r="C122" t="s">
-        <v>136</v>
+        <v>52</v>
       </c>
       <c r="E122" t="s">
         <v>116</v>
       </c>
       <c r="F122" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="123" spans="1:6" x14ac:dyDescent="0.3">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A123" t="s">
         <v>32</v>
       </c>
@@ -3264,16 +3284,16 @@
         <v>118</v>
       </c>
       <c r="C123" t="s">
-        <v>146</v>
+        <v>129</v>
       </c>
       <c r="E123" t="s">
         <v>116</v>
       </c>
       <c r="F123" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="124" spans="1:6" x14ac:dyDescent="0.3">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A124" t="s">
         <v>32</v>
       </c>
@@ -3281,16 +3301,16 @@
         <v>118</v>
       </c>
       <c r="C124" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="E124" t="s">
         <v>116</v>
       </c>
       <c r="F124" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="125" spans="1:6" x14ac:dyDescent="0.3">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="125" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A125" t="s">
         <v>32</v>
       </c>
@@ -3298,109 +3318,109 @@
         <v>118</v>
       </c>
       <c r="C125" t="s">
+        <v>136</v>
+      </c>
+      <c r="E125" t="s">
+        <v>116</v>
+      </c>
+      <c r="F125" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="126" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A126" t="s">
+        <v>32</v>
+      </c>
+      <c r="B126" t="s">
+        <v>118</v>
+      </c>
+      <c r="C126" t="s">
+        <v>146</v>
+      </c>
+      <c r="E126" t="s">
+        <v>116</v>
+      </c>
+      <c r="F126" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="127" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A127" t="s">
+        <v>32</v>
+      </c>
+      <c r="B127" t="s">
+        <v>118</v>
+      </c>
+      <c r="C127" t="s">
+        <v>120</v>
+      </c>
+      <c r="E127" t="s">
+        <v>116</v>
+      </c>
+      <c r="F127" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="128" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A128" t="s">
+        <v>32</v>
+      </c>
+      <c r="B128" t="s">
+        <v>118</v>
+      </c>
+      <c r="C128" t="s">
         <v>51</v>
       </c>
-      <c r="E125" t="s">
-        <v>116</v>
-      </c>
-      <c r="F125" t="s">
+      <c r="E128" t="s">
+        <v>116</v>
+      </c>
+      <c r="F128" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="126" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A126" t="s">
-        <v>32</v>
-      </c>
-      <c r="B126" t="s">
+    <row r="129" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A129" t="s">
+        <v>32</v>
+      </c>
+      <c r="B129" t="s">
         <v>165</v>
       </c>
-      <c r="D126" t="s">
+      <c r="D129" t="s">
         <v>87</v>
       </c>
-      <c r="E126" t="s">
-        <v>116</v>
-      </c>
-      <c r="F126" t="s">
+      <c r="E129" t="s">
+        <v>116</v>
+      </c>
+      <c r="F129" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="127" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A127" t="s">
-        <v>32</v>
-      </c>
-      <c r="B127" t="s">
+    <row r="130" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A130" t="s">
+        <v>32</v>
+      </c>
+      <c r="B130" t="s">
         <v>165</v>
       </c>
-      <c r="C127" t="s">
+      <c r="C130" t="s">
         <v>166</v>
       </c>
-      <c r="E127" t="s">
-        <v>116</v>
-      </c>
-      <c r="F127" t="s">
+      <c r="E130" t="s">
+        <v>116</v>
+      </c>
+      <c r="F130" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="128" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A128" t="s">
-        <v>32</v>
-      </c>
-      <c r="B128" t="s">
-        <v>149</v>
-      </c>
-      <c r="D128" t="s">
-        <v>68</v>
-      </c>
-      <c r="E128" t="s">
-        <v>116</v>
-      </c>
-      <c r="F128" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="129" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A129" t="s">
-        <v>32</v>
-      </c>
-      <c r="B129" t="s">
-        <v>149</v>
-      </c>
-      <c r="C129" t="s">
-        <v>151</v>
-      </c>
-      <c r="E129" t="s">
-        <v>116</v>
-      </c>
-      <c r="F129" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="130" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A130" t="s">
-        <v>32</v>
-      </c>
-      <c r="B130" t="s">
-        <v>149</v>
-      </c>
-      <c r="C130" t="s">
-        <v>49</v>
-      </c>
-      <c r="E130" t="s">
-        <v>116</v>
-      </c>
-      <c r="F130" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="131" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A131" t="s">
         <v>32</v>
       </c>
       <c r="B131" t="s">
         <v>149</v>
       </c>
-      <c r="C131" t="s">
-        <v>150</v>
+      <c r="D131" t="s">
+        <v>68</v>
       </c>
       <c r="E131" t="s">
         <v>116</v>
@@ -3409,7 +3429,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="132" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A132" t="s">
         <v>32</v>
       </c>
@@ -3417,7 +3437,7 @@
         <v>149</v>
       </c>
       <c r="C132" t="s">
-        <v>50</v>
+        <v>151</v>
       </c>
       <c r="E132" t="s">
         <v>116</v>
@@ -3426,32 +3446,32 @@
         <v>147</v>
       </c>
     </row>
-    <row r="133" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A133" t="s">
         <v>32</v>
       </c>
       <c r="B133" t="s">
-        <v>138</v>
-      </c>
-      <c r="D133" t="s">
-        <v>68</v>
+        <v>149</v>
+      </c>
+      <c r="C133" t="s">
+        <v>49</v>
       </c>
       <c r="E133" t="s">
         <v>116</v>
       </c>
       <c r="F133" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="134" spans="1:6" x14ac:dyDescent="0.3">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="134" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A134" t="s">
         <v>32</v>
       </c>
       <c r="B134" t="s">
-        <v>138</v>
+        <v>149</v>
       </c>
       <c r="C134" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="E134" t="s">
         <v>116</v>
@@ -3460,32 +3480,32 @@
         <v>147</v>
       </c>
     </row>
-    <row r="135" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A135" t="s">
         <v>32</v>
       </c>
       <c r="B135" t="s">
-        <v>138</v>
+        <v>149</v>
       </c>
       <c r="C135" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="E135" t="s">
         <v>116</v>
       </c>
       <c r="F135" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="136" spans="1:6" x14ac:dyDescent="0.3">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="136" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A136" t="s">
         <v>32</v>
       </c>
       <c r="B136" t="s">
         <v>138</v>
       </c>
-      <c r="C136" t="s">
-        <v>57</v>
+      <c r="D136" t="s">
+        <v>68</v>
       </c>
       <c r="E136" t="s">
         <v>116</v>
@@ -3494,7 +3514,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="137" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A137" t="s">
         <v>32</v>
       </c>
@@ -3502,16 +3522,16 @@
         <v>138</v>
       </c>
       <c r="C137" t="s">
-        <v>156</v>
+        <v>148</v>
       </c>
       <c r="E137" t="s">
         <v>116</v>
       </c>
       <c r="F137" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="138" spans="1:6" x14ac:dyDescent="0.3">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="138" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A138" t="s">
         <v>32</v>
       </c>
@@ -3519,16 +3539,16 @@
         <v>138</v>
       </c>
       <c r="C138" t="s">
-        <v>154</v>
+        <v>58</v>
       </c>
       <c r="E138" t="s">
         <v>116</v>
       </c>
       <c r="F138" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="139" spans="1:6" x14ac:dyDescent="0.3">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="139" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A139" t="s">
         <v>32</v>
       </c>
@@ -3536,16 +3556,16 @@
         <v>138</v>
       </c>
       <c r="C139" t="s">
-        <v>184</v>
+        <v>57</v>
       </c>
       <c r="E139" t="s">
         <v>116</v>
       </c>
       <c r="F139" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="140" spans="1:6" x14ac:dyDescent="0.3">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="140" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A140" t="s">
         <v>32</v>
       </c>
@@ -3553,7 +3573,7 @@
         <v>138</v>
       </c>
       <c r="C140" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="E140" t="s">
         <v>116</v>
@@ -3562,100 +3582,100 @@
         <v>158</v>
       </c>
     </row>
-    <row r="141" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A141" t="s">
         <v>32</v>
       </c>
       <c r="B141" t="s">
+        <v>138</v>
+      </c>
+      <c r="C141" t="s">
+        <v>154</v>
+      </c>
+      <c r="E141" t="s">
+        <v>116</v>
+      </c>
+      <c r="F141" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="142" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A142" t="s">
+        <v>32</v>
+      </c>
+      <c r="B142" t="s">
+        <v>138</v>
+      </c>
+      <c r="C142" t="s">
+        <v>184</v>
+      </c>
+      <c r="E142" t="s">
+        <v>116</v>
+      </c>
+      <c r="F142" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="143" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A143" t="s">
+        <v>32</v>
+      </c>
+      <c r="B143" t="s">
+        <v>138</v>
+      </c>
+      <c r="C143" t="s">
+        <v>157</v>
+      </c>
+      <c r="E143" t="s">
+        <v>116</v>
+      </c>
+      <c r="F143" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="144" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A144" t="s">
+        <v>32</v>
+      </c>
+      <c r="B144" t="s">
         <v>125</v>
       </c>
-      <c r="D141" t="s">
+      <c r="D144" t="s">
         <v>68</v>
       </c>
-      <c r="E141" t="s">
-        <v>116</v>
-      </c>
-      <c r="F141" t="s">
+      <c r="E144" t="s">
+        <v>116</v>
+      </c>
+      <c r="F144" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="142" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A142" t="s">
-        <v>32</v>
-      </c>
-      <c r="B142" t="s">
+    <row r="145" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A145" t="s">
+        <v>32</v>
+      </c>
+      <c r="B145" t="s">
         <v>125</v>
       </c>
-      <c r="C142" t="s">
+      <c r="C145" t="s">
         <v>127</v>
       </c>
-      <c r="E142" t="s">
-        <v>116</v>
-      </c>
-      <c r="F142" t="s">
+      <c r="E145" t="s">
+        <v>116</v>
+      </c>
+      <c r="F145" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="143" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A143" t="s">
-        <v>32</v>
-      </c>
-      <c r="B143" t="s">
-        <v>131</v>
-      </c>
-      <c r="D143" t="s">
-        <v>68</v>
-      </c>
-      <c r="E143" t="s">
-        <v>116</v>
-      </c>
-      <c r="F143" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="144" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A144" t="s">
-        <v>32</v>
-      </c>
-      <c r="B144" t="s">
-        <v>131</v>
-      </c>
-      <c r="C144" t="s">
-        <v>132</v>
-      </c>
-      <c r="E144" t="s">
-        <v>116</v>
-      </c>
-      <c r="F144" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="145" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A145" t="s">
-        <v>32</v>
-      </c>
-      <c r="B145" t="s">
-        <v>131</v>
-      </c>
-      <c r="C145" t="s">
-        <v>133</v>
-      </c>
-      <c r="E145" t="s">
-        <v>116</v>
-      </c>
-      <c r="F145" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="146" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A146" t="s">
         <v>32</v>
       </c>
       <c r="B146" t="s">
         <v>131</v>
       </c>
-      <c r="C146" t="s">
-        <v>134</v>
+      <c r="D146" t="s">
+        <v>68</v>
       </c>
       <c r="E146" t="s">
         <v>116</v>
@@ -3664,7 +3684,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="147" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A147" t="s">
         <v>32</v>
       </c>
@@ -3672,7 +3692,7 @@
         <v>131</v>
       </c>
       <c r="C147" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="E147" t="s">
         <v>116</v>
@@ -3681,126 +3701,117 @@
         <v>130</v>
       </c>
     </row>
-    <row r="148" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A148" t="s">
         <v>32</v>
       </c>
       <c r="B148" t="s">
+        <v>131</v>
+      </c>
+      <c r="C148" t="s">
+        <v>133</v>
+      </c>
+      <c r="E148" t="s">
+        <v>116</v>
+      </c>
+      <c r="F148" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="149" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A149" t="s">
+        <v>32</v>
+      </c>
+      <c r="B149" t="s">
+        <v>131</v>
+      </c>
+      <c r="C149" t="s">
+        <v>134</v>
+      </c>
+      <c r="E149" t="s">
+        <v>116</v>
+      </c>
+      <c r="F149" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="150" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A150" t="s">
+        <v>32</v>
+      </c>
+      <c r="B150" t="s">
+        <v>131</v>
+      </c>
+      <c r="C150" t="s">
+        <v>135</v>
+      </c>
+      <c r="E150" t="s">
+        <v>116</v>
+      </c>
+      <c r="F150" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="151" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A151" t="s">
+        <v>32</v>
+      </c>
+      <c r="B151" t="s">
         <v>126</v>
       </c>
-      <c r="D148" t="s">
+      <c r="D151" t="s">
         <v>68</v>
       </c>
-      <c r="E148" t="s">
-        <v>116</v>
-      </c>
-      <c r="F148" t="s">
+      <c r="E151" t="s">
+        <v>116</v>
+      </c>
+      <c r="F151" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="149" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A149" t="s">
-        <v>32</v>
-      </c>
-      <c r="B149" t="s">
+    <row r="152" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A152" t="s">
+        <v>32</v>
+      </c>
+      <c r="B152" t="s">
         <v>126</v>
       </c>
-      <c r="C149" t="s">
+      <c r="C152" t="s">
         <v>128</v>
       </c>
-      <c r="E149" t="s">
-        <v>116</v>
-      </c>
-      <c r="F149" t="s">
+      <c r="E152" t="s">
+        <v>116</v>
+      </c>
+      <c r="F152" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="150" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A150" t="s">
-        <v>32</v>
-      </c>
-      <c r="B150" t="s">
+    <row r="153" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A153" t="s">
+        <v>32</v>
+      </c>
+      <c r="B153" t="s">
         <v>98</v>
       </c>
-      <c r="D150" t="s">
+      <c r="D153" t="s">
         <v>87</v>
-      </c>
-      <c r="E150" t="s">
-        <v>14</v>
-      </c>
-      <c r="F150" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="151" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A151" t="s">
-        <v>32</v>
-      </c>
-      <c r="B151" t="s">
-        <v>13</v>
-      </c>
-      <c r="D151" t="s">
-        <v>87</v>
-      </c>
-      <c r="E151" t="s">
-        <v>14</v>
-      </c>
-      <c r="F151" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="152" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A152" t="s">
-        <v>32</v>
-      </c>
-      <c r="B152" t="s">
-        <v>13</v>
-      </c>
-      <c r="C152" t="s">
-        <v>10</v>
-      </c>
-      <c r="D152">
-        <v>1</v>
-      </c>
-      <c r="E152" t="s">
-        <v>14</v>
-      </c>
-      <c r="F152" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="153" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A153" t="s">
-        <v>32</v>
-      </c>
-      <c r="B153" t="s">
-        <v>13</v>
-      </c>
-      <c r="C153" t="s">
-        <v>20</v>
-      </c>
-      <c r="D153">
-        <v>1</v>
       </c>
       <c r="E153" t="s">
         <v>14</v>
       </c>
       <c r="F153" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="154" spans="1:6" x14ac:dyDescent="0.3">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="154" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A154" t="s">
         <v>32</v>
       </c>
       <c r="B154" t="s">
         <v>13</v>
       </c>
-      <c r="C154" t="s">
-        <v>18</v>
-      </c>
-      <c r="D154">
-        <v>1</v>
+      <c r="D154" t="s">
+        <v>87</v>
       </c>
       <c r="E154" t="s">
         <v>14</v>
@@ -3809,69 +3820,75 @@
         <v>17</v>
       </c>
     </row>
-    <row r="155" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A155" t="s">
         <v>32</v>
       </c>
       <c r="B155" t="s">
+        <v>13</v>
+      </c>
+      <c r="C155" t="s">
+        <v>10</v>
+      </c>
+      <c r="D155">
+        <v>1</v>
+      </c>
+      <c r="E155" t="s">
+        <v>14</v>
+      </c>
+      <c r="F155" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="156" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A156" t="s">
+        <v>32</v>
+      </c>
+      <c r="B156" t="s">
+        <v>13</v>
+      </c>
+      <c r="C156" t="s">
+        <v>20</v>
+      </c>
+      <c r="D156">
+        <v>1</v>
+      </c>
+      <c r="E156" t="s">
+        <v>14</v>
+      </c>
+      <c r="F156" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="157" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A157" t="s">
+        <v>32</v>
+      </c>
+      <c r="B157" t="s">
+        <v>13</v>
+      </c>
+      <c r="C157" t="s">
+        <v>18</v>
+      </c>
+      <c r="D157">
+        <v>1</v>
+      </c>
+      <c r="E157" t="s">
+        <v>14</v>
+      </c>
+      <c r="F157" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="158" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A158" t="s">
+        <v>32</v>
+      </c>
+      <c r="B158" t="s">
         <v>97</v>
       </c>
-      <c r="D155" t="s">
+      <c r="D158" t="s">
         <v>87</v>
-      </c>
-      <c r="E155" t="s">
-        <v>54</v>
-      </c>
-      <c r="F155" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="156" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A156" t="s">
-        <v>32</v>
-      </c>
-      <c r="B156" t="s">
-        <v>97</v>
-      </c>
-      <c r="C156" t="s">
-        <v>191</v>
-      </c>
-      <c r="E156" t="s">
-        <v>24</v>
-      </c>
-      <c r="F156" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="157" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A157" t="s">
-        <v>32</v>
-      </c>
-      <c r="B157" t="s">
-        <v>33</v>
-      </c>
-      <c r="D157" t="s">
-        <v>87</v>
-      </c>
-      <c r="E157" t="s">
-        <v>54</v>
-      </c>
-      <c r="F157" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="158" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A158" t="s">
-        <v>32</v>
-      </c>
-      <c r="B158" t="s">
-        <v>33</v>
-      </c>
-      <c r="C158" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="D158">
-        <v>1</v>
       </c>
       <c r="E158" t="s">
         <v>54</v>
@@ -3880,35 +3897,32 @@
         <v>63</v>
       </c>
     </row>
-    <row r="159" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A159" t="s">
         <v>32</v>
       </c>
       <c r="B159" t="s">
-        <v>33</v>
-      </c>
-      <c r="C159" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="D159">
-        <v>1</v>
+        <v>97</v>
+      </c>
+      <c r="C159" t="s">
+        <v>191</v>
       </c>
       <c r="E159" t="s">
-        <v>54</v>
+        <v>24</v>
       </c>
       <c r="F159" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="160" spans="1:6" x14ac:dyDescent="0.3">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="160" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A160" t="s">
         <v>32</v>
       </c>
       <c r="B160" t="s">
         <v>33</v>
       </c>
-      <c r="C160" s="1" t="s">
-        <v>57</v>
+      <c r="D160" t="s">
+        <v>87</v>
       </c>
       <c r="E160" t="s">
         <v>54</v>
@@ -3917,7 +3931,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="161" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A161" t="s">
         <v>32</v>
       </c>
@@ -3925,47 +3939,104 @@
         <v>33</v>
       </c>
       <c r="C161" s="1" t="s">
-        <v>195</v>
+        <v>39</v>
+      </c>
+      <c r="D161">
+        <v>1</v>
       </c>
       <c r="E161" t="s">
         <v>54</v>
       </c>
       <c r="F161" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="162" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A162" t="s">
+        <v>32</v>
+      </c>
+      <c r="B162" t="s">
+        <v>33</v>
+      </c>
+      <c r="C162" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D162">
+        <v>1</v>
+      </c>
+      <c r="E162" t="s">
+        <v>54</v>
+      </c>
+      <c r="F162" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="163" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A163" t="s">
+        <v>32</v>
+      </c>
+      <c r="B163" t="s">
+        <v>33</v>
+      </c>
+      <c r="C163" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="E163" t="s">
+        <v>54</v>
+      </c>
+      <c r="F163" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="164" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A164" t="s">
+        <v>32</v>
+      </c>
+      <c r="B164" t="s">
+        <v>33</v>
+      </c>
+      <c r="C164" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="E164" t="s">
+        <v>54</v>
+      </c>
+      <c r="F164" t="s">
         <v>193</v>
       </c>
     </row>
-    <row r="162" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A162" t="s">
-        <v>32</v>
-      </c>
-      <c r="B162" t="s">
+    <row r="165" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A165" t="s">
+        <v>32</v>
+      </c>
+      <c r="B165" t="s">
         <v>182</v>
       </c>
-      <c r="C162" s="1"/>
-      <c r="D162" t="s">
+      <c r="C165" s="1"/>
+      <c r="D165" t="s">
         <v>68</v>
       </c>
-      <c r="E162" t="s">
-        <v>116</v>
-      </c>
-      <c r="F162" t="s">
+      <c r="E165" t="s">
+        <v>116</v>
+      </c>
+      <c r="F165" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="163" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A163" t="s">
-        <v>32</v>
-      </c>
-      <c r="B163" t="s">
+    <row r="166" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A166" t="s">
+        <v>32</v>
+      </c>
+      <c r="B166" t="s">
         <v>88</v>
       </c>
-      <c r="D163" t="s">
+      <c r="D166" t="s">
         <v>65</v>
       </c>
-      <c r="E163" t="s">
+      <c r="E166" t="s">
         <v>24</v>
       </c>
-      <c r="F163" t="s">
+      <c r="F166" t="s">
         <v>89</v>
       </c>
     </row>

</xml_diff>

<commit_message>
[PowerPoint] (Shape) Add snippet that gets Base64 image (#1068)
</commit_message>
<xml_diff>
--- a/snippet-extractor-metadata/powerpoint.xlsx
+++ b/snippet-extractor-metadata/powerpoint.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{995B1E0C-ED6E-4740-AEB3-BEC61464CEDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7C414EC-35C0-4625-9957-123F9D615DF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{CB5595D7-4492-4192-A1C1-2583BA1957AA}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25180" windowHeight="16140" xr2:uid="{CB5595D7-4492-4192-A1C1-2583BA1957AA}"/>
   </bookViews>
   <sheets>
     <sheet name="Snippets" sheetId="2" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="816" uniqueCount="210">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="831" uniqueCount="215">
   <si>
     <t>Class</t>
   </si>
@@ -650,6 +650,21 @@
   </si>
   <si>
     <t>updateHyperlinkOnShape</t>
+  </si>
+  <si>
+    <t>ShapeGetImageOptions</t>
+  </si>
+  <si>
+    <t>powerpoint-shapes-get-shape-as-image</t>
+  </si>
+  <si>
+    <t>getImageWithAllOptions</t>
+  </si>
+  <si>
+    <t>getImageDefault</t>
+  </si>
+  <si>
+    <t>ShapeGetImageFormatType</t>
   </si>
 </sst>
 </file>
@@ -730,10 +745,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{78C585A5-D505-49C6-9CA1-8E6558948317}" name="Snippets" displayName="Snippets" ref="A1:F163" totalsRowShown="0" headerRowDxfId="4">
-  <autoFilter ref="A1:F163" xr:uid="{EAC65D03-FDD2-4352-A5F3-1CDEDE6251B2}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F159">
-    <sortCondition ref="B1:B159"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{78C585A5-D505-49C6-9CA1-8E6558948317}" name="Snippets" displayName="Snippets" ref="A1:F166" totalsRowShown="0" headerRowDxfId="4">
+  <autoFilter ref="A1:F166" xr:uid="{EAC65D03-FDD2-4352-A5F3-1CDEDE6251B2}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F162">
+    <sortCondition ref="B1:B162"/>
   </sortState>
   <tableColumns count="6">
     <tableColumn id="6" xr3:uid="{408888B8-C1DD-4B51-B1EB-5663F091D142}" name="Package"/>
@@ -1044,19 +1059,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{809930CD-A227-47DC-AAA4-BB816AEDEB59}">
-  <dimension ref="A1:F163"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:F166"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="26.5546875" customWidth="1"/>
-    <col min="3" max="3" width="26.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.54296875" customWidth="1"/>
+    <col min="3" max="3" width="26.54296875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="23" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="42.77734375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="42.81640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="55" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="31" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>31</v>
       </c>
@@ -1076,7 +1091,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>32</v>
       </c>
@@ -1093,7 +1108,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>32</v>
       </c>
@@ -1110,7 +1125,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>32</v>
       </c>
@@ -1130,7 +1145,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>32</v>
       </c>
@@ -1147,7 +1162,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>32</v>
       </c>
@@ -1167,7 +1182,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>32</v>
       </c>
@@ -1187,7 +1202,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>32</v>
       </c>
@@ -1204,7 +1219,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>32</v>
       </c>
@@ -1221,7 +1236,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>32</v>
       </c>
@@ -1238,7 +1253,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>32</v>
       </c>
@@ -1255,7 +1270,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>32</v>
       </c>
@@ -1272,7 +1287,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>32</v>
       </c>
@@ -1289,7 +1304,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>32</v>
       </c>
@@ -1306,7 +1321,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>32</v>
       </c>
@@ -1323,7 +1338,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>32</v>
       </c>
@@ -1340,7 +1355,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>32</v>
       </c>
@@ -1357,7 +1372,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>32</v>
       </c>
@@ -1374,7 +1389,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>32</v>
       </c>
@@ -1391,7 +1406,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>32</v>
       </c>
@@ -1408,7 +1423,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>32</v>
       </c>
@@ -1425,7 +1440,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>32</v>
       </c>
@@ -1442,7 +1457,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>32</v>
       </c>
@@ -1459,7 +1474,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>32</v>
       </c>
@@ -1476,7 +1491,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>32</v>
       </c>
@@ -1493,14 +1508,14 @@
         <v>102</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>32</v>
       </c>
       <c r="B26" t="s">
         <v>100</v>
       </c>
-      <c r="C26" s="2" t="s">
+      <c r="C26" t="s">
         <v>20</v>
       </c>
       <c r="D26">
@@ -1509,11 +1524,11 @@
       <c r="E26" t="s">
         <v>103</v>
       </c>
-      <c r="F26" s="2" t="s">
+      <c r="F26" t="s">
         <v>207</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>32</v>
       </c>
@@ -1530,7 +1545,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>32</v>
       </c>
@@ -1547,7 +1562,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>32</v>
       </c>
@@ -1564,7 +1579,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>32</v>
       </c>
@@ -1581,7 +1596,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>32</v>
       </c>
@@ -1598,7 +1613,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>32</v>
       </c>
@@ -1615,7 +1630,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>32</v>
       </c>
@@ -1632,7 +1647,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>32</v>
       </c>
@@ -1649,7 +1664,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>32</v>
       </c>
@@ -1666,7 +1681,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>32</v>
       </c>
@@ -1686,7 +1701,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>32</v>
       </c>
@@ -1706,7 +1721,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>32</v>
       </c>
@@ -1726,7 +1741,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>32</v>
       </c>
@@ -1746,7 +1761,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>32</v>
       </c>
@@ -1766,7 +1781,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>32</v>
       </c>
@@ -1786,7 +1801,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>32</v>
       </c>
@@ -1806,7 +1821,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>32</v>
       </c>
@@ -1826,7 +1841,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>32</v>
       </c>
@@ -1846,7 +1861,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>32</v>
       </c>
@@ -1866,7 +1881,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>32</v>
       </c>
@@ -1886,7 +1901,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>32</v>
       </c>
@@ -1903,7 +1918,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>32</v>
       </c>
@@ -1920,7 +1935,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>32</v>
       </c>
@@ -1940,47 +1955,47 @@
         <v>96</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>32</v>
       </c>
       <c r="B50" t="s">
         <v>45</v>
       </c>
-      <c r="C50" t="s">
-        <v>161</v>
+      <c r="C50" s="2" t="s">
+        <v>106</v>
       </c>
       <c r="D50">
         <v>1</v>
       </c>
-      <c r="E50" t="s">
-        <v>116</v>
-      </c>
-      <c r="F50" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E50" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="F50" s="2" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>32</v>
       </c>
       <c r="B51" t="s">
         <v>45</v>
       </c>
-      <c r="C51" s="2" t="s">
-        <v>208</v>
+      <c r="C51" t="s">
+        <v>161</v>
       </c>
       <c r="D51">
         <v>1</v>
       </c>
-      <c r="E51" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="F51" s="2" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E51" t="s">
+        <v>116</v>
+      </c>
+      <c r="F51" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>32</v>
       </c>
@@ -1988,19 +2003,19 @@
         <v>45</v>
       </c>
       <c r="C52" t="s">
-        <v>176</v>
+        <v>208</v>
       </c>
       <c r="D52">
         <v>1</v>
       </c>
       <c r="E52" t="s">
-        <v>168</v>
+        <v>103</v>
       </c>
       <c r="F52" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>32</v>
       </c>
@@ -2008,16 +2023,19 @@
         <v>45</v>
       </c>
       <c r="C53" t="s">
-        <v>58</v>
+        <v>176</v>
+      </c>
+      <c r="D53">
+        <v>1</v>
       </c>
       <c r="E53" t="s">
-        <v>53</v>
+        <v>168</v>
       </c>
       <c r="F53" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>32</v>
       </c>
@@ -2025,16 +2043,16 @@
         <v>45</v>
       </c>
       <c r="C54" t="s">
-        <v>108</v>
+        <v>58</v>
       </c>
       <c r="E54" t="s">
-        <v>109</v>
+        <v>53</v>
       </c>
       <c r="F54" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>32</v>
       </c>
@@ -2042,16 +2060,16 @@
         <v>45</v>
       </c>
       <c r="C55" t="s">
-        <v>52</v>
+        <v>108</v>
       </c>
       <c r="E55" t="s">
-        <v>53</v>
+        <v>109</v>
       </c>
       <c r="F55" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>32</v>
       </c>
@@ -2059,7 +2077,7 @@
         <v>45</v>
       </c>
       <c r="C56" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="E56" t="s">
         <v>53</v>
@@ -2068,7 +2086,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>32</v>
       </c>
@@ -2076,16 +2094,16 @@
         <v>45</v>
       </c>
       <c r="C57" t="s">
-        <v>196</v>
+        <v>49</v>
       </c>
       <c r="E57" t="s">
-        <v>85</v>
+        <v>53</v>
       </c>
       <c r="F57" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>32</v>
       </c>
@@ -2093,16 +2111,16 @@
         <v>45</v>
       </c>
       <c r="C58" t="s">
-        <v>50</v>
+        <v>196</v>
       </c>
       <c r="E58" t="s">
-        <v>53</v>
+        <v>85</v>
       </c>
       <c r="F58" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.3">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>32</v>
       </c>
@@ -2110,16 +2128,16 @@
         <v>45</v>
       </c>
       <c r="C59" t="s">
-        <v>86</v>
+        <v>50</v>
       </c>
       <c r="E59" t="s">
-        <v>85</v>
+        <v>53</v>
       </c>
       <c r="F59" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.3">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>32</v>
       </c>
@@ -2127,16 +2145,16 @@
         <v>45</v>
       </c>
       <c r="C60" t="s">
-        <v>51</v>
+        <v>86</v>
       </c>
       <c r="E60" t="s">
-        <v>53</v>
+        <v>85</v>
       </c>
       <c r="F60" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.3">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>32</v>
       </c>
@@ -2144,87 +2162,84 @@
         <v>45</v>
       </c>
       <c r="C61" t="s">
+        <v>51</v>
+      </c>
+      <c r="E61" t="s">
+        <v>53</v>
+      </c>
+      <c r="F61" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A62" t="s">
+        <v>32</v>
+      </c>
+      <c r="B62" t="s">
+        <v>45</v>
+      </c>
+      <c r="C62" t="s">
         <v>178</v>
       </c>
-      <c r="E61" t="s">
+      <c r="E62" t="s">
         <v>168</v>
       </c>
-      <c r="F61" t="s">
+      <c r="F62" t="s">
         <v>177</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A62" t="s">
-        <v>32</v>
-      </c>
-      <c r="B62" t="s">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A63" t="s">
+        <v>32</v>
+      </c>
+      <c r="B63" t="s">
         <v>95</v>
       </c>
-      <c r="D62" t="s">
+      <c r="D63" t="s">
         <v>68</v>
-      </c>
-      <c r="E62" t="s">
-        <v>24</v>
-      </c>
-      <c r="F62" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A63" t="s">
-        <v>32</v>
-      </c>
-      <c r="B63" t="s">
-        <v>187</v>
-      </c>
-      <c r="D63" t="s">
-        <v>65</v>
       </c>
       <c r="E63" t="s">
         <v>24</v>
       </c>
       <c r="F63" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A64" t="s">
+        <v>32</v>
+      </c>
+      <c r="B64" t="s">
+        <v>187</v>
+      </c>
+      <c r="D64" t="s">
+        <v>65</v>
+      </c>
+      <c r="E64" t="s">
+        <v>24</v>
+      </c>
+      <c r="F64" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A64" t="s">
-        <v>32</v>
-      </c>
-      <c r="B64" t="s">
-        <v>21</v>
-      </c>
-      <c r="D64" t="s">
-        <v>87</v>
-      </c>
-      <c r="E64" t="s">
-        <v>85</v>
-      </c>
-      <c r="F64" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>32</v>
       </c>
       <c r="B65" t="s">
         <v>21</v>
       </c>
-      <c r="C65" t="s">
-        <v>25</v>
-      </c>
-      <c r="D65">
-        <v>1</v>
+      <c r="D65" t="s">
+        <v>87</v>
       </c>
       <c r="E65" t="s">
-        <v>24</v>
+        <v>85</v>
       </c>
       <c r="F65" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.3">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>32</v>
       </c>
@@ -2232,19 +2247,19 @@
         <v>21</v>
       </c>
       <c r="C66" t="s">
-        <v>111</v>
+        <v>25</v>
       </c>
       <c r="D66">
         <v>1</v>
       </c>
       <c r="E66" t="s">
-        <v>109</v>
+        <v>24</v>
       </c>
       <c r="F66" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>32</v>
       </c>
@@ -2252,19 +2267,19 @@
         <v>21</v>
       </c>
       <c r="C67" t="s">
-        <v>27</v>
+        <v>111</v>
       </c>
       <c r="D67">
         <v>1</v>
       </c>
       <c r="E67" t="s">
-        <v>24</v>
+        <v>109</v>
       </c>
       <c r="F67" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>32</v>
       </c>
@@ -2272,19 +2287,19 @@
         <v>21</v>
       </c>
       <c r="C68" t="s">
-        <v>115</v>
+        <v>27</v>
       </c>
       <c r="D68">
         <v>1</v>
       </c>
       <c r="E68" t="s">
-        <v>116</v>
+        <v>24</v>
       </c>
       <c r="F68" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.3">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>32</v>
       </c>
@@ -2292,19 +2307,19 @@
         <v>21</v>
       </c>
       <c r="C69" t="s">
-        <v>29</v>
+        <v>115</v>
       </c>
       <c r="D69">
         <v>1</v>
       </c>
       <c r="E69" t="s">
-        <v>24</v>
+        <v>116</v>
       </c>
       <c r="F69" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.3">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>32</v>
       </c>
@@ -2312,19 +2327,19 @@
         <v>21</v>
       </c>
       <c r="C70" t="s">
-        <v>91</v>
+        <v>29</v>
       </c>
       <c r="D70">
         <v>1</v>
       </c>
       <c r="E70" t="s">
-        <v>116</v>
+        <v>24</v>
       </c>
       <c r="F70" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>32</v>
       </c>
@@ -2332,19 +2347,19 @@
         <v>21</v>
       </c>
       <c r="C71" t="s">
-        <v>16</v>
+        <v>91</v>
       </c>
       <c r="D71">
         <v>1</v>
       </c>
       <c r="E71" t="s">
-        <v>14</v>
+        <v>116</v>
       </c>
       <c r="F71" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.3">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>32</v>
       </c>
@@ -2352,27 +2367,30 @@
         <v>21</v>
       </c>
       <c r="C72" t="s">
+        <v>16</v>
+      </c>
+      <c r="D72">
+        <v>1</v>
+      </c>
+      <c r="E72" t="s">
+        <v>14</v>
+      </c>
+      <c r="F72" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A73" t="s">
+        <v>32</v>
+      </c>
+      <c r="B73" t="s">
+        <v>21</v>
+      </c>
+      <c r="C73" t="s">
         <v>70</v>
       </c>
-      <c r="D72">
+      <c r="D73">
         <v>2</v>
-      </c>
-      <c r="E72" t="s">
-        <v>85</v>
-      </c>
-      <c r="F72" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A73" t="s">
-        <v>32</v>
-      </c>
-      <c r="B73" t="s">
-        <v>59</v>
-      </c>
-      <c r="D73" t="s">
-        <v>87</v>
       </c>
       <c r="E73" t="s">
         <v>85</v>
@@ -2381,27 +2399,24 @@
         <v>81</v>
       </c>
     </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>32</v>
       </c>
       <c r="B74" t="s">
         <v>59</v>
       </c>
-      <c r="C74" t="s">
-        <v>179</v>
-      </c>
-      <c r="D74">
-        <v>1</v>
+      <c r="D74" t="s">
+        <v>87</v>
       </c>
       <c r="E74" t="s">
-        <v>168</v>
+        <v>85</v>
       </c>
       <c r="F74" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.3">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>32</v>
       </c>
@@ -2409,19 +2424,19 @@
         <v>59</v>
       </c>
       <c r="C75" t="s">
-        <v>60</v>
+        <v>179</v>
       </c>
       <c r="D75">
         <v>1</v>
       </c>
       <c r="E75" t="s">
-        <v>53</v>
+        <v>168</v>
       </c>
       <c r="F75" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.3">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>32</v>
       </c>
@@ -2429,16 +2444,19 @@
         <v>59</v>
       </c>
       <c r="C76" t="s">
-        <v>93</v>
+        <v>60</v>
+      </c>
+      <c r="D76">
+        <v>1</v>
       </c>
       <c r="E76" t="s">
         <v>53</v>
       </c>
       <c r="F76" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.3">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>32</v>
       </c>
@@ -2446,16 +2464,16 @@
         <v>59</v>
       </c>
       <c r="C77" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="E77" t="s">
-        <v>85</v>
+        <v>53</v>
       </c>
       <c r="F77" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.3">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
         <v>32</v>
       </c>
@@ -2463,24 +2481,24 @@
         <v>59</v>
       </c>
       <c r="C78" t="s">
+        <v>82</v>
+      </c>
+      <c r="E78" t="s">
+        <v>85</v>
+      </c>
+      <c r="F78" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A79" t="s">
+        <v>32</v>
+      </c>
+      <c r="B79" t="s">
+        <v>59</v>
+      </c>
+      <c r="C79" t="s">
         <v>86</v>
-      </c>
-      <c r="E78" t="s">
-        <v>53</v>
-      </c>
-      <c r="F78" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A79" t="s">
-        <v>32</v>
-      </c>
-      <c r="B79" t="s">
-        <v>189</v>
-      </c>
-      <c r="D79" t="s">
-        <v>65</v>
       </c>
       <c r="E79" t="s">
         <v>53</v>
@@ -2489,41 +2507,41 @@
         <v>44</v>
       </c>
     </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
         <v>32</v>
       </c>
       <c r="B80" t="s">
-        <v>61</v>
+        <v>189</v>
       </c>
       <c r="D80" t="s">
-        <v>87</v>
+        <v>65</v>
       </c>
       <c r="E80" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F80" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.3">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
         <v>32</v>
       </c>
       <c r="B81" t="s">
         <v>61</v>
       </c>
-      <c r="C81" t="s">
-        <v>62</v>
+      <c r="D81" t="s">
+        <v>87</v>
       </c>
       <c r="E81" t="s">
         <v>54</v>
       </c>
       <c r="F81" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.3">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
         <v>32</v>
       </c>
@@ -2531,24 +2549,24 @@
         <v>61</v>
       </c>
       <c r="C82" t="s">
+        <v>62</v>
+      </c>
+      <c r="E82" t="s">
+        <v>54</v>
+      </c>
+      <c r="F82" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A83" t="s">
+        <v>32</v>
+      </c>
+      <c r="B83" t="s">
+        <v>61</v>
+      </c>
+      <c r="C83" t="s">
         <v>190</v>
-      </c>
-      <c r="E82" t="s">
-        <v>24</v>
-      </c>
-      <c r="F82" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A83" t="s">
-        <v>32</v>
-      </c>
-      <c r="B83" t="s">
-        <v>188</v>
-      </c>
-      <c r="D83" t="s">
-        <v>65</v>
       </c>
       <c r="E83" t="s">
         <v>24</v>
@@ -2557,140 +2575,139 @@
         <v>89</v>
       </c>
     </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
         <v>32</v>
       </c>
       <c r="B84" t="s">
+        <v>188</v>
+      </c>
+      <c r="D84" t="s">
+        <v>65</v>
+      </c>
+      <c r="E84" t="s">
+        <v>24</v>
+      </c>
+      <c r="F84" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A85" t="s">
+        <v>32</v>
+      </c>
+      <c r="B85" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="C85" s="2"/>
+      <c r="D85" t="s">
+        <v>65</v>
+      </c>
+      <c r="E85" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="F85" s="2" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A86" t="s">
+        <v>32</v>
+      </c>
+      <c r="B86" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="C86" s="2"/>
+      <c r="D86" t="s">
+        <v>68</v>
+      </c>
+      <c r="E86" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="F86" s="2" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A87" t="s">
+        <v>32</v>
+      </c>
+      <c r="B87" t="s">
         <v>113</v>
-      </c>
-      <c r="D84" t="s">
-        <v>87</v>
-      </c>
-      <c r="E84" t="s">
-        <v>109</v>
-      </c>
-      <c r="F84" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A85" t="s">
-        <v>32</v>
-      </c>
-      <c r="B85" t="s">
-        <v>113</v>
-      </c>
-      <c r="C85" t="s">
-        <v>114</v>
-      </c>
-      <c r="D85">
-        <v>1</v>
-      </c>
-      <c r="E85" t="s">
-        <v>109</v>
-      </c>
-      <c r="F85" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A86" t="s">
-        <v>32</v>
-      </c>
-      <c r="B86" t="s">
-        <v>80</v>
-      </c>
-      <c r="D86" t="s">
-        <v>65</v>
-      </c>
-      <c r="E86" t="s">
-        <v>85</v>
-      </c>
-      <c r="F86" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A87" t="s">
-        <v>32</v>
-      </c>
-      <c r="B87" t="s">
-        <v>83</v>
       </c>
       <c r="D87" t="s">
         <v>87</v>
       </c>
       <c r="E87" t="s">
+        <v>109</v>
+      </c>
+      <c r="F87" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A88" t="s">
+        <v>32</v>
+      </c>
+      <c r="B88" t="s">
+        <v>113</v>
+      </c>
+      <c r="C88" t="s">
+        <v>114</v>
+      </c>
+      <c r="D88">
+        <v>1</v>
+      </c>
+      <c r="E88" t="s">
+        <v>109</v>
+      </c>
+      <c r="F88" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A89" t="s">
+        <v>32</v>
+      </c>
+      <c r="B89" t="s">
+        <v>80</v>
+      </c>
+      <c r="D89" t="s">
+        <v>65</v>
+      </c>
+      <c r="E89" t="s">
         <v>85</v>
       </c>
-      <c r="F87" t="s">
+      <c r="F89" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A88" t="s">
-        <v>32</v>
-      </c>
-      <c r="B88" t="s">
+    <row r="90" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A90" t="s">
+        <v>32</v>
+      </c>
+      <c r="B90" t="s">
         <v>83</v>
       </c>
-      <c r="C88" t="s">
+      <c r="D90" t="s">
+        <v>87</v>
+      </c>
+      <c r="E90" t="s">
+        <v>85</v>
+      </c>
+      <c r="F90" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A91" t="s">
+        <v>32</v>
+      </c>
+      <c r="B91" t="s">
+        <v>83</v>
+      </c>
+      <c r="C91" t="s">
         <v>84</v>
-      </c>
-      <c r="E88" t="s">
-        <v>85</v>
-      </c>
-      <c r="F88" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A89" t="s">
-        <v>32</v>
-      </c>
-      <c r="B89" t="s">
-        <v>90</v>
-      </c>
-      <c r="D89" t="s">
-        <v>87</v>
-      </c>
-      <c r="E89" t="s">
-        <v>53</v>
-      </c>
-      <c r="F89" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A90" t="s">
-        <v>32</v>
-      </c>
-      <c r="B90" t="s">
-        <v>90</v>
-      </c>
-      <c r="C90" t="s">
-        <v>91</v>
-      </c>
-      <c r="D90">
-        <v>1</v>
-      </c>
-      <c r="E90" t="s">
-        <v>53</v>
-      </c>
-      <c r="F90" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A91" t="s">
-        <v>32</v>
-      </c>
-      <c r="B91" t="s">
-        <v>78</v>
-      </c>
-      <c r="D91" t="s">
-        <v>65</v>
       </c>
       <c r="E91" t="s">
         <v>85</v>
@@ -2699,118 +2716,112 @@
         <v>79</v>
       </c>
     </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
         <v>32</v>
       </c>
       <c r="B92" t="s">
+        <v>90</v>
+      </c>
+      <c r="D92" t="s">
+        <v>87</v>
+      </c>
+      <c r="E92" t="s">
+        <v>53</v>
+      </c>
+      <c r="F92" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A93" t="s">
+        <v>32</v>
+      </c>
+      <c r="B93" t="s">
+        <v>90</v>
+      </c>
+      <c r="C93" t="s">
+        <v>91</v>
+      </c>
+      <c r="D93">
+        <v>1</v>
+      </c>
+      <c r="E93" t="s">
+        <v>53</v>
+      </c>
+      <c r="F93" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A94" t="s">
+        <v>32</v>
+      </c>
+      <c r="B94" t="s">
+        <v>78</v>
+      </c>
+      <c r="D94" t="s">
+        <v>65</v>
+      </c>
+      <c r="E94" t="s">
+        <v>85</v>
+      </c>
+      <c r="F94" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A95" t="s">
+        <v>32</v>
+      </c>
+      <c r="B95" t="s">
         <v>180</v>
       </c>
-      <c r="D92" t="s">
+      <c r="D95" t="s">
         <v>65</v>
       </c>
-      <c r="E92" t="s">
+      <c r="E95" t="s">
         <v>168</v>
       </c>
-      <c r="F92" t="s">
+      <c r="F95" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A93" t="s">
-        <v>32</v>
-      </c>
-      <c r="B93" t="s">
+    <row r="96" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A96" t="s">
+        <v>32</v>
+      </c>
+      <c r="B96" t="s">
         <v>180</v>
       </c>
-      <c r="D93" t="s">
+      <c r="D96" t="s">
         <v>65</v>
       </c>
-      <c r="E93" t="s">
+      <c r="E96" t="s">
         <v>168</v>
       </c>
-      <c r="F93" t="s">
+      <c r="F96" t="s">
         <v>177</v>
       </c>
     </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A94" t="s">
-        <v>32</v>
-      </c>
-      <c r="B94" t="s">
-        <v>19</v>
-      </c>
-      <c r="D94" t="s">
-        <v>87</v>
-      </c>
-      <c r="E94" t="s">
-        <v>53</v>
-      </c>
-      <c r="F94" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A95" t="s">
-        <v>32</v>
-      </c>
-      <c r="B95" t="s">
-        <v>19</v>
-      </c>
-      <c r="C95" t="s">
-        <v>20</v>
-      </c>
-      <c r="D95">
-        <v>1</v>
-      </c>
-      <c r="E95" t="s">
-        <v>40</v>
-      </c>
-      <c r="F95" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A96" t="s">
-        <v>32</v>
-      </c>
-      <c r="B96" t="s">
-        <v>19</v>
-      </c>
-      <c r="C96" t="s">
-        <v>104</v>
-      </c>
-      <c r="D96">
-        <v>1</v>
-      </c>
-      <c r="E96" t="s">
-        <v>105</v>
-      </c>
-      <c r="F96" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
         <v>32</v>
       </c>
       <c r="B97" t="s">
         <v>19</v>
       </c>
-      <c r="C97" t="s">
-        <v>106</v>
-      </c>
-      <c r="D97">
-        <v>1</v>
+      <c r="D97" t="s">
+        <v>87</v>
       </c>
       <c r="E97" t="s">
-        <v>105</v>
+        <v>53</v>
       </c>
       <c r="F97" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.3">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A98" t="s">
         <v>32</v>
       </c>
@@ -2818,19 +2829,19 @@
         <v>19</v>
       </c>
       <c r="C98" t="s">
-        <v>38</v>
+        <v>20</v>
       </c>
       <c r="D98">
         <v>1</v>
       </c>
       <c r="E98" t="s">
-        <v>53</v>
+        <v>40</v>
       </c>
       <c r="F98" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.3">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A99" t="s">
         <v>32</v>
       </c>
@@ -2838,19 +2849,19 @@
         <v>19</v>
       </c>
       <c r="C99" t="s">
-        <v>38</v>
+        <v>104</v>
       </c>
       <c r="D99">
         <v>1</v>
       </c>
       <c r="E99" t="s">
-        <v>53</v>
+        <v>105</v>
       </c>
       <c r="F99" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.3">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A100" t="s">
         <v>32</v>
       </c>
@@ -2858,152 +2869,158 @@
         <v>19</v>
       </c>
       <c r="C100" t="s">
+        <v>106</v>
+      </c>
+      <c r="D100">
+        <v>1</v>
+      </c>
+      <c r="E100" t="s">
+        <v>105</v>
+      </c>
+      <c r="F100" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A101" t="s">
+        <v>32</v>
+      </c>
+      <c r="B101" t="s">
+        <v>19</v>
+      </c>
+      <c r="C101" t="s">
+        <v>38</v>
+      </c>
+      <c r="D101">
+        <v>1</v>
+      </c>
+      <c r="E101" t="s">
+        <v>53</v>
+      </c>
+      <c r="F101" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A102" t="s">
+        <v>32</v>
+      </c>
+      <c r="B102" t="s">
+        <v>19</v>
+      </c>
+      <c r="C102" t="s">
+        <v>38</v>
+      </c>
+      <c r="D102">
+        <v>1</v>
+      </c>
+      <c r="E102" t="s">
+        <v>53</v>
+      </c>
+      <c r="F102" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A103" t="s">
+        <v>32</v>
+      </c>
+      <c r="B103" t="s">
+        <v>19</v>
+      </c>
+      <c r="C103" t="s">
         <v>206</v>
       </c>
-      <c r="E100" t="s">
+      <c r="E103" t="s">
         <v>103</v>
       </c>
-      <c r="F100" t="s">
+      <c r="F103" t="s">
         <v>204</v>
       </c>
     </row>
-    <row r="101" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A101" t="s">
-        <v>32</v>
-      </c>
-      <c r="B101" t="s">
+    <row r="104" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A104" t="s">
+        <v>32</v>
+      </c>
+      <c r="B104" t="s">
         <v>9</v>
       </c>
-      <c r="D101" t="s">
+      <c r="D104" t="s">
         <v>87</v>
       </c>
-      <c r="E101" t="s">
+      <c r="E104" t="s">
         <v>11</v>
       </c>
-      <c r="F101" t="s">
+      <c r="F104" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="102" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A102" t="s">
-        <v>32</v>
-      </c>
-      <c r="B102" t="s">
+    <row r="105" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A105" t="s">
+        <v>32</v>
+      </c>
+      <c r="B105" t="s">
         <v>9</v>
       </c>
-      <c r="C102" t="s">
+      <c r="C105" t="s">
         <v>10</v>
       </c>
-      <c r="D102">
-        <v>1</v>
-      </c>
-      <c r="E102" t="s">
-        <v>11</v>
-      </c>
-      <c r="F102" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="103" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A103" t="s">
-        <v>32</v>
-      </c>
-      <c r="B103" t="s">
-        <v>9</v>
-      </c>
-      <c r="C103" t="s">
-        <v>16</v>
-      </c>
-      <c r="D103">
-        <v>1</v>
-      </c>
-      <c r="E103" t="s">
-        <v>40</v>
-      </c>
-      <c r="F103" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="104" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A104" t="s">
-        <v>32</v>
-      </c>
-      <c r="B104" t="s">
-        <v>185</v>
-      </c>
-      <c r="D104" t="s">
-        <v>68</v>
-      </c>
-      <c r="E104" t="s">
-        <v>105</v>
-      </c>
-      <c r="F104" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="105" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A105" t="s">
-        <v>32</v>
-      </c>
-      <c r="B105" t="s">
-        <v>75</v>
-      </c>
-      <c r="D105" t="s">
-        <v>87</v>
+      <c r="D105">
+        <v>1</v>
       </c>
       <c r="E105" t="s">
         <v>11</v>
       </c>
       <c r="F105" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="106" spans="1:6" x14ac:dyDescent="0.3">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A106" t="s">
         <v>32</v>
       </c>
       <c r="B106" t="s">
+        <v>9</v>
+      </c>
+      <c r="C106" t="s">
+        <v>16</v>
+      </c>
+      <c r="D106">
+        <v>1</v>
+      </c>
+      <c r="E106" t="s">
+        <v>40</v>
+      </c>
+      <c r="F106" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A107" t="s">
+        <v>32</v>
+      </c>
+      <c r="B107" t="s">
+        <v>185</v>
+      </c>
+      <c r="D107" t="s">
+        <v>68</v>
+      </c>
+      <c r="E107" t="s">
+        <v>105</v>
+      </c>
+      <c r="F107" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A108" t="s">
+        <v>32</v>
+      </c>
+      <c r="B108" t="s">
         <v>75</v>
       </c>
-      <c r="C106" t="s">
-        <v>74</v>
-      </c>
-      <c r="E106" t="s">
-        <v>11</v>
-      </c>
-      <c r="F106" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="107" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A107" t="s">
-        <v>32</v>
-      </c>
-      <c r="B107" t="s">
-        <v>72</v>
-      </c>
-      <c r="D107" t="s">
+      <c r="D108" t="s">
         <v>87</v>
-      </c>
-      <c r="E107" t="s">
-        <v>11</v>
-      </c>
-      <c r="F107" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="108" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A108" t="s">
-        <v>32</v>
-      </c>
-      <c r="B108" t="s">
-        <v>72</v>
-      </c>
-      <c r="C108" t="s">
-        <v>70</v>
-      </c>
-      <c r="D108">
-        <v>2</v>
       </c>
       <c r="E108" t="s">
         <v>11</v>
@@ -3012,29 +3029,29 @@
         <v>71</v>
       </c>
     </row>
-    <row r="109" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A109" t="s">
         <v>32</v>
       </c>
       <c r="B109" t="s">
-        <v>186</v>
-      </c>
-      <c r="D109" t="s">
-        <v>65</v>
+        <v>75</v>
+      </c>
+      <c r="C109" t="s">
+        <v>74</v>
       </c>
       <c r="E109" t="s">
-        <v>85</v>
+        <v>11</v>
       </c>
       <c r="F109" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="110" spans="1:6" x14ac:dyDescent="0.3">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A110" t="s">
         <v>32</v>
       </c>
       <c r="B110" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D110" t="s">
         <v>87</v>
@@ -3046,15 +3063,18 @@
         <v>71</v>
       </c>
     </row>
-    <row r="111" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A111" t="s">
         <v>32</v>
       </c>
       <c r="B111" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C111" t="s">
-        <v>74</v>
+        <v>70</v>
+      </c>
+      <c r="D111">
+        <v>2</v>
       </c>
       <c r="E111" t="s">
         <v>11</v>
@@ -3063,35 +3083,32 @@
         <v>71</v>
       </c>
     </row>
-    <row r="112" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A112" t="s">
         <v>32</v>
       </c>
       <c r="B112" t="s">
-        <v>69</v>
+        <v>186</v>
       </c>
       <c r="D112" t="s">
+        <v>65</v>
+      </c>
+      <c r="E112" t="s">
+        <v>85</v>
+      </c>
+      <c r="F112" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A113" t="s">
+        <v>32</v>
+      </c>
+      <c r="B113" t="s">
+        <v>73</v>
+      </c>
+      <c r="D113" t="s">
         <v>87</v>
-      </c>
-      <c r="E112" t="s">
-        <v>11</v>
-      </c>
-      <c r="F112" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="113" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A113" t="s">
-        <v>32</v>
-      </c>
-      <c r="B113" t="s">
-        <v>69</v>
-      </c>
-      <c r="C113" t="s">
-        <v>70</v>
-      </c>
-      <c r="D113">
-        <v>2</v>
       </c>
       <c r="E113" t="s">
         <v>11</v>
@@ -3100,129 +3117,132 @@
         <v>71</v>
       </c>
     </row>
-    <row r="114" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A114" t="s">
         <v>32</v>
       </c>
       <c r="B114" t="s">
-        <v>92</v>
-      </c>
-      <c r="D114" t="s">
-        <v>87</v>
+        <v>73</v>
+      </c>
+      <c r="C114" t="s">
+        <v>74</v>
       </c>
       <c r="E114" t="s">
-        <v>53</v>
+        <v>11</v>
       </c>
       <c r="F114" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="115" spans="1:6" x14ac:dyDescent="0.3">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A115" t="s">
         <v>32</v>
       </c>
       <c r="B115" t="s">
-        <v>162</v>
+        <v>69</v>
       </c>
       <c r="D115" t="s">
         <v>87</v>
       </c>
       <c r="E115" t="s">
-        <v>116</v>
+        <v>11</v>
       </c>
       <c r="F115" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A116" t="s">
+        <v>32</v>
+      </c>
+      <c r="B116" t="s">
+        <v>69</v>
+      </c>
+      <c r="C116" t="s">
+        <v>70</v>
+      </c>
+      <c r="D116">
+        <v>2</v>
+      </c>
+      <c r="E116" t="s">
+        <v>11</v>
+      </c>
+      <c r="F116" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A117" t="s">
+        <v>32</v>
+      </c>
+      <c r="B117" t="s">
+        <v>92</v>
+      </c>
+      <c r="D117" t="s">
+        <v>87</v>
+      </c>
+      <c r="E117" t="s">
+        <v>53</v>
+      </c>
+      <c r="F117" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A118" t="s">
+        <v>32</v>
+      </c>
+      <c r="B118" t="s">
+        <v>162</v>
+      </c>
+      <c r="D118" t="s">
+        <v>87</v>
+      </c>
+      <c r="E118" t="s">
+        <v>116</v>
+      </c>
+      <c r="F118" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="116" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A116" t="s">
-        <v>32</v>
-      </c>
-      <c r="B116" t="s">
+    <row r="119" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A119" t="s">
+        <v>32</v>
+      </c>
+      <c r="B119" t="s">
         <v>162</v>
       </c>
-      <c r="C116" t="s">
+      <c r="C119" t="s">
         <v>164</v>
       </c>
-      <c r="D116">
-        <v>1</v>
-      </c>
-      <c r="E116" t="s">
-        <v>116</v>
-      </c>
-      <c r="F116" t="s">
+      <c r="D119">
+        <v>1</v>
+      </c>
+      <c r="E119" t="s">
+        <v>116</v>
+      </c>
+      <c r="F119" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="117" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A117" t="s">
-        <v>32</v>
-      </c>
-      <c r="B117" t="s">
-        <v>118</v>
-      </c>
-      <c r="D117" t="s">
-        <v>68</v>
-      </c>
-      <c r="E117" t="s">
-        <v>116</v>
-      </c>
-      <c r="F117" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="118" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A118" t="s">
-        <v>32</v>
-      </c>
-      <c r="B118" t="s">
-        <v>118</v>
-      </c>
-      <c r="C118" t="s">
-        <v>124</v>
-      </c>
-      <c r="E118" t="s">
-        <v>116</v>
-      </c>
-      <c r="F118" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="119" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A119" t="s">
-        <v>32</v>
-      </c>
-      <c r="B119" t="s">
-        <v>118</v>
-      </c>
-      <c r="C119" t="s">
-        <v>52</v>
-      </c>
-      <c r="E119" t="s">
-        <v>116</v>
-      </c>
-      <c r="F119" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="120" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A120" t="s">
         <v>32</v>
       </c>
       <c r="B120" t="s">
         <v>118</v>
       </c>
-      <c r="C120" t="s">
-        <v>129</v>
+      <c r="D120" t="s">
+        <v>68</v>
       </c>
       <c r="E120" t="s">
         <v>116</v>
       </c>
       <c r="F120" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="121" spans="1:6" x14ac:dyDescent="0.3">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A121" t="s">
         <v>32</v>
       </c>
@@ -3230,7 +3250,7 @@
         <v>118</v>
       </c>
       <c r="C121" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="E121" t="s">
         <v>116</v>
@@ -3239,7 +3259,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="122" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A122" t="s">
         <v>32</v>
       </c>
@@ -3247,16 +3267,16 @@
         <v>118</v>
       </c>
       <c r="C122" t="s">
-        <v>136</v>
+        <v>52</v>
       </c>
       <c r="E122" t="s">
         <v>116</v>
       </c>
       <c r="F122" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="123" spans="1:6" x14ac:dyDescent="0.3">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A123" t="s">
         <v>32</v>
       </c>
@@ -3264,16 +3284,16 @@
         <v>118</v>
       </c>
       <c r="C123" t="s">
-        <v>146</v>
+        <v>129</v>
       </c>
       <c r="E123" t="s">
         <v>116</v>
       </c>
       <c r="F123" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="124" spans="1:6" x14ac:dyDescent="0.3">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A124" t="s">
         <v>32</v>
       </c>
@@ -3281,16 +3301,16 @@
         <v>118</v>
       </c>
       <c r="C124" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="E124" t="s">
         <v>116</v>
       </c>
       <c r="F124" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="125" spans="1:6" x14ac:dyDescent="0.3">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="125" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A125" t="s">
         <v>32</v>
       </c>
@@ -3298,109 +3318,109 @@
         <v>118</v>
       </c>
       <c r="C125" t="s">
+        <v>136</v>
+      </c>
+      <c r="E125" t="s">
+        <v>116</v>
+      </c>
+      <c r="F125" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="126" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A126" t="s">
+        <v>32</v>
+      </c>
+      <c r="B126" t="s">
+        <v>118</v>
+      </c>
+      <c r="C126" t="s">
+        <v>146</v>
+      </c>
+      <c r="E126" t="s">
+        <v>116</v>
+      </c>
+      <c r="F126" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="127" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A127" t="s">
+        <v>32</v>
+      </c>
+      <c r="B127" t="s">
+        <v>118</v>
+      </c>
+      <c r="C127" t="s">
+        <v>120</v>
+      </c>
+      <c r="E127" t="s">
+        <v>116</v>
+      </c>
+      <c r="F127" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="128" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A128" t="s">
+        <v>32</v>
+      </c>
+      <c r="B128" t="s">
+        <v>118</v>
+      </c>
+      <c r="C128" t="s">
         <v>51</v>
       </c>
-      <c r="E125" t="s">
-        <v>116</v>
-      </c>
-      <c r="F125" t="s">
+      <c r="E128" t="s">
+        <v>116</v>
+      </c>
+      <c r="F128" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="126" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A126" t="s">
-        <v>32</v>
-      </c>
-      <c r="B126" t="s">
+    <row r="129" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A129" t="s">
+        <v>32</v>
+      </c>
+      <c r="B129" t="s">
         <v>165</v>
       </c>
-      <c r="D126" t="s">
+      <c r="D129" t="s">
         <v>87</v>
       </c>
-      <c r="E126" t="s">
-        <v>116</v>
-      </c>
-      <c r="F126" t="s">
+      <c r="E129" t="s">
+        <v>116</v>
+      </c>
+      <c r="F129" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="127" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A127" t="s">
-        <v>32</v>
-      </c>
-      <c r="B127" t="s">
+    <row r="130" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A130" t="s">
+        <v>32</v>
+      </c>
+      <c r="B130" t="s">
         <v>165</v>
       </c>
-      <c r="C127" t="s">
+      <c r="C130" t="s">
         <v>166</v>
       </c>
-      <c r="E127" t="s">
-        <v>116</v>
-      </c>
-      <c r="F127" t="s">
+      <c r="E130" t="s">
+        <v>116</v>
+      </c>
+      <c r="F130" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="128" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A128" t="s">
-        <v>32</v>
-      </c>
-      <c r="B128" t="s">
-        <v>149</v>
-      </c>
-      <c r="D128" t="s">
-        <v>68</v>
-      </c>
-      <c r="E128" t="s">
-        <v>116</v>
-      </c>
-      <c r="F128" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="129" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A129" t="s">
-        <v>32</v>
-      </c>
-      <c r="B129" t="s">
-        <v>149</v>
-      </c>
-      <c r="C129" t="s">
-        <v>151</v>
-      </c>
-      <c r="E129" t="s">
-        <v>116</v>
-      </c>
-      <c r="F129" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="130" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A130" t="s">
-        <v>32</v>
-      </c>
-      <c r="B130" t="s">
-        <v>149</v>
-      </c>
-      <c r="C130" t="s">
-        <v>49</v>
-      </c>
-      <c r="E130" t="s">
-        <v>116</v>
-      </c>
-      <c r="F130" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="131" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A131" t="s">
         <v>32</v>
       </c>
       <c r="B131" t="s">
         <v>149</v>
       </c>
-      <c r="C131" t="s">
-        <v>150</v>
+      <c r="D131" t="s">
+        <v>68</v>
       </c>
       <c r="E131" t="s">
         <v>116</v>
@@ -3409,7 +3429,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="132" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A132" t="s">
         <v>32</v>
       </c>
@@ -3417,7 +3437,7 @@
         <v>149</v>
       </c>
       <c r="C132" t="s">
-        <v>50</v>
+        <v>151</v>
       </c>
       <c r="E132" t="s">
         <v>116</v>
@@ -3426,32 +3446,32 @@
         <v>147</v>
       </c>
     </row>
-    <row r="133" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A133" t="s">
         <v>32</v>
       </c>
       <c r="B133" t="s">
-        <v>138</v>
-      </c>
-      <c r="D133" t="s">
-        <v>68</v>
+        <v>149</v>
+      </c>
+      <c r="C133" t="s">
+        <v>49</v>
       </c>
       <c r="E133" t="s">
         <v>116</v>
       </c>
       <c r="F133" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="134" spans="1:6" x14ac:dyDescent="0.3">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="134" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A134" t="s">
         <v>32</v>
       </c>
       <c r="B134" t="s">
-        <v>138</v>
+        <v>149</v>
       </c>
       <c r="C134" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="E134" t="s">
         <v>116</v>
@@ -3460,32 +3480,32 @@
         <v>147</v>
       </c>
     </row>
-    <row r="135" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A135" t="s">
         <v>32</v>
       </c>
       <c r="B135" t="s">
-        <v>138</v>
+        <v>149</v>
       </c>
       <c r="C135" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="E135" t="s">
         <v>116</v>
       </c>
       <c r="F135" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="136" spans="1:6" x14ac:dyDescent="0.3">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="136" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A136" t="s">
         <v>32</v>
       </c>
       <c r="B136" t="s">
         <v>138</v>
       </c>
-      <c r="C136" t="s">
-        <v>57</v>
+      <c r="D136" t="s">
+        <v>68</v>
       </c>
       <c r="E136" t="s">
         <v>116</v>
@@ -3494,7 +3514,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="137" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A137" t="s">
         <v>32</v>
       </c>
@@ -3502,16 +3522,16 @@
         <v>138</v>
       </c>
       <c r="C137" t="s">
-        <v>156</v>
+        <v>148</v>
       </c>
       <c r="E137" t="s">
         <v>116</v>
       </c>
       <c r="F137" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="138" spans="1:6" x14ac:dyDescent="0.3">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="138" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A138" t="s">
         <v>32</v>
       </c>
@@ -3519,16 +3539,16 @@
         <v>138</v>
       </c>
       <c r="C138" t="s">
-        <v>154</v>
+        <v>58</v>
       </c>
       <c r="E138" t="s">
         <v>116</v>
       </c>
       <c r="F138" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="139" spans="1:6" x14ac:dyDescent="0.3">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="139" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A139" t="s">
         <v>32</v>
       </c>
@@ -3536,16 +3556,16 @@
         <v>138</v>
       </c>
       <c r="C139" t="s">
-        <v>184</v>
+        <v>57</v>
       </c>
       <c r="E139" t="s">
         <v>116</v>
       </c>
       <c r="F139" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="140" spans="1:6" x14ac:dyDescent="0.3">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="140" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A140" t="s">
         <v>32</v>
       </c>
@@ -3553,7 +3573,7 @@
         <v>138</v>
       </c>
       <c r="C140" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="E140" t="s">
         <v>116</v>
@@ -3562,100 +3582,100 @@
         <v>158</v>
       </c>
     </row>
-    <row r="141" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A141" t="s">
         <v>32</v>
       </c>
       <c r="B141" t="s">
+        <v>138</v>
+      </c>
+      <c r="C141" t="s">
+        <v>154</v>
+      </c>
+      <c r="E141" t="s">
+        <v>116</v>
+      </c>
+      <c r="F141" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="142" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A142" t="s">
+        <v>32</v>
+      </c>
+      <c r="B142" t="s">
+        <v>138</v>
+      </c>
+      <c r="C142" t="s">
+        <v>184</v>
+      </c>
+      <c r="E142" t="s">
+        <v>116</v>
+      </c>
+      <c r="F142" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="143" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A143" t="s">
+        <v>32</v>
+      </c>
+      <c r="B143" t="s">
+        <v>138</v>
+      </c>
+      <c r="C143" t="s">
+        <v>157</v>
+      </c>
+      <c r="E143" t="s">
+        <v>116</v>
+      </c>
+      <c r="F143" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="144" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A144" t="s">
+        <v>32</v>
+      </c>
+      <c r="B144" t="s">
         <v>125</v>
       </c>
-      <c r="D141" t="s">
+      <c r="D144" t="s">
         <v>68</v>
       </c>
-      <c r="E141" t="s">
-        <v>116</v>
-      </c>
-      <c r="F141" t="s">
+      <c r="E144" t="s">
+        <v>116</v>
+      </c>
+      <c r="F144" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="142" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A142" t="s">
-        <v>32</v>
-      </c>
-      <c r="B142" t="s">
+    <row r="145" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A145" t="s">
+        <v>32</v>
+      </c>
+      <c r="B145" t="s">
         <v>125</v>
       </c>
-      <c r="C142" t="s">
+      <c r="C145" t="s">
         <v>127</v>
       </c>
-      <c r="E142" t="s">
-        <v>116</v>
-      </c>
-      <c r="F142" t="s">
+      <c r="E145" t="s">
+        <v>116</v>
+      </c>
+      <c r="F145" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="143" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A143" t="s">
-        <v>32</v>
-      </c>
-      <c r="B143" t="s">
-        <v>131</v>
-      </c>
-      <c r="D143" t="s">
-        <v>68</v>
-      </c>
-      <c r="E143" t="s">
-        <v>116</v>
-      </c>
-      <c r="F143" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="144" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A144" t="s">
-        <v>32</v>
-      </c>
-      <c r="B144" t="s">
-        <v>131</v>
-      </c>
-      <c r="C144" t="s">
-        <v>132</v>
-      </c>
-      <c r="E144" t="s">
-        <v>116</v>
-      </c>
-      <c r="F144" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="145" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A145" t="s">
-        <v>32</v>
-      </c>
-      <c r="B145" t="s">
-        <v>131</v>
-      </c>
-      <c r="C145" t="s">
-        <v>133</v>
-      </c>
-      <c r="E145" t="s">
-        <v>116</v>
-      </c>
-      <c r="F145" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="146" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A146" t="s">
         <v>32</v>
       </c>
       <c r="B146" t="s">
         <v>131</v>
       </c>
-      <c r="C146" t="s">
-        <v>134</v>
+      <c r="D146" t="s">
+        <v>68</v>
       </c>
       <c r="E146" t="s">
         <v>116</v>
@@ -3664,7 +3684,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="147" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A147" t="s">
         <v>32</v>
       </c>
@@ -3672,7 +3692,7 @@
         <v>131</v>
       </c>
       <c r="C147" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="E147" t="s">
         <v>116</v>
@@ -3681,126 +3701,117 @@
         <v>130</v>
       </c>
     </row>
-    <row r="148" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A148" t="s">
         <v>32</v>
       </c>
       <c r="B148" t="s">
+        <v>131</v>
+      </c>
+      <c r="C148" t="s">
+        <v>133</v>
+      </c>
+      <c r="E148" t="s">
+        <v>116</v>
+      </c>
+      <c r="F148" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="149" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A149" t="s">
+        <v>32</v>
+      </c>
+      <c r="B149" t="s">
+        <v>131</v>
+      </c>
+      <c r="C149" t="s">
+        <v>134</v>
+      </c>
+      <c r="E149" t="s">
+        <v>116</v>
+      </c>
+      <c r="F149" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="150" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A150" t="s">
+        <v>32</v>
+      </c>
+      <c r="B150" t="s">
+        <v>131</v>
+      </c>
+      <c r="C150" t="s">
+        <v>135</v>
+      </c>
+      <c r="E150" t="s">
+        <v>116</v>
+      </c>
+      <c r="F150" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="151" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A151" t="s">
+        <v>32</v>
+      </c>
+      <c r="B151" t="s">
         <v>126</v>
       </c>
-      <c r="D148" t="s">
+      <c r="D151" t="s">
         <v>68</v>
       </c>
-      <c r="E148" t="s">
-        <v>116</v>
-      </c>
-      <c r="F148" t="s">
+      <c r="E151" t="s">
+        <v>116</v>
+      </c>
+      <c r="F151" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="149" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A149" t="s">
-        <v>32</v>
-      </c>
-      <c r="B149" t="s">
+    <row r="152" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A152" t="s">
+        <v>32</v>
+      </c>
+      <c r="B152" t="s">
         <v>126</v>
       </c>
-      <c r="C149" t="s">
+      <c r="C152" t="s">
         <v>128</v>
       </c>
-      <c r="E149" t="s">
-        <v>116</v>
-      </c>
-      <c r="F149" t="s">
+      <c r="E152" t="s">
+        <v>116</v>
+      </c>
+      <c r="F152" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="150" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A150" t="s">
-        <v>32</v>
-      </c>
-      <c r="B150" t="s">
+    <row r="153" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A153" t="s">
+        <v>32</v>
+      </c>
+      <c r="B153" t="s">
         <v>98</v>
       </c>
-      <c r="D150" t="s">
+      <c r="D153" t="s">
         <v>87</v>
-      </c>
-      <c r="E150" t="s">
-        <v>14</v>
-      </c>
-      <c r="F150" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="151" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A151" t="s">
-        <v>32</v>
-      </c>
-      <c r="B151" t="s">
-        <v>13</v>
-      </c>
-      <c r="D151" t="s">
-        <v>87</v>
-      </c>
-      <c r="E151" t="s">
-        <v>14</v>
-      </c>
-      <c r="F151" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="152" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A152" t="s">
-        <v>32</v>
-      </c>
-      <c r="B152" t="s">
-        <v>13</v>
-      </c>
-      <c r="C152" t="s">
-        <v>10</v>
-      </c>
-      <c r="D152">
-        <v>1</v>
-      </c>
-      <c r="E152" t="s">
-        <v>14</v>
-      </c>
-      <c r="F152" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="153" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A153" t="s">
-        <v>32</v>
-      </c>
-      <c r="B153" t="s">
-        <v>13</v>
-      </c>
-      <c r="C153" t="s">
-        <v>20</v>
-      </c>
-      <c r="D153">
-        <v>1</v>
       </c>
       <c r="E153" t="s">
         <v>14</v>
       </c>
       <c r="F153" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="154" spans="1:6" x14ac:dyDescent="0.3">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="154" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A154" t="s">
         <v>32</v>
       </c>
       <c r="B154" t="s">
         <v>13</v>
       </c>
-      <c r="C154" t="s">
-        <v>18</v>
-      </c>
-      <c r="D154">
-        <v>1</v>
+      <c r="D154" t="s">
+        <v>87</v>
       </c>
       <c r="E154" t="s">
         <v>14</v>
@@ -3809,69 +3820,75 @@
         <v>17</v>
       </c>
     </row>
-    <row r="155" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A155" t="s">
         <v>32</v>
       </c>
       <c r="B155" t="s">
+        <v>13</v>
+      </c>
+      <c r="C155" t="s">
+        <v>10</v>
+      </c>
+      <c r="D155">
+        <v>1</v>
+      </c>
+      <c r="E155" t="s">
+        <v>14</v>
+      </c>
+      <c r="F155" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="156" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A156" t="s">
+        <v>32</v>
+      </c>
+      <c r="B156" t="s">
+        <v>13</v>
+      </c>
+      <c r="C156" t="s">
+        <v>20</v>
+      </c>
+      <c r="D156">
+        <v>1</v>
+      </c>
+      <c r="E156" t="s">
+        <v>14</v>
+      </c>
+      <c r="F156" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="157" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A157" t="s">
+        <v>32</v>
+      </c>
+      <c r="B157" t="s">
+        <v>13</v>
+      </c>
+      <c r="C157" t="s">
+        <v>18</v>
+      </c>
+      <c r="D157">
+        <v>1</v>
+      </c>
+      <c r="E157" t="s">
+        <v>14</v>
+      </c>
+      <c r="F157" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="158" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A158" t="s">
+        <v>32</v>
+      </c>
+      <c r="B158" t="s">
         <v>97</v>
       </c>
-      <c r="D155" t="s">
+      <c r="D158" t="s">
         <v>87</v>
-      </c>
-      <c r="E155" t="s">
-        <v>54</v>
-      </c>
-      <c r="F155" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="156" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A156" t="s">
-        <v>32</v>
-      </c>
-      <c r="B156" t="s">
-        <v>97</v>
-      </c>
-      <c r="C156" t="s">
-        <v>191</v>
-      </c>
-      <c r="E156" t="s">
-        <v>24</v>
-      </c>
-      <c r="F156" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="157" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A157" t="s">
-        <v>32</v>
-      </c>
-      <c r="B157" t="s">
-        <v>33</v>
-      </c>
-      <c r="D157" t="s">
-        <v>87</v>
-      </c>
-      <c r="E157" t="s">
-        <v>54</v>
-      </c>
-      <c r="F157" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="158" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A158" t="s">
-        <v>32</v>
-      </c>
-      <c r="B158" t="s">
-        <v>33</v>
-      </c>
-      <c r="C158" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="D158">
-        <v>1</v>
       </c>
       <c r="E158" t="s">
         <v>54</v>
@@ -3880,35 +3897,32 @@
         <v>63</v>
       </c>
     </row>
-    <row r="159" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A159" t="s">
         <v>32</v>
       </c>
       <c r="B159" t="s">
-        <v>33</v>
-      </c>
-      <c r="C159" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="D159">
-        <v>1</v>
+        <v>97</v>
+      </c>
+      <c r="C159" t="s">
+        <v>191</v>
       </c>
       <c r="E159" t="s">
-        <v>54</v>
+        <v>24</v>
       </c>
       <c r="F159" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="160" spans="1:6" x14ac:dyDescent="0.3">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="160" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A160" t="s">
         <v>32</v>
       </c>
       <c r="B160" t="s">
         <v>33</v>
       </c>
-      <c r="C160" s="1" t="s">
-        <v>57</v>
+      <c r="D160" t="s">
+        <v>87</v>
       </c>
       <c r="E160" t="s">
         <v>54</v>
@@ -3917,7 +3931,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="161" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A161" t="s">
         <v>32</v>
       </c>
@@ -3925,47 +3939,104 @@
         <v>33</v>
       </c>
       <c r="C161" s="1" t="s">
-        <v>195</v>
+        <v>39</v>
+      </c>
+      <c r="D161">
+        <v>1</v>
       </c>
       <c r="E161" t="s">
         <v>54</v>
       </c>
       <c r="F161" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="162" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A162" t="s">
+        <v>32</v>
+      </c>
+      <c r="B162" t="s">
+        <v>33</v>
+      </c>
+      <c r="C162" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D162">
+        <v>1</v>
+      </c>
+      <c r="E162" t="s">
+        <v>54</v>
+      </c>
+      <c r="F162" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="163" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A163" t="s">
+        <v>32</v>
+      </c>
+      <c r="B163" t="s">
+        <v>33</v>
+      </c>
+      <c r="C163" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="E163" t="s">
+        <v>54</v>
+      </c>
+      <c r="F163" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="164" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A164" t="s">
+        <v>32</v>
+      </c>
+      <c r="B164" t="s">
+        <v>33</v>
+      </c>
+      <c r="C164" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="E164" t="s">
+        <v>54</v>
+      </c>
+      <c r="F164" t="s">
         <v>193</v>
       </c>
     </row>
-    <row r="162" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A162" t="s">
-        <v>32</v>
-      </c>
-      <c r="B162" t="s">
+    <row r="165" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A165" t="s">
+        <v>32</v>
+      </c>
+      <c r="B165" t="s">
         <v>182</v>
       </c>
-      <c r="C162" s="1"/>
-      <c r="D162" t="s">
+      <c r="C165" s="1"/>
+      <c r="D165" t="s">
         <v>68</v>
       </c>
-      <c r="E162" t="s">
-        <v>116</v>
-      </c>
-      <c r="F162" t="s">
+      <c r="E165" t="s">
+        <v>116</v>
+      </c>
+      <c r="F165" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="163" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A163" t="s">
-        <v>32</v>
-      </c>
-      <c r="B163" t="s">
+    <row r="166" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A166" t="s">
+        <v>32</v>
+      </c>
+      <c r="B166" t="s">
         <v>88</v>
       </c>
-      <c r="D163" t="s">
+      <c r="D166" t="s">
         <v>65</v>
       </c>
-      <c r="E163" t="s">
+      <c r="E166" t="s">
         <v>24</v>
       </c>
-      <c r="F163" t="s">
+      <c r="F166" t="s">
         <v>89</v>
       </c>
     </row>

</xml_diff>

<commit_message>
[PowerPoint] Added snippets that acts on selections
</commit_message>
<xml_diff>
--- a/snippet-extractor-metadata/powerpoint.xlsx
+++ b/snippet-extractor-metadata/powerpoint.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7C414EC-35C0-4625-9957-123F9D615DF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A2CA723-45CB-4135-8A1A-0329A73196F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25180" windowHeight="16140" xr2:uid="{CB5595D7-4492-4192-A1C1-2583BA1957AA}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="831" uniqueCount="215">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="856" uniqueCount="223">
   <si>
     <t>Class</t>
   </si>
@@ -665,6 +665,30 @@
   </si>
   <si>
     <t>ShapeGetImageFormatType</t>
+  </si>
+  <si>
+    <t>getParentTextFrame</t>
+  </si>
+  <si>
+    <t>getParentShape</t>
+  </si>
+  <si>
+    <t>getParentSlide</t>
+  </si>
+  <si>
+    <t>getSlideById</t>
+  </si>
+  <si>
+    <t>powerpoint-slide-management-get-slide-by-id</t>
+  </si>
+  <si>
+    <t>getItemOrNullObject</t>
+  </si>
+  <si>
+    <t>powerpoint-shapes-get-shape-by-id</t>
+  </si>
+  <si>
+    <t>getShapeById</t>
   </si>
 </sst>
 </file>
@@ -745,10 +769,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{78C585A5-D505-49C6-9CA1-8E6558948317}" name="Snippets" displayName="Snippets" ref="A1:F166" totalsRowShown="0" headerRowDxfId="4">
-  <autoFilter ref="A1:F166" xr:uid="{EAC65D03-FDD2-4352-A5F3-1CDEDE6251B2}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F162">
-    <sortCondition ref="B1:B162"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{78C585A5-D505-49C6-9CA1-8E6558948317}" name="Snippets" displayName="Snippets" ref="A1:F171" totalsRowShown="0" headerRowDxfId="4">
+  <autoFilter ref="A1:F171" xr:uid="{EAC65D03-FDD2-4352-A5F3-1CDEDE6251B2}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F167">
+    <sortCondition ref="B1:B167"/>
   </sortState>
   <tableColumns count="6">
     <tableColumn id="6" xr3:uid="{408888B8-C1DD-4B51-B1EB-5663F091D142}" name="Package"/>
@@ -1059,7 +1083,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{809930CD-A227-47DC-AAA4-BB816AEDEB59}">
-  <dimension ref="A1:F166"/>
+  <dimension ref="A1:F171"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="11.453125" bestFit="1" customWidth="1"/>
@@ -1962,16 +1986,16 @@
       <c r="B50" t="s">
         <v>45</v>
       </c>
-      <c r="C50" s="2" t="s">
+      <c r="C50" t="s">
         <v>106</v>
       </c>
       <c r="D50">
         <v>1</v>
       </c>
-      <c r="E50" s="2" t="s">
+      <c r="E50" t="s">
         <v>211</v>
       </c>
-      <c r="F50" s="2" t="s">
+      <c r="F50" t="s">
         <v>213</v>
       </c>
     </row>
@@ -1982,17 +2006,17 @@
       <c r="B51" t="s">
         <v>45</v>
       </c>
-      <c r="C51" t="s">
-        <v>161</v>
+      <c r="C51" s="2" t="s">
+        <v>217</v>
       </c>
       <c r="D51">
         <v>1</v>
       </c>
-      <c r="E51" t="s">
-        <v>116</v>
-      </c>
-      <c r="F51" t="s">
-        <v>160</v>
+      <c r="E51" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="F51" s="2" t="s">
+        <v>193</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.35">
@@ -2003,16 +2027,16 @@
         <v>45</v>
       </c>
       <c r="C52" t="s">
-        <v>208</v>
+        <v>161</v>
       </c>
       <c r="D52">
         <v>1</v>
       </c>
       <c r="E52" t="s">
-        <v>103</v>
+        <v>116</v>
       </c>
       <c r="F52" t="s">
-        <v>209</v>
+        <v>160</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.35">
@@ -2023,16 +2047,16 @@
         <v>45</v>
       </c>
       <c r="C53" t="s">
-        <v>176</v>
+        <v>208</v>
       </c>
       <c r="D53">
         <v>1</v>
       </c>
       <c r="E53" t="s">
-        <v>168</v>
+        <v>103</v>
       </c>
       <c r="F53" t="s">
-        <v>177</v>
+        <v>209</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.35">
@@ -2043,13 +2067,16 @@
         <v>45</v>
       </c>
       <c r="C54" t="s">
-        <v>58</v>
+        <v>176</v>
+      </c>
+      <c r="D54">
+        <v>1</v>
       </c>
       <c r="E54" t="s">
-        <v>53</v>
+        <v>168</v>
       </c>
       <c r="F54" t="s">
-        <v>44</v>
+        <v>177</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.35">
@@ -2060,13 +2087,13 @@
         <v>45</v>
       </c>
       <c r="C55" t="s">
-        <v>108</v>
+        <v>58</v>
       </c>
       <c r="E55" t="s">
-        <v>109</v>
+        <v>53</v>
       </c>
       <c r="F55" t="s">
-        <v>110</v>
+        <v>44</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.35">
@@ -2077,13 +2104,13 @@
         <v>45</v>
       </c>
       <c r="C56" t="s">
-        <v>52</v>
+        <v>108</v>
       </c>
       <c r="E56" t="s">
-        <v>53</v>
+        <v>109</v>
       </c>
       <c r="F56" t="s">
-        <v>48</v>
+        <v>110</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.35">
@@ -2094,7 +2121,7 @@
         <v>45</v>
       </c>
       <c r="C57" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="E57" t="s">
         <v>53</v>
@@ -2111,13 +2138,13 @@
         <v>45</v>
       </c>
       <c r="C58" t="s">
-        <v>196</v>
+        <v>49</v>
       </c>
       <c r="E58" t="s">
-        <v>85</v>
+        <v>53</v>
       </c>
       <c r="F58" t="s">
-        <v>197</v>
+        <v>48</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.35">
@@ -2128,13 +2155,13 @@
         <v>45</v>
       </c>
       <c r="C59" t="s">
-        <v>50</v>
+        <v>196</v>
       </c>
       <c r="E59" t="s">
-        <v>53</v>
+        <v>85</v>
       </c>
       <c r="F59" t="s">
-        <v>48</v>
+        <v>197</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.35">
@@ -2145,13 +2172,13 @@
         <v>45</v>
       </c>
       <c r="C60" t="s">
-        <v>86</v>
+        <v>50</v>
       </c>
       <c r="E60" t="s">
-        <v>85</v>
+        <v>53</v>
       </c>
       <c r="F60" t="s">
-        <v>81</v>
+        <v>48</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.35">
@@ -2162,13 +2189,13 @@
         <v>45</v>
       </c>
       <c r="C61" t="s">
-        <v>51</v>
+        <v>86</v>
       </c>
       <c r="E61" t="s">
-        <v>53</v>
+        <v>85</v>
       </c>
       <c r="F61" t="s">
-        <v>48</v>
+        <v>81</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.35">
@@ -2179,13 +2206,13 @@
         <v>45</v>
       </c>
       <c r="C62" t="s">
-        <v>178</v>
+        <v>51</v>
       </c>
       <c r="E62" t="s">
-        <v>168</v>
+        <v>53</v>
       </c>
       <c r="F62" t="s">
-        <v>177</v>
+        <v>48</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.35">
@@ -2193,16 +2220,16 @@
         <v>32</v>
       </c>
       <c r="B63" t="s">
-        <v>95</v>
-      </c>
-      <c r="D63" t="s">
-        <v>68</v>
+        <v>45</v>
+      </c>
+      <c r="C63" t="s">
+        <v>178</v>
       </c>
       <c r="E63" t="s">
-        <v>24</v>
+        <v>168</v>
       </c>
       <c r="F63" t="s">
-        <v>26</v>
+        <v>177</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.35">
@@ -2210,16 +2237,16 @@
         <v>32</v>
       </c>
       <c r="B64" t="s">
-        <v>187</v>
+        <v>95</v>
       </c>
       <c r="D64" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="E64" t="s">
         <v>24</v>
       </c>
       <c r="F64" t="s">
-        <v>89</v>
+        <v>26</v>
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.35">
@@ -2227,16 +2254,16 @@
         <v>32</v>
       </c>
       <c r="B65" t="s">
-        <v>21</v>
+        <v>187</v>
       </c>
       <c r="D65" t="s">
-        <v>87</v>
+        <v>65</v>
       </c>
       <c r="E65" t="s">
-        <v>85</v>
+        <v>24</v>
       </c>
       <c r="F65" t="s">
-        <v>81</v>
+        <v>89</v>
       </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.35">
@@ -2246,17 +2273,14 @@
       <c r="B66" t="s">
         <v>21</v>
       </c>
-      <c r="C66" t="s">
-        <v>25</v>
-      </c>
-      <c r="D66">
-        <v>1</v>
+      <c r="D66" t="s">
+        <v>87</v>
       </c>
       <c r="E66" t="s">
-        <v>24</v>
+        <v>85</v>
       </c>
       <c r="F66" t="s">
-        <v>26</v>
+        <v>81</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.35">
@@ -2267,16 +2291,16 @@
         <v>21</v>
       </c>
       <c r="C67" t="s">
-        <v>111</v>
+        <v>25</v>
       </c>
       <c r="D67">
         <v>1</v>
       </c>
       <c r="E67" t="s">
-        <v>109</v>
+        <v>24</v>
       </c>
       <c r="F67" t="s">
-        <v>112</v>
+        <v>26</v>
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.35">
@@ -2287,16 +2311,16 @@
         <v>21</v>
       </c>
       <c r="C68" t="s">
-        <v>27</v>
+        <v>111</v>
       </c>
       <c r="D68">
         <v>1</v>
       </c>
       <c r="E68" t="s">
-        <v>24</v>
+        <v>109</v>
       </c>
       <c r="F68" t="s">
-        <v>28</v>
+        <v>112</v>
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.35">
@@ -2307,16 +2331,16 @@
         <v>21</v>
       </c>
       <c r="C69" t="s">
-        <v>115</v>
+        <v>27</v>
       </c>
       <c r="D69">
         <v>1</v>
       </c>
       <c r="E69" t="s">
-        <v>116</v>
+        <v>24</v>
       </c>
       <c r="F69" t="s">
-        <v>117</v>
+        <v>28</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.35">
@@ -2327,16 +2351,16 @@
         <v>21</v>
       </c>
       <c r="C70" t="s">
-        <v>29</v>
+        <v>115</v>
       </c>
       <c r="D70">
         <v>1</v>
       </c>
       <c r="E70" t="s">
-        <v>24</v>
+        <v>116</v>
       </c>
       <c r="F70" t="s">
-        <v>30</v>
+        <v>117</v>
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.35">
@@ -2347,16 +2371,16 @@
         <v>21</v>
       </c>
       <c r="C71" t="s">
-        <v>91</v>
+        <v>29</v>
       </c>
       <c r="D71">
         <v>1</v>
       </c>
       <c r="E71" t="s">
-        <v>116</v>
+        <v>24</v>
       </c>
       <c r="F71" t="s">
-        <v>160</v>
+        <v>30</v>
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.35">
@@ -2367,16 +2391,16 @@
         <v>21</v>
       </c>
       <c r="C72" t="s">
-        <v>16</v>
+        <v>91</v>
       </c>
       <c r="D72">
         <v>1</v>
       </c>
       <c r="E72" t="s">
-        <v>14</v>
+        <v>116</v>
       </c>
       <c r="F72" t="s">
-        <v>22</v>
+        <v>160</v>
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.35">
@@ -2387,16 +2411,16 @@
         <v>21</v>
       </c>
       <c r="C73" t="s">
-        <v>70</v>
+        <v>16</v>
       </c>
       <c r="D73">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E73" t="s">
-        <v>85</v>
+        <v>14</v>
       </c>
       <c r="F73" t="s">
-        <v>81</v>
+        <v>22</v>
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.35">
@@ -2404,10 +2428,13 @@
         <v>32</v>
       </c>
       <c r="B74" t="s">
-        <v>59</v>
-      </c>
-      <c r="D74" t="s">
-        <v>87</v>
+        <v>21</v>
+      </c>
+      <c r="C74" t="s">
+        <v>70</v>
+      </c>
+      <c r="D74">
+        <v>2</v>
       </c>
       <c r="E74" t="s">
         <v>85</v>
@@ -2423,17 +2450,14 @@
       <c r="B75" t="s">
         <v>59</v>
       </c>
-      <c r="C75" t="s">
-        <v>179</v>
-      </c>
-      <c r="D75">
-        <v>1</v>
+      <c r="D75" t="s">
+        <v>87</v>
       </c>
       <c r="E75" t="s">
-        <v>168</v>
+        <v>85</v>
       </c>
       <c r="F75" t="s">
-        <v>173</v>
+        <v>81</v>
       </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.35">
@@ -2444,16 +2468,16 @@
         <v>59</v>
       </c>
       <c r="C76" t="s">
-        <v>60</v>
+        <v>179</v>
       </c>
       <c r="D76">
         <v>1</v>
       </c>
       <c r="E76" t="s">
-        <v>53</v>
+        <v>168</v>
       </c>
       <c r="F76" t="s">
-        <v>44</v>
+        <v>173</v>
       </c>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.35">
@@ -2464,13 +2488,16 @@
         <v>59</v>
       </c>
       <c r="C77" t="s">
-        <v>93</v>
+        <v>60</v>
+      </c>
+      <c r="D77">
+        <v>1</v>
       </c>
       <c r="E77" t="s">
         <v>53</v>
       </c>
       <c r="F77" t="s">
-        <v>94</v>
+        <v>44</v>
       </c>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.35">
@@ -2481,13 +2508,13 @@
         <v>59</v>
       </c>
       <c r="C78" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="E78" t="s">
-        <v>85</v>
+        <v>53</v>
       </c>
       <c r="F78" t="s">
-        <v>81</v>
+        <v>94</v>
       </c>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.35">
@@ -2498,13 +2525,13 @@
         <v>59</v>
       </c>
       <c r="C79" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="E79" t="s">
-        <v>53</v>
+        <v>85</v>
       </c>
       <c r="F79" t="s">
-        <v>44</v>
+        <v>81</v>
       </c>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.35">
@@ -2512,10 +2539,10 @@
         <v>32</v>
       </c>
       <c r="B80" t="s">
-        <v>189</v>
-      </c>
-      <c r="D80" t="s">
-        <v>65</v>
+        <v>59</v>
+      </c>
+      <c r="C80" t="s">
+        <v>86</v>
       </c>
       <c r="E80" t="s">
         <v>53</v>
@@ -2529,16 +2556,16 @@
         <v>32</v>
       </c>
       <c r="B81" t="s">
-        <v>61</v>
+        <v>189</v>
       </c>
       <c r="D81" t="s">
-        <v>87</v>
+        <v>65</v>
       </c>
       <c r="E81" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F81" t="s">
-        <v>193</v>
+        <v>44</v>
       </c>
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.35">
@@ -2548,14 +2575,14 @@
       <c r="B82" t="s">
         <v>61</v>
       </c>
-      <c r="C82" t="s">
-        <v>62</v>
+      <c r="D82" t="s">
+        <v>87</v>
       </c>
       <c r="E82" t="s">
         <v>54</v>
       </c>
       <c r="F82" t="s">
-        <v>56</v>
+        <v>193</v>
       </c>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.35">
@@ -2566,13 +2593,13 @@
         <v>61</v>
       </c>
       <c r="C83" t="s">
-        <v>190</v>
+        <v>62</v>
       </c>
       <c r="E83" t="s">
-        <v>24</v>
+        <v>54</v>
       </c>
       <c r="F83" t="s">
-        <v>89</v>
+        <v>56</v>
       </c>
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.35">
@@ -2580,10 +2607,10 @@
         <v>32</v>
       </c>
       <c r="B84" t="s">
-        <v>188</v>
-      </c>
-      <c r="D84" t="s">
-        <v>65</v>
+        <v>61</v>
+      </c>
+      <c r="C84" t="s">
+        <v>190</v>
       </c>
       <c r="E84" t="s">
         <v>24</v>
@@ -2596,35 +2623,33 @@
       <c r="A85" t="s">
         <v>32</v>
       </c>
-      <c r="B85" s="2" t="s">
-        <v>214</v>
-      </c>
-      <c r="C85" s="2"/>
+      <c r="B85" t="s">
+        <v>188</v>
+      </c>
       <c r="D85" t="s">
         <v>65</v>
       </c>
-      <c r="E85" s="2" t="s">
-        <v>211</v>
-      </c>
-      <c r="F85" s="2" t="s">
-        <v>212</v>
+      <c r="E85" t="s">
+        <v>24</v>
+      </c>
+      <c r="F85" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
         <v>32</v>
       </c>
-      <c r="B86" s="2" t="s">
-        <v>210</v>
-      </c>
-      <c r="C86" s="2"/>
+      <c r="B86" t="s">
+        <v>214</v>
+      </c>
       <c r="D86" t="s">
-        <v>68</v>
-      </c>
-      <c r="E86" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="E86" t="s">
         <v>211</v>
       </c>
-      <c r="F86" s="2" t="s">
+      <c r="F86" t="s">
         <v>212</v>
       </c>
     </row>
@@ -2633,16 +2658,16 @@
         <v>32</v>
       </c>
       <c r="B87" t="s">
-        <v>113</v>
+        <v>210</v>
       </c>
       <c r="D87" t="s">
-        <v>87</v>
+        <v>68</v>
       </c>
       <c r="E87" t="s">
-        <v>109</v>
+        <v>211</v>
       </c>
       <c r="F87" t="s">
-        <v>110</v>
+        <v>212</v>
       </c>
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.35">
@@ -2652,11 +2677,8 @@
       <c r="B88" t="s">
         <v>113</v>
       </c>
-      <c r="C88" t="s">
-        <v>114</v>
-      </c>
-      <c r="D88">
-        <v>1</v>
+      <c r="D88" t="s">
+        <v>87</v>
       </c>
       <c r="E88" t="s">
         <v>109</v>
@@ -2670,16 +2692,19 @@
         <v>32</v>
       </c>
       <c r="B89" t="s">
-        <v>80</v>
-      </c>
-      <c r="D89" t="s">
-        <v>65</v>
+        <v>113</v>
+      </c>
+      <c r="C89" t="s">
+        <v>114</v>
+      </c>
+      <c r="D89">
+        <v>1</v>
       </c>
       <c r="E89" t="s">
-        <v>85</v>
+        <v>109</v>
       </c>
       <c r="F89" t="s">
-        <v>79</v>
+        <v>110</v>
       </c>
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.35">
@@ -2687,10 +2712,10 @@
         <v>32</v>
       </c>
       <c r="B90" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="D90" t="s">
-        <v>87</v>
+        <v>65</v>
       </c>
       <c r="E90" t="s">
         <v>85</v>
@@ -2706,8 +2731,8 @@
       <c r="B91" t="s">
         <v>83</v>
       </c>
-      <c r="C91" t="s">
-        <v>84</v>
+      <c r="D91" t="s">
+        <v>87</v>
       </c>
       <c r="E91" t="s">
         <v>85</v>
@@ -2721,16 +2746,16 @@
         <v>32</v>
       </c>
       <c r="B92" t="s">
-        <v>90</v>
-      </c>
-      <c r="D92" t="s">
-        <v>87</v>
+        <v>83</v>
+      </c>
+      <c r="C92" t="s">
+        <v>84</v>
       </c>
       <c r="E92" t="s">
-        <v>53</v>
+        <v>85</v>
       </c>
       <c r="F92" t="s">
-        <v>44</v>
+        <v>79</v>
       </c>
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.35">
@@ -2740,17 +2765,14 @@
       <c r="B93" t="s">
         <v>90</v>
       </c>
-      <c r="C93" t="s">
-        <v>91</v>
-      </c>
-      <c r="D93">
-        <v>1</v>
+      <c r="D93" t="s">
+        <v>87</v>
       </c>
       <c r="E93" t="s">
         <v>53</v>
       </c>
       <c r="F93" t="s">
-        <v>35</v>
+        <v>44</v>
       </c>
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.35">
@@ -2758,16 +2780,19 @@
         <v>32</v>
       </c>
       <c r="B94" t="s">
-        <v>78</v>
-      </c>
-      <c r="D94" t="s">
-        <v>65</v>
+        <v>90</v>
+      </c>
+      <c r="C94" t="s">
+        <v>91</v>
+      </c>
+      <c r="D94">
+        <v>1</v>
       </c>
       <c r="E94" t="s">
-        <v>85</v>
+        <v>53</v>
       </c>
       <c r="F94" t="s">
-        <v>79</v>
+        <v>35</v>
       </c>
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.35">
@@ -2775,16 +2800,19 @@
         <v>32</v>
       </c>
       <c r="B95" t="s">
-        <v>180</v>
-      </c>
-      <c r="D95" t="s">
-        <v>65</v>
-      </c>
-      <c r="E95" t="s">
-        <v>168</v>
-      </c>
-      <c r="F95" t="s">
-        <v>181</v>
+        <v>90</v>
+      </c>
+      <c r="C95" s="2" t="s">
+        <v>220</v>
+      </c>
+      <c r="D95">
+        <v>1</v>
+      </c>
+      <c r="E95" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="F95" s="2" t="s">
+        <v>222</v>
       </c>
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.35">
@@ -2792,16 +2820,16 @@
         <v>32</v>
       </c>
       <c r="B96" t="s">
-        <v>180</v>
+        <v>78</v>
       </c>
       <c r="D96" t="s">
         <v>65</v>
       </c>
       <c r="E96" t="s">
-        <v>168</v>
+        <v>85</v>
       </c>
       <c r="F96" t="s">
-        <v>177</v>
+        <v>79</v>
       </c>
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.35">
@@ -2809,16 +2837,16 @@
         <v>32</v>
       </c>
       <c r="B97" t="s">
-        <v>19</v>
+        <v>180</v>
       </c>
       <c r="D97" t="s">
-        <v>87</v>
+        <v>65</v>
       </c>
       <c r="E97" t="s">
-        <v>53</v>
+        <v>168</v>
       </c>
       <c r="F97" t="s">
-        <v>46</v>
+        <v>181</v>
       </c>
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.35">
@@ -2826,19 +2854,16 @@
         <v>32</v>
       </c>
       <c r="B98" t="s">
-        <v>19</v>
-      </c>
-      <c r="C98" t="s">
-        <v>20</v>
-      </c>
-      <c r="D98">
-        <v>1</v>
+        <v>180</v>
+      </c>
+      <c r="D98" t="s">
+        <v>65</v>
       </c>
       <c r="E98" t="s">
-        <v>40</v>
+        <v>168</v>
       </c>
       <c r="F98" t="s">
-        <v>43</v>
+        <v>177</v>
       </c>
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.35">
@@ -2848,17 +2873,14 @@
       <c r="B99" t="s">
         <v>19</v>
       </c>
-      <c r="C99" t="s">
-        <v>104</v>
-      </c>
-      <c r="D99">
-        <v>1</v>
+      <c r="D99" t="s">
+        <v>87</v>
       </c>
       <c r="E99" t="s">
-        <v>105</v>
+        <v>53</v>
       </c>
       <c r="F99" t="s">
-        <v>107</v>
+        <v>46</v>
       </c>
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.35">
@@ -2869,16 +2891,16 @@
         <v>19</v>
       </c>
       <c r="C100" t="s">
-        <v>106</v>
+        <v>20</v>
       </c>
       <c r="D100">
         <v>1</v>
       </c>
       <c r="E100" t="s">
-        <v>105</v>
+        <v>40</v>
       </c>
       <c r="F100" t="s">
-        <v>107</v>
+        <v>43</v>
       </c>
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.35">
@@ -2889,16 +2911,16 @@
         <v>19</v>
       </c>
       <c r="C101" t="s">
-        <v>38</v>
+        <v>104</v>
       </c>
       <c r="D101">
         <v>1</v>
       </c>
       <c r="E101" t="s">
-        <v>53</v>
+        <v>105</v>
       </c>
       <c r="F101" t="s">
-        <v>46</v>
+        <v>107</v>
       </c>
     </row>
     <row r="102" spans="1:6" x14ac:dyDescent="0.35">
@@ -2909,16 +2931,16 @@
         <v>19</v>
       </c>
       <c r="C102" t="s">
-        <v>38</v>
+        <v>106</v>
       </c>
       <c r="D102">
         <v>1</v>
       </c>
       <c r="E102" t="s">
-        <v>53</v>
+        <v>105</v>
       </c>
       <c r="F102" t="s">
-        <v>38</v>
+        <v>107</v>
       </c>
     </row>
     <row r="103" spans="1:6" x14ac:dyDescent="0.35">
@@ -2929,13 +2951,16 @@
         <v>19</v>
       </c>
       <c r="C103" t="s">
-        <v>206</v>
+        <v>38</v>
+      </c>
+      <c r="D103">
+        <v>1</v>
       </c>
       <c r="E103" t="s">
-        <v>103</v>
+        <v>53</v>
       </c>
       <c r="F103" t="s">
-        <v>204</v>
+        <v>46</v>
       </c>
     </row>
     <row r="104" spans="1:6" x14ac:dyDescent="0.35">
@@ -2943,16 +2968,19 @@
         <v>32</v>
       </c>
       <c r="B104" t="s">
-        <v>9</v>
-      </c>
-      <c r="D104" t="s">
-        <v>87</v>
+        <v>19</v>
+      </c>
+      <c r="C104" t="s">
+        <v>38</v>
+      </c>
+      <c r="D104">
+        <v>1</v>
       </c>
       <c r="E104" t="s">
-        <v>11</v>
+        <v>53</v>
       </c>
       <c r="F104" t="s">
-        <v>12</v>
+        <v>38</v>
       </c>
     </row>
     <row r="105" spans="1:6" x14ac:dyDescent="0.35">
@@ -2960,19 +2988,16 @@
         <v>32</v>
       </c>
       <c r="B105" t="s">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="C105" t="s">
-        <v>10</v>
-      </c>
-      <c r="D105">
-        <v>1</v>
+        <v>206</v>
       </c>
       <c r="E105" t="s">
-        <v>11</v>
+        <v>103</v>
       </c>
       <c r="F105" t="s">
-        <v>12</v>
+        <v>204</v>
       </c>
     </row>
     <row r="106" spans="1:6" x14ac:dyDescent="0.35">
@@ -2982,17 +3007,14 @@
       <c r="B106" t="s">
         <v>9</v>
       </c>
-      <c r="C106" t="s">
-        <v>16</v>
-      </c>
-      <c r="D106">
-        <v>1</v>
+      <c r="D106" t="s">
+        <v>87</v>
       </c>
       <c r="E106" t="s">
-        <v>40</v>
+        <v>11</v>
       </c>
       <c r="F106" t="s">
-        <v>37</v>
+        <v>12</v>
       </c>
     </row>
     <row r="107" spans="1:6" x14ac:dyDescent="0.35">
@@ -3000,16 +3022,19 @@
         <v>32</v>
       </c>
       <c r="B107" t="s">
-        <v>185</v>
-      </c>
-      <c r="D107" t="s">
-        <v>68</v>
+        <v>9</v>
+      </c>
+      <c r="C107" t="s">
+        <v>10</v>
+      </c>
+      <c r="D107">
+        <v>1</v>
       </c>
       <c r="E107" t="s">
-        <v>105</v>
+        <v>11</v>
       </c>
       <c r="F107" t="s">
-        <v>107</v>
+        <v>12</v>
       </c>
     </row>
     <row r="108" spans="1:6" x14ac:dyDescent="0.35">
@@ -3017,16 +3042,19 @@
         <v>32</v>
       </c>
       <c r="B108" t="s">
-        <v>75</v>
-      </c>
-      <c r="D108" t="s">
-        <v>87</v>
+        <v>9</v>
+      </c>
+      <c r="C108" t="s">
+        <v>16</v>
+      </c>
+      <c r="D108">
+        <v>1</v>
       </c>
       <c r="E108" t="s">
-        <v>11</v>
+        <v>40</v>
       </c>
       <c r="F108" t="s">
-        <v>71</v>
+        <v>37</v>
       </c>
     </row>
     <row r="109" spans="1:6" x14ac:dyDescent="0.35">
@@ -3034,16 +3062,16 @@
         <v>32</v>
       </c>
       <c r="B109" t="s">
-        <v>75</v>
-      </c>
-      <c r="C109" t="s">
-        <v>74</v>
+        <v>185</v>
+      </c>
+      <c r="D109" t="s">
+        <v>68</v>
       </c>
       <c r="E109" t="s">
-        <v>11</v>
+        <v>105</v>
       </c>
       <c r="F109" t="s">
-        <v>71</v>
+        <v>107</v>
       </c>
     </row>
     <row r="110" spans="1:6" x14ac:dyDescent="0.35">
@@ -3051,7 +3079,7 @@
         <v>32</v>
       </c>
       <c r="B110" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="D110" t="s">
         <v>87</v>
@@ -3068,13 +3096,10 @@
         <v>32</v>
       </c>
       <c r="B111" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="C111" t="s">
-        <v>70</v>
-      </c>
-      <c r="D111">
-        <v>2</v>
+        <v>74</v>
       </c>
       <c r="E111" t="s">
         <v>11</v>
@@ -3088,16 +3113,16 @@
         <v>32</v>
       </c>
       <c r="B112" t="s">
-        <v>186</v>
+        <v>72</v>
       </c>
       <c r="D112" t="s">
-        <v>65</v>
+        <v>87</v>
       </c>
       <c r="E112" t="s">
-        <v>85</v>
+        <v>11</v>
       </c>
       <c r="F112" t="s">
-        <v>79</v>
+        <v>71</v>
       </c>
     </row>
     <row r="113" spans="1:6" x14ac:dyDescent="0.35">
@@ -3105,10 +3130,13 @@
         <v>32</v>
       </c>
       <c r="B113" t="s">
-        <v>73</v>
-      </c>
-      <c r="D113" t="s">
-        <v>87</v>
+        <v>72</v>
+      </c>
+      <c r="C113" t="s">
+        <v>70</v>
+      </c>
+      <c r="D113">
+        <v>2</v>
       </c>
       <c r="E113" t="s">
         <v>11</v>
@@ -3122,16 +3150,16 @@
         <v>32</v>
       </c>
       <c r="B114" t="s">
-        <v>73</v>
-      </c>
-      <c r="C114" t="s">
-        <v>74</v>
+        <v>186</v>
+      </c>
+      <c r="D114" t="s">
+        <v>65</v>
       </c>
       <c r="E114" t="s">
-        <v>11</v>
+        <v>85</v>
       </c>
       <c r="F114" t="s">
-        <v>71</v>
+        <v>79</v>
       </c>
     </row>
     <row r="115" spans="1:6" x14ac:dyDescent="0.35">
@@ -3139,7 +3167,7 @@
         <v>32</v>
       </c>
       <c r="B115" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="D115" t="s">
         <v>87</v>
@@ -3156,13 +3184,10 @@
         <v>32</v>
       </c>
       <c r="B116" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="C116" t="s">
-        <v>70</v>
-      </c>
-      <c r="D116">
-        <v>2</v>
+        <v>74</v>
       </c>
       <c r="E116" t="s">
         <v>11</v>
@@ -3176,16 +3201,16 @@
         <v>32</v>
       </c>
       <c r="B117" t="s">
-        <v>92</v>
+        <v>69</v>
       </c>
       <c r="D117" t="s">
         <v>87</v>
       </c>
       <c r="E117" t="s">
-        <v>53</v>
+        <v>11</v>
       </c>
       <c r="F117" t="s">
-        <v>47</v>
+        <v>71</v>
       </c>
     </row>
     <row r="118" spans="1:6" x14ac:dyDescent="0.35">
@@ -3193,16 +3218,19 @@
         <v>32</v>
       </c>
       <c r="B118" t="s">
-        <v>162</v>
-      </c>
-      <c r="D118" t="s">
-        <v>87</v>
+        <v>69</v>
+      </c>
+      <c r="C118" t="s">
+        <v>70</v>
+      </c>
+      <c r="D118">
+        <v>2</v>
       </c>
       <c r="E118" t="s">
-        <v>116</v>
+        <v>11</v>
       </c>
       <c r="F118" t="s">
-        <v>163</v>
+        <v>71</v>
       </c>
     </row>
     <row r="119" spans="1:6" x14ac:dyDescent="0.35">
@@ -3210,19 +3238,16 @@
         <v>32</v>
       </c>
       <c r="B119" t="s">
-        <v>162</v>
-      </c>
-      <c r="C119" t="s">
-        <v>164</v>
-      </c>
-      <c r="D119">
-        <v>1</v>
+        <v>92</v>
+      </c>
+      <c r="D119" t="s">
+        <v>87</v>
       </c>
       <c r="E119" t="s">
-        <v>116</v>
+        <v>53</v>
       </c>
       <c r="F119" t="s">
-        <v>163</v>
+        <v>47</v>
       </c>
     </row>
     <row r="120" spans="1:6" x14ac:dyDescent="0.35">
@@ -3230,16 +3255,19 @@
         <v>32</v>
       </c>
       <c r="B120" t="s">
-        <v>118</v>
-      </c>
-      <c r="D120" t="s">
-        <v>68</v>
-      </c>
-      <c r="E120" t="s">
-        <v>116</v>
-      </c>
-      <c r="F120" t="s">
-        <v>119</v>
+        <v>92</v>
+      </c>
+      <c r="C120" s="2" t="s">
+        <v>220</v>
+      </c>
+      <c r="D120">
+        <v>1</v>
+      </c>
+      <c r="E120" s="2" t="s">
+        <v>219</v>
+      </c>
+      <c r="F120" s="2" t="s">
+        <v>218</v>
       </c>
     </row>
     <row r="121" spans="1:6" x14ac:dyDescent="0.35">
@@ -3247,16 +3275,16 @@
         <v>32</v>
       </c>
       <c r="B121" t="s">
-        <v>118</v>
-      </c>
-      <c r="C121" t="s">
-        <v>124</v>
+        <v>162</v>
+      </c>
+      <c r="D121" t="s">
+        <v>87</v>
       </c>
       <c r="E121" t="s">
         <v>116</v>
       </c>
       <c r="F121" t="s">
-        <v>121</v>
+        <v>163</v>
       </c>
     </row>
     <row r="122" spans="1:6" x14ac:dyDescent="0.35">
@@ -3264,16 +3292,19 @@
         <v>32</v>
       </c>
       <c r="B122" t="s">
-        <v>118</v>
+        <v>162</v>
       </c>
       <c r="C122" t="s">
-        <v>52</v>
+        <v>164</v>
+      </c>
+      <c r="D122">
+        <v>1</v>
       </c>
       <c r="E122" t="s">
         <v>116</v>
       </c>
       <c r="F122" t="s">
-        <v>119</v>
+        <v>163</v>
       </c>
     </row>
     <row r="123" spans="1:6" x14ac:dyDescent="0.35">
@@ -3283,14 +3314,14 @@
       <c r="B123" t="s">
         <v>118</v>
       </c>
-      <c r="C123" t="s">
-        <v>129</v>
+      <c r="D123" t="s">
+        <v>68</v>
       </c>
       <c r="E123" t="s">
         <v>116</v>
       </c>
       <c r="F123" t="s">
-        <v>130</v>
+        <v>119</v>
       </c>
     </row>
     <row r="124" spans="1:6" x14ac:dyDescent="0.35">
@@ -3301,7 +3332,7 @@
         <v>118</v>
       </c>
       <c r="C124" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="E124" t="s">
         <v>116</v>
@@ -3318,13 +3349,13 @@
         <v>118</v>
       </c>
       <c r="C125" t="s">
-        <v>136</v>
+        <v>52</v>
       </c>
       <c r="E125" t="s">
         <v>116</v>
       </c>
       <c r="F125" t="s">
-        <v>137</v>
+        <v>119</v>
       </c>
     </row>
     <row r="126" spans="1:6" x14ac:dyDescent="0.35">
@@ -3335,13 +3366,13 @@
         <v>118</v>
       </c>
       <c r="C126" t="s">
-        <v>146</v>
+        <v>129</v>
       </c>
       <c r="E126" t="s">
         <v>116</v>
       </c>
       <c r="F126" t="s">
-        <v>147</v>
+        <v>130</v>
       </c>
     </row>
     <row r="127" spans="1:6" x14ac:dyDescent="0.35">
@@ -3352,13 +3383,13 @@
         <v>118</v>
       </c>
       <c r="C127" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="E127" t="s">
         <v>116</v>
       </c>
       <c r="F127" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="128" spans="1:6" x14ac:dyDescent="0.35">
@@ -3369,13 +3400,13 @@
         <v>118</v>
       </c>
       <c r="C128" t="s">
-        <v>51</v>
+        <v>136</v>
       </c>
       <c r="E128" t="s">
         <v>116</v>
       </c>
       <c r="F128" t="s">
-        <v>119</v>
+        <v>137</v>
       </c>
     </row>
     <row r="129" spans="1:6" x14ac:dyDescent="0.35">
@@ -3383,16 +3414,16 @@
         <v>32</v>
       </c>
       <c r="B129" t="s">
-        <v>165</v>
-      </c>
-      <c r="D129" t="s">
-        <v>87</v>
+        <v>118</v>
+      </c>
+      <c r="C129" t="s">
+        <v>146</v>
       </c>
       <c r="E129" t="s">
         <v>116</v>
       </c>
       <c r="F129" t="s">
-        <v>163</v>
+        <v>147</v>
       </c>
     </row>
     <row r="130" spans="1:6" x14ac:dyDescent="0.35">
@@ -3400,16 +3431,16 @@
         <v>32</v>
       </c>
       <c r="B130" t="s">
-        <v>165</v>
+        <v>118</v>
       </c>
       <c r="C130" t="s">
-        <v>166</v>
+        <v>120</v>
       </c>
       <c r="E130" t="s">
         <v>116</v>
       </c>
       <c r="F130" t="s">
-        <v>163</v>
+        <v>122</v>
       </c>
     </row>
     <row r="131" spans="1:6" x14ac:dyDescent="0.35">
@@ -3417,16 +3448,16 @@
         <v>32</v>
       </c>
       <c r="B131" t="s">
-        <v>149</v>
-      </c>
-      <c r="D131" t="s">
-        <v>68</v>
+        <v>118</v>
+      </c>
+      <c r="C131" t="s">
+        <v>51</v>
       </c>
       <c r="E131" t="s">
         <v>116</v>
       </c>
       <c r="F131" t="s">
-        <v>147</v>
+        <v>119</v>
       </c>
     </row>
     <row r="132" spans="1:6" x14ac:dyDescent="0.35">
@@ -3434,16 +3465,16 @@
         <v>32</v>
       </c>
       <c r="B132" t="s">
-        <v>149</v>
-      </c>
-      <c r="C132" t="s">
-        <v>151</v>
+        <v>165</v>
+      </c>
+      <c r="D132" t="s">
+        <v>87</v>
       </c>
       <c r="E132" t="s">
         <v>116</v>
       </c>
       <c r="F132" t="s">
-        <v>147</v>
+        <v>163</v>
       </c>
     </row>
     <row r="133" spans="1:6" x14ac:dyDescent="0.35">
@@ -3451,16 +3482,16 @@
         <v>32</v>
       </c>
       <c r="B133" t="s">
-        <v>149</v>
+        <v>165</v>
       </c>
       <c r="C133" t="s">
-        <v>49</v>
+        <v>166</v>
       </c>
       <c r="E133" t="s">
         <v>116</v>
       </c>
       <c r="F133" t="s">
-        <v>147</v>
+        <v>163</v>
       </c>
     </row>
     <row r="134" spans="1:6" x14ac:dyDescent="0.35">
@@ -3470,8 +3501,8 @@
       <c r="B134" t="s">
         <v>149</v>
       </c>
-      <c r="C134" t="s">
-        <v>150</v>
+      <c r="D134" t="s">
+        <v>68</v>
       </c>
       <c r="E134" t="s">
         <v>116</v>
@@ -3488,7 +3519,7 @@
         <v>149</v>
       </c>
       <c r="C135" t="s">
-        <v>50</v>
+        <v>151</v>
       </c>
       <c r="E135" t="s">
         <v>116</v>
@@ -3502,16 +3533,16 @@
         <v>32</v>
       </c>
       <c r="B136" t="s">
-        <v>138</v>
-      </c>
-      <c r="D136" t="s">
-        <v>68</v>
+        <v>149</v>
+      </c>
+      <c r="C136" t="s">
+        <v>49</v>
       </c>
       <c r="E136" t="s">
         <v>116</v>
       </c>
       <c r="F136" t="s">
-        <v>137</v>
+        <v>147</v>
       </c>
     </row>
     <row r="137" spans="1:6" x14ac:dyDescent="0.35">
@@ -3519,10 +3550,10 @@
         <v>32</v>
       </c>
       <c r="B137" t="s">
-        <v>138</v>
+        <v>149</v>
       </c>
       <c r="C137" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="E137" t="s">
         <v>116</v>
@@ -3536,16 +3567,16 @@
         <v>32</v>
       </c>
       <c r="B138" t="s">
-        <v>138</v>
+        <v>149</v>
       </c>
       <c r="C138" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="E138" t="s">
         <v>116</v>
       </c>
       <c r="F138" t="s">
-        <v>137</v>
+        <v>147</v>
       </c>
     </row>
     <row r="139" spans="1:6" x14ac:dyDescent="0.35">
@@ -3555,8 +3586,8 @@
       <c r="B139" t="s">
         <v>138</v>
       </c>
-      <c r="C139" t="s">
-        <v>57</v>
+      <c r="D139" t="s">
+        <v>68</v>
       </c>
       <c r="E139" t="s">
         <v>116</v>
@@ -3573,13 +3604,13 @@
         <v>138</v>
       </c>
       <c r="C140" t="s">
-        <v>156</v>
+        <v>148</v>
       </c>
       <c r="E140" t="s">
         <v>116</v>
       </c>
       <c r="F140" t="s">
-        <v>158</v>
+        <v>147</v>
       </c>
     </row>
     <row r="141" spans="1:6" x14ac:dyDescent="0.35">
@@ -3590,13 +3621,13 @@
         <v>138</v>
       </c>
       <c r="C141" t="s">
-        <v>154</v>
+        <v>58</v>
       </c>
       <c r="E141" t="s">
         <v>116</v>
       </c>
       <c r="F141" t="s">
-        <v>155</v>
+        <v>137</v>
       </c>
     </row>
     <row r="142" spans="1:6" x14ac:dyDescent="0.35">
@@ -3607,13 +3638,13 @@
         <v>138</v>
       </c>
       <c r="C142" t="s">
-        <v>184</v>
+        <v>57</v>
       </c>
       <c r="E142" t="s">
         <v>116</v>
       </c>
       <c r="F142" t="s">
-        <v>183</v>
+        <v>137</v>
       </c>
     </row>
     <row r="143" spans="1:6" x14ac:dyDescent="0.35">
@@ -3624,7 +3655,7 @@
         <v>138</v>
       </c>
       <c r="C143" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="E143" t="s">
         <v>116</v>
@@ -3638,16 +3669,16 @@
         <v>32</v>
       </c>
       <c r="B144" t="s">
-        <v>125</v>
-      </c>
-      <c r="D144" t="s">
-        <v>68</v>
+        <v>138</v>
+      </c>
+      <c r="C144" t="s">
+        <v>154</v>
       </c>
       <c r="E144" t="s">
         <v>116</v>
       </c>
       <c r="F144" t="s">
-        <v>121</v>
+        <v>155</v>
       </c>
     </row>
     <row r="145" spans="1:6" x14ac:dyDescent="0.35">
@@ -3655,16 +3686,16 @@
         <v>32</v>
       </c>
       <c r="B145" t="s">
-        <v>125</v>
+        <v>138</v>
       </c>
       <c r="C145" t="s">
-        <v>127</v>
+        <v>184</v>
       </c>
       <c r="E145" t="s">
         <v>116</v>
       </c>
       <c r="F145" t="s">
-        <v>121</v>
+        <v>183</v>
       </c>
     </row>
     <row r="146" spans="1:6" x14ac:dyDescent="0.35">
@@ -3672,16 +3703,16 @@
         <v>32</v>
       </c>
       <c r="B146" t="s">
-        <v>131</v>
-      </c>
-      <c r="D146" t="s">
-        <v>68</v>
+        <v>138</v>
+      </c>
+      <c r="C146" t="s">
+        <v>157</v>
       </c>
       <c r="E146" t="s">
         <v>116</v>
       </c>
       <c r="F146" t="s">
-        <v>130</v>
+        <v>158</v>
       </c>
     </row>
     <row r="147" spans="1:6" x14ac:dyDescent="0.35">
@@ -3689,16 +3720,16 @@
         <v>32</v>
       </c>
       <c r="B147" t="s">
-        <v>131</v>
-      </c>
-      <c r="C147" t="s">
-        <v>132</v>
+        <v>125</v>
+      </c>
+      <c r="D147" t="s">
+        <v>68</v>
       </c>
       <c r="E147" t="s">
         <v>116</v>
       </c>
       <c r="F147" t="s">
-        <v>130</v>
+        <v>121</v>
       </c>
     </row>
     <row r="148" spans="1:6" x14ac:dyDescent="0.35">
@@ -3706,16 +3737,16 @@
         <v>32</v>
       </c>
       <c r="B148" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
       <c r="C148" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="E148" t="s">
         <v>116</v>
       </c>
       <c r="F148" t="s">
-        <v>130</v>
+        <v>121</v>
       </c>
     </row>
     <row r="149" spans="1:6" x14ac:dyDescent="0.35">
@@ -3725,8 +3756,8 @@
       <c r="B149" t="s">
         <v>131</v>
       </c>
-      <c r="C149" t="s">
-        <v>134</v>
+      <c r="D149" t="s">
+        <v>68</v>
       </c>
       <c r="E149" t="s">
         <v>116</v>
@@ -3743,7 +3774,7 @@
         <v>131</v>
       </c>
       <c r="C150" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="E150" t="s">
         <v>116</v>
@@ -3757,16 +3788,16 @@
         <v>32</v>
       </c>
       <c r="B151" t="s">
-        <v>126</v>
-      </c>
-      <c r="D151" t="s">
-        <v>68</v>
+        <v>131</v>
+      </c>
+      <c r="C151" t="s">
+        <v>133</v>
       </c>
       <c r="E151" t="s">
         <v>116</v>
       </c>
       <c r="F151" t="s">
-        <v>121</v>
+        <v>130</v>
       </c>
     </row>
     <row r="152" spans="1:6" x14ac:dyDescent="0.35">
@@ -3774,16 +3805,16 @@
         <v>32</v>
       </c>
       <c r="B152" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="C152" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="E152" t="s">
         <v>116</v>
       </c>
       <c r="F152" t="s">
-        <v>121</v>
+        <v>130</v>
       </c>
     </row>
     <row r="153" spans="1:6" x14ac:dyDescent="0.35">
@@ -3791,16 +3822,16 @@
         <v>32</v>
       </c>
       <c r="B153" t="s">
-        <v>98</v>
-      </c>
-      <c r="D153" t="s">
-        <v>87</v>
+        <v>131</v>
+      </c>
+      <c r="C153" t="s">
+        <v>135</v>
       </c>
       <c r="E153" t="s">
-        <v>14</v>
+        <v>116</v>
       </c>
       <c r="F153" t="s">
-        <v>99</v>
+        <v>130</v>
       </c>
     </row>
     <row r="154" spans="1:6" x14ac:dyDescent="0.35">
@@ -3808,16 +3839,16 @@
         <v>32</v>
       </c>
       <c r="B154" t="s">
-        <v>13</v>
+        <v>126</v>
       </c>
       <c r="D154" t="s">
-        <v>87</v>
+        <v>68</v>
       </c>
       <c r="E154" t="s">
-        <v>14</v>
+        <v>116</v>
       </c>
       <c r="F154" t="s">
-        <v>17</v>
+        <v>121</v>
       </c>
     </row>
     <row r="155" spans="1:6" x14ac:dyDescent="0.35">
@@ -3825,19 +3856,16 @@
         <v>32</v>
       </c>
       <c r="B155" t="s">
-        <v>13</v>
+        <v>126</v>
       </c>
       <c r="C155" t="s">
-        <v>10</v>
-      </c>
-      <c r="D155">
-        <v>1</v>
+        <v>128</v>
       </c>
       <c r="E155" t="s">
-        <v>14</v>
+        <v>116</v>
       </c>
       <c r="F155" t="s">
-        <v>15</v>
+        <v>121</v>
       </c>
     </row>
     <row r="156" spans="1:6" x14ac:dyDescent="0.35">
@@ -3845,19 +3873,16 @@
         <v>32</v>
       </c>
       <c r="B156" t="s">
-        <v>13</v>
-      </c>
-      <c r="C156" t="s">
-        <v>20</v>
-      </c>
-      <c r="D156">
-        <v>1</v>
+        <v>98</v>
+      </c>
+      <c r="D156" t="s">
+        <v>87</v>
       </c>
       <c r="E156" t="s">
         <v>14</v>
       </c>
       <c r="F156" t="s">
-        <v>23</v>
+        <v>99</v>
       </c>
     </row>
     <row r="157" spans="1:6" x14ac:dyDescent="0.35">
@@ -3867,11 +3892,8 @@
       <c r="B157" t="s">
         <v>13</v>
       </c>
-      <c r="C157" t="s">
-        <v>18</v>
-      </c>
-      <c r="D157">
-        <v>1</v>
+      <c r="D157" t="s">
+        <v>87</v>
       </c>
       <c r="E157" t="s">
         <v>14</v>
@@ -3885,16 +3907,19 @@
         <v>32</v>
       </c>
       <c r="B158" t="s">
-        <v>97</v>
-      </c>
-      <c r="D158" t="s">
-        <v>87</v>
+        <v>13</v>
+      </c>
+      <c r="C158" t="s">
+        <v>10</v>
+      </c>
+      <c r="D158">
+        <v>1</v>
       </c>
       <c r="E158" t="s">
-        <v>54</v>
+        <v>14</v>
       </c>
       <c r="F158" t="s">
-        <v>63</v>
+        <v>15</v>
       </c>
     </row>
     <row r="159" spans="1:6" x14ac:dyDescent="0.35">
@@ -3902,16 +3927,19 @@
         <v>32</v>
       </c>
       <c r="B159" t="s">
-        <v>97</v>
+        <v>13</v>
       </c>
       <c r="C159" t="s">
-        <v>191</v>
+        <v>20</v>
+      </c>
+      <c r="D159">
+        <v>1</v>
       </c>
       <c r="E159" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F159" t="s">
-        <v>89</v>
+        <v>23</v>
       </c>
     </row>
     <row r="160" spans="1:6" x14ac:dyDescent="0.35">
@@ -3919,16 +3947,19 @@
         <v>32</v>
       </c>
       <c r="B160" t="s">
-        <v>33</v>
-      </c>
-      <c r="D160" t="s">
-        <v>87</v>
+        <v>13</v>
+      </c>
+      <c r="C160" t="s">
+        <v>18</v>
+      </c>
+      <c r="D160">
+        <v>1</v>
       </c>
       <c r="E160" t="s">
-        <v>54</v>
+        <v>14</v>
       </c>
       <c r="F160" t="s">
-        <v>56</v>
+        <v>17</v>
       </c>
     </row>
     <row r="161" spans="1:6" x14ac:dyDescent="0.35">
@@ -3936,13 +3967,10 @@
         <v>32</v>
       </c>
       <c r="B161" t="s">
-        <v>33</v>
-      </c>
-      <c r="C161" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="D161">
-        <v>1</v>
+        <v>97</v>
+      </c>
+      <c r="D161" t="s">
+        <v>87</v>
       </c>
       <c r="E161" t="s">
         <v>54</v>
@@ -3956,10 +3984,10 @@
         <v>32</v>
       </c>
       <c r="B162" t="s">
-        <v>33</v>
-      </c>
-      <c r="C162" s="1" t="s">
-        <v>39</v>
+        <v>97</v>
+      </c>
+      <c r="C162" s="2" t="s">
+        <v>216</v>
       </c>
       <c r="D162">
         <v>1</v>
@@ -3967,8 +3995,8 @@
       <c r="E162" t="s">
         <v>54</v>
       </c>
-      <c r="F162" t="s">
-        <v>55</v>
+      <c r="F162" s="2" t="s">
+        <v>193</v>
       </c>
     </row>
     <row r="163" spans="1:6" x14ac:dyDescent="0.35">
@@ -3976,16 +4004,16 @@
         <v>32</v>
       </c>
       <c r="B163" t="s">
-        <v>33</v>
-      </c>
-      <c r="C163" s="1" t="s">
-        <v>57</v>
+        <v>97</v>
+      </c>
+      <c r="C163" t="s">
+        <v>191</v>
       </c>
       <c r="E163" t="s">
-        <v>54</v>
+        <v>24</v>
       </c>
       <c r="F163" t="s">
-        <v>56</v>
+        <v>89</v>
       </c>
     </row>
     <row r="164" spans="1:6" x14ac:dyDescent="0.35">
@@ -3995,14 +4023,14 @@
       <c r="B164" t="s">
         <v>33</v>
       </c>
-      <c r="C164" s="1" t="s">
-        <v>195</v>
+      <c r="D164" t="s">
+        <v>87</v>
       </c>
       <c r="E164" t="s">
         <v>54</v>
       </c>
       <c r="F164" t="s">
-        <v>193</v>
+        <v>56</v>
       </c>
     </row>
     <row r="165" spans="1:6" x14ac:dyDescent="0.35">
@@ -4010,17 +4038,19 @@
         <v>32</v>
       </c>
       <c r="B165" t="s">
-        <v>182</v>
-      </c>
-      <c r="C165" s="1"/>
-      <c r="D165" t="s">
-        <v>68</v>
+        <v>33</v>
+      </c>
+      <c r="C165" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="D165">
+        <v>1</v>
       </c>
       <c r="E165" t="s">
-        <v>116</v>
+        <v>54</v>
       </c>
       <c r="F165" t="s">
-        <v>183</v>
+        <v>193</v>
       </c>
     </row>
     <row r="166" spans="1:6" x14ac:dyDescent="0.35">
@@ -4028,15 +4058,107 @@
         <v>32</v>
       </c>
       <c r="B166" t="s">
+        <v>33</v>
+      </c>
+      <c r="C166" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D166">
+        <v>1</v>
+      </c>
+      <c r="E166" t="s">
+        <v>54</v>
+      </c>
+      <c r="F166" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="167" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A167" t="s">
+        <v>32</v>
+      </c>
+      <c r="B167" t="s">
+        <v>33</v>
+      </c>
+      <c r="C167" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D167">
+        <v>1</v>
+      </c>
+      <c r="E167" t="s">
+        <v>54</v>
+      </c>
+      <c r="F167" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="168" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A168" t="s">
+        <v>32</v>
+      </c>
+      <c r="B168" t="s">
+        <v>33</v>
+      </c>
+      <c r="C168" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="E168" t="s">
+        <v>54</v>
+      </c>
+      <c r="F168" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="169" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A169" t="s">
+        <v>32</v>
+      </c>
+      <c r="B169" t="s">
+        <v>33</v>
+      </c>
+      <c r="C169" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="E169" t="s">
+        <v>54</v>
+      </c>
+      <c r="F169" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="170" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A170" t="s">
+        <v>32</v>
+      </c>
+      <c r="B170" t="s">
+        <v>182</v>
+      </c>
+      <c r="C170" s="1"/>
+      <c r="D170" t="s">
+        <v>68</v>
+      </c>
+      <c r="E170" t="s">
+        <v>116</v>
+      </c>
+      <c r="F170" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="171" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A171" t="s">
+        <v>32</v>
+      </c>
+      <c r="B171" t="s">
         <v>88</v>
       </c>
-      <c r="D166" t="s">
+      <c r="D171" t="s">
         <v>65</v>
       </c>
-      <c r="E166" t="s">
+      <c r="E171" t="s">
         <v>24</v>
       </c>
-      <c r="F166" t="s">
+      <c r="F171" t="s">
         <v>89</v>
       </c>
     </row>

</xml_diff>

<commit_message>
[PowerPoint] Added snippets that act on selections (#1069)
* [PowerPoint] Added snippets that acts on selections

* Apply suggestions from code review

Co-authored-by: Alex Jerabek <38896772+AlexJerabek@users.noreply.github.com>

* Updates based on feedback

* Tweak setup

* Update other affected setup functions

* Apply suggestions from code review

Co-authored-by: Alex Jerabek <38896772+AlexJerabek@users.noreply.github.com>

* Updates based on feedback

---------

Co-authored-by: Alex Jerabek <38896772+AlexJerabek@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/snippet-extractor-metadata/powerpoint.xlsx
+++ b/snippet-extractor-metadata/powerpoint.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7C414EC-35C0-4625-9957-123F9D615DF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A2CA723-45CB-4135-8A1A-0329A73196F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25180" windowHeight="16140" xr2:uid="{CB5595D7-4492-4192-A1C1-2583BA1957AA}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="831" uniqueCount="215">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="856" uniqueCount="223">
   <si>
     <t>Class</t>
   </si>
@@ -665,6 +665,30 @@
   </si>
   <si>
     <t>ShapeGetImageFormatType</t>
+  </si>
+  <si>
+    <t>getParentTextFrame</t>
+  </si>
+  <si>
+    <t>getParentShape</t>
+  </si>
+  <si>
+    <t>getParentSlide</t>
+  </si>
+  <si>
+    <t>getSlideById</t>
+  </si>
+  <si>
+    <t>powerpoint-slide-management-get-slide-by-id</t>
+  </si>
+  <si>
+    <t>getItemOrNullObject</t>
+  </si>
+  <si>
+    <t>powerpoint-shapes-get-shape-by-id</t>
+  </si>
+  <si>
+    <t>getShapeById</t>
   </si>
 </sst>
 </file>
@@ -745,10 +769,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{78C585A5-D505-49C6-9CA1-8E6558948317}" name="Snippets" displayName="Snippets" ref="A1:F166" totalsRowShown="0" headerRowDxfId="4">
-  <autoFilter ref="A1:F166" xr:uid="{EAC65D03-FDD2-4352-A5F3-1CDEDE6251B2}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F162">
-    <sortCondition ref="B1:B162"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{78C585A5-D505-49C6-9CA1-8E6558948317}" name="Snippets" displayName="Snippets" ref="A1:F171" totalsRowShown="0" headerRowDxfId="4">
+  <autoFilter ref="A1:F171" xr:uid="{EAC65D03-FDD2-4352-A5F3-1CDEDE6251B2}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F167">
+    <sortCondition ref="B1:B167"/>
   </sortState>
   <tableColumns count="6">
     <tableColumn id="6" xr3:uid="{408888B8-C1DD-4B51-B1EB-5663F091D142}" name="Package"/>
@@ -1059,7 +1083,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{809930CD-A227-47DC-AAA4-BB816AEDEB59}">
-  <dimension ref="A1:F166"/>
+  <dimension ref="A1:F171"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="11.453125" bestFit="1" customWidth="1"/>
@@ -1962,16 +1986,16 @@
       <c r="B50" t="s">
         <v>45</v>
       </c>
-      <c r="C50" s="2" t="s">
+      <c r="C50" t="s">
         <v>106</v>
       </c>
       <c r="D50">
         <v>1</v>
       </c>
-      <c r="E50" s="2" t="s">
+      <c r="E50" t="s">
         <v>211</v>
       </c>
-      <c r="F50" s="2" t="s">
+      <c r="F50" t="s">
         <v>213</v>
       </c>
     </row>
@@ -1982,17 +2006,17 @@
       <c r="B51" t="s">
         <v>45</v>
       </c>
-      <c r="C51" t="s">
-        <v>161</v>
+      <c r="C51" s="2" t="s">
+        <v>217</v>
       </c>
       <c r="D51">
         <v>1</v>
       </c>
-      <c r="E51" t="s">
-        <v>116</v>
-      </c>
-      <c r="F51" t="s">
-        <v>160</v>
+      <c r="E51" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="F51" s="2" t="s">
+        <v>193</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.35">
@@ -2003,16 +2027,16 @@
         <v>45</v>
       </c>
       <c r="C52" t="s">
-        <v>208</v>
+        <v>161</v>
       </c>
       <c r="D52">
         <v>1</v>
       </c>
       <c r="E52" t="s">
-        <v>103</v>
+        <v>116</v>
       </c>
       <c r="F52" t="s">
-        <v>209</v>
+        <v>160</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.35">
@@ -2023,16 +2047,16 @@
         <v>45</v>
       </c>
       <c r="C53" t="s">
-        <v>176</v>
+        <v>208</v>
       </c>
       <c r="D53">
         <v>1</v>
       </c>
       <c r="E53" t="s">
-        <v>168</v>
+        <v>103</v>
       </c>
       <c r="F53" t="s">
-        <v>177</v>
+        <v>209</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.35">
@@ -2043,13 +2067,16 @@
         <v>45</v>
       </c>
       <c r="C54" t="s">
-        <v>58</v>
+        <v>176</v>
+      </c>
+      <c r="D54">
+        <v>1</v>
       </c>
       <c r="E54" t="s">
-        <v>53</v>
+        <v>168</v>
       </c>
       <c r="F54" t="s">
-        <v>44</v>
+        <v>177</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.35">
@@ -2060,13 +2087,13 @@
         <v>45</v>
       </c>
       <c r="C55" t="s">
-        <v>108</v>
+        <v>58</v>
       </c>
       <c r="E55" t="s">
-        <v>109</v>
+        <v>53</v>
       </c>
       <c r="F55" t="s">
-        <v>110</v>
+        <v>44</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.35">
@@ -2077,13 +2104,13 @@
         <v>45</v>
       </c>
       <c r="C56" t="s">
-        <v>52</v>
+        <v>108</v>
       </c>
       <c r="E56" t="s">
-        <v>53</v>
+        <v>109</v>
       </c>
       <c r="F56" t="s">
-        <v>48</v>
+        <v>110</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.35">
@@ -2094,7 +2121,7 @@
         <v>45</v>
       </c>
       <c r="C57" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="E57" t="s">
         <v>53</v>
@@ -2111,13 +2138,13 @@
         <v>45</v>
       </c>
       <c r="C58" t="s">
-        <v>196</v>
+        <v>49</v>
       </c>
       <c r="E58" t="s">
-        <v>85</v>
+        <v>53</v>
       </c>
       <c r="F58" t="s">
-        <v>197</v>
+        <v>48</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.35">
@@ -2128,13 +2155,13 @@
         <v>45</v>
       </c>
       <c r="C59" t="s">
-        <v>50</v>
+        <v>196</v>
       </c>
       <c r="E59" t="s">
-        <v>53</v>
+        <v>85</v>
       </c>
       <c r="F59" t="s">
-        <v>48</v>
+        <v>197</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.35">
@@ -2145,13 +2172,13 @@
         <v>45</v>
       </c>
       <c r="C60" t="s">
-        <v>86</v>
+        <v>50</v>
       </c>
       <c r="E60" t="s">
-        <v>85</v>
+        <v>53</v>
       </c>
       <c r="F60" t="s">
-        <v>81</v>
+        <v>48</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.35">
@@ -2162,13 +2189,13 @@
         <v>45</v>
       </c>
       <c r="C61" t="s">
-        <v>51</v>
+        <v>86</v>
       </c>
       <c r="E61" t="s">
-        <v>53</v>
+        <v>85</v>
       </c>
       <c r="F61" t="s">
-        <v>48</v>
+        <v>81</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.35">
@@ -2179,13 +2206,13 @@
         <v>45</v>
       </c>
       <c r="C62" t="s">
-        <v>178</v>
+        <v>51</v>
       </c>
       <c r="E62" t="s">
-        <v>168</v>
+        <v>53</v>
       </c>
       <c r="F62" t="s">
-        <v>177</v>
+        <v>48</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.35">
@@ -2193,16 +2220,16 @@
         <v>32</v>
       </c>
       <c r="B63" t="s">
-        <v>95</v>
-      </c>
-      <c r="D63" t="s">
-        <v>68</v>
+        <v>45</v>
+      </c>
+      <c r="C63" t="s">
+        <v>178</v>
       </c>
       <c r="E63" t="s">
-        <v>24</v>
+        <v>168</v>
       </c>
       <c r="F63" t="s">
-        <v>26</v>
+        <v>177</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.35">
@@ -2210,16 +2237,16 @@
         <v>32</v>
       </c>
       <c r="B64" t="s">
-        <v>187</v>
+        <v>95</v>
       </c>
       <c r="D64" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="E64" t="s">
         <v>24</v>
       </c>
       <c r="F64" t="s">
-        <v>89</v>
+        <v>26</v>
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.35">
@@ -2227,16 +2254,16 @@
         <v>32</v>
       </c>
       <c r="B65" t="s">
-        <v>21</v>
+        <v>187</v>
       </c>
       <c r="D65" t="s">
-        <v>87</v>
+        <v>65</v>
       </c>
       <c r="E65" t="s">
-        <v>85</v>
+        <v>24</v>
       </c>
       <c r="F65" t="s">
-        <v>81</v>
+        <v>89</v>
       </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.35">
@@ -2246,17 +2273,14 @@
       <c r="B66" t="s">
         <v>21</v>
       </c>
-      <c r="C66" t="s">
-        <v>25</v>
-      </c>
-      <c r="D66">
-        <v>1</v>
+      <c r="D66" t="s">
+        <v>87</v>
       </c>
       <c r="E66" t="s">
-        <v>24</v>
+        <v>85</v>
       </c>
       <c r="F66" t="s">
-        <v>26</v>
+        <v>81</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.35">
@@ -2267,16 +2291,16 @@
         <v>21</v>
       </c>
       <c r="C67" t="s">
-        <v>111</v>
+        <v>25</v>
       </c>
       <c r="D67">
         <v>1</v>
       </c>
       <c r="E67" t="s">
-        <v>109</v>
+        <v>24</v>
       </c>
       <c r="F67" t="s">
-        <v>112</v>
+        <v>26</v>
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.35">
@@ -2287,16 +2311,16 @@
         <v>21</v>
       </c>
       <c r="C68" t="s">
-        <v>27</v>
+        <v>111</v>
       </c>
       <c r="D68">
         <v>1</v>
       </c>
       <c r="E68" t="s">
-        <v>24</v>
+        <v>109</v>
       </c>
       <c r="F68" t="s">
-        <v>28</v>
+        <v>112</v>
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.35">
@@ -2307,16 +2331,16 @@
         <v>21</v>
       </c>
       <c r="C69" t="s">
-        <v>115</v>
+        <v>27</v>
       </c>
       <c r="D69">
         <v>1</v>
       </c>
       <c r="E69" t="s">
-        <v>116</v>
+        <v>24</v>
       </c>
       <c r="F69" t="s">
-        <v>117</v>
+        <v>28</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.35">
@@ -2327,16 +2351,16 @@
         <v>21</v>
       </c>
       <c r="C70" t="s">
-        <v>29</v>
+        <v>115</v>
       </c>
       <c r="D70">
         <v>1</v>
       </c>
       <c r="E70" t="s">
-        <v>24</v>
+        <v>116</v>
       </c>
       <c r="F70" t="s">
-        <v>30</v>
+        <v>117</v>
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.35">
@@ -2347,16 +2371,16 @@
         <v>21</v>
       </c>
       <c r="C71" t="s">
-        <v>91</v>
+        <v>29</v>
       </c>
       <c r="D71">
         <v>1</v>
       </c>
       <c r="E71" t="s">
-        <v>116</v>
+        <v>24</v>
       </c>
       <c r="F71" t="s">
-        <v>160</v>
+        <v>30</v>
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.35">
@@ -2367,16 +2391,16 @@
         <v>21</v>
       </c>
       <c r="C72" t="s">
-        <v>16</v>
+        <v>91</v>
       </c>
       <c r="D72">
         <v>1</v>
       </c>
       <c r="E72" t="s">
-        <v>14</v>
+        <v>116</v>
       </c>
       <c r="F72" t="s">
-        <v>22</v>
+        <v>160</v>
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.35">
@@ -2387,16 +2411,16 @@
         <v>21</v>
       </c>
       <c r="C73" t="s">
-        <v>70</v>
+        <v>16</v>
       </c>
       <c r="D73">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E73" t="s">
-        <v>85</v>
+        <v>14</v>
       </c>
       <c r="F73" t="s">
-        <v>81</v>
+        <v>22</v>
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.35">
@@ -2404,10 +2428,13 @@
         <v>32</v>
       </c>
       <c r="B74" t="s">
-        <v>59</v>
-      </c>
-      <c r="D74" t="s">
-        <v>87</v>
+        <v>21</v>
+      </c>
+      <c r="C74" t="s">
+        <v>70</v>
+      </c>
+      <c r="D74">
+        <v>2</v>
       </c>
       <c r="E74" t="s">
         <v>85</v>
@@ -2423,17 +2450,14 @@
       <c r="B75" t="s">
         <v>59</v>
       </c>
-      <c r="C75" t="s">
-        <v>179</v>
-      </c>
-      <c r="D75">
-        <v>1</v>
+      <c r="D75" t="s">
+        <v>87</v>
       </c>
       <c r="E75" t="s">
-        <v>168</v>
+        <v>85</v>
       </c>
       <c r="F75" t="s">
-        <v>173</v>
+        <v>81</v>
       </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.35">
@@ -2444,16 +2468,16 @@
         <v>59</v>
       </c>
       <c r="C76" t="s">
-        <v>60</v>
+        <v>179</v>
       </c>
       <c r="D76">
         <v>1</v>
       </c>
       <c r="E76" t="s">
-        <v>53</v>
+        <v>168</v>
       </c>
       <c r="F76" t="s">
-        <v>44</v>
+        <v>173</v>
       </c>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.35">
@@ -2464,13 +2488,16 @@
         <v>59</v>
       </c>
       <c r="C77" t="s">
-        <v>93</v>
+        <v>60</v>
+      </c>
+      <c r="D77">
+        <v>1</v>
       </c>
       <c r="E77" t="s">
         <v>53</v>
       </c>
       <c r="F77" t="s">
-        <v>94</v>
+        <v>44</v>
       </c>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.35">
@@ -2481,13 +2508,13 @@
         <v>59</v>
       </c>
       <c r="C78" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="E78" t="s">
-        <v>85</v>
+        <v>53</v>
       </c>
       <c r="F78" t="s">
-        <v>81</v>
+        <v>94</v>
       </c>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.35">
@@ -2498,13 +2525,13 @@
         <v>59</v>
       </c>
       <c r="C79" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="E79" t="s">
-        <v>53</v>
+        <v>85</v>
       </c>
       <c r="F79" t="s">
-        <v>44</v>
+        <v>81</v>
       </c>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.35">
@@ -2512,10 +2539,10 @@
         <v>32</v>
       </c>
       <c r="B80" t="s">
-        <v>189</v>
-      </c>
-      <c r="D80" t="s">
-        <v>65</v>
+        <v>59</v>
+      </c>
+      <c r="C80" t="s">
+        <v>86</v>
       </c>
       <c r="E80" t="s">
         <v>53</v>
@@ -2529,16 +2556,16 @@
         <v>32</v>
       </c>
       <c r="B81" t="s">
-        <v>61</v>
+        <v>189</v>
       </c>
       <c r="D81" t="s">
-        <v>87</v>
+        <v>65</v>
       </c>
       <c r="E81" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F81" t="s">
-        <v>193</v>
+        <v>44</v>
       </c>
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.35">
@@ -2548,14 +2575,14 @@
       <c r="B82" t="s">
         <v>61</v>
       </c>
-      <c r="C82" t="s">
-        <v>62</v>
+      <c r="D82" t="s">
+        <v>87</v>
       </c>
       <c r="E82" t="s">
         <v>54</v>
       </c>
       <c r="F82" t="s">
-        <v>56</v>
+        <v>193</v>
       </c>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.35">
@@ -2566,13 +2593,13 @@
         <v>61</v>
       </c>
       <c r="C83" t="s">
-        <v>190</v>
+        <v>62</v>
       </c>
       <c r="E83" t="s">
-        <v>24</v>
+        <v>54</v>
       </c>
       <c r="F83" t="s">
-        <v>89</v>
+        <v>56</v>
       </c>
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.35">
@@ -2580,10 +2607,10 @@
         <v>32</v>
       </c>
       <c r="B84" t="s">
-        <v>188</v>
-      </c>
-      <c r="D84" t="s">
-        <v>65</v>
+        <v>61</v>
+      </c>
+      <c r="C84" t="s">
+        <v>190</v>
       </c>
       <c r="E84" t="s">
         <v>24</v>
@@ -2596,35 +2623,33 @@
       <c r="A85" t="s">
         <v>32</v>
       </c>
-      <c r="B85" s="2" t="s">
-        <v>214</v>
-      </c>
-      <c r="C85" s="2"/>
+      <c r="B85" t="s">
+        <v>188</v>
+      </c>
       <c r="D85" t="s">
         <v>65</v>
       </c>
-      <c r="E85" s="2" t="s">
-        <v>211</v>
-      </c>
-      <c r="F85" s="2" t="s">
-        <v>212</v>
+      <c r="E85" t="s">
+        <v>24</v>
+      </c>
+      <c r="F85" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
         <v>32</v>
       </c>
-      <c r="B86" s="2" t="s">
-        <v>210</v>
-      </c>
-      <c r="C86" s="2"/>
+      <c r="B86" t="s">
+        <v>214</v>
+      </c>
       <c r="D86" t="s">
-        <v>68</v>
-      </c>
-      <c r="E86" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="E86" t="s">
         <v>211</v>
       </c>
-      <c r="F86" s="2" t="s">
+      <c r="F86" t="s">
         <v>212</v>
       </c>
     </row>
@@ -2633,16 +2658,16 @@
         <v>32</v>
       </c>
       <c r="B87" t="s">
-        <v>113</v>
+        <v>210</v>
       </c>
       <c r="D87" t="s">
-        <v>87</v>
+        <v>68</v>
       </c>
       <c r="E87" t="s">
-        <v>109</v>
+        <v>211</v>
       </c>
       <c r="F87" t="s">
-        <v>110</v>
+        <v>212</v>
       </c>
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.35">
@@ -2652,11 +2677,8 @@
       <c r="B88" t="s">
         <v>113</v>
       </c>
-      <c r="C88" t="s">
-        <v>114</v>
-      </c>
-      <c r="D88">
-        <v>1</v>
+      <c r="D88" t="s">
+        <v>87</v>
       </c>
       <c r="E88" t="s">
         <v>109</v>
@@ -2670,16 +2692,19 @@
         <v>32</v>
       </c>
       <c r="B89" t="s">
-        <v>80</v>
-      </c>
-      <c r="D89" t="s">
-        <v>65</v>
+        <v>113</v>
+      </c>
+      <c r="C89" t="s">
+        <v>114</v>
+      </c>
+      <c r="D89">
+        <v>1</v>
       </c>
       <c r="E89" t="s">
-        <v>85</v>
+        <v>109</v>
       </c>
       <c r="F89" t="s">
-        <v>79</v>
+        <v>110</v>
       </c>
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.35">
@@ -2687,10 +2712,10 @@
         <v>32</v>
       </c>
       <c r="B90" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="D90" t="s">
-        <v>87</v>
+        <v>65</v>
       </c>
       <c r="E90" t="s">
         <v>85</v>
@@ -2706,8 +2731,8 @@
       <c r="B91" t="s">
         <v>83</v>
       </c>
-      <c r="C91" t="s">
-        <v>84</v>
+      <c r="D91" t="s">
+        <v>87</v>
       </c>
       <c r="E91" t="s">
         <v>85</v>
@@ -2721,16 +2746,16 @@
         <v>32</v>
       </c>
       <c r="B92" t="s">
-        <v>90</v>
-      </c>
-      <c r="D92" t="s">
-        <v>87</v>
+        <v>83</v>
+      </c>
+      <c r="C92" t="s">
+        <v>84</v>
       </c>
       <c r="E92" t="s">
-        <v>53</v>
+        <v>85</v>
       </c>
       <c r="F92" t="s">
-        <v>44</v>
+        <v>79</v>
       </c>
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.35">
@@ -2740,17 +2765,14 @@
       <c r="B93" t="s">
         <v>90</v>
       </c>
-      <c r="C93" t="s">
-        <v>91</v>
-      </c>
-      <c r="D93">
-        <v>1</v>
+      <c r="D93" t="s">
+        <v>87</v>
       </c>
       <c r="E93" t="s">
         <v>53</v>
       </c>
       <c r="F93" t="s">
-        <v>35</v>
+        <v>44</v>
       </c>
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.35">
@@ -2758,16 +2780,19 @@
         <v>32</v>
       </c>
       <c r="B94" t="s">
-        <v>78</v>
-      </c>
-      <c r="D94" t="s">
-        <v>65</v>
+        <v>90</v>
+      </c>
+      <c r="C94" t="s">
+        <v>91</v>
+      </c>
+      <c r="D94">
+        <v>1</v>
       </c>
       <c r="E94" t="s">
-        <v>85</v>
+        <v>53</v>
       </c>
       <c r="F94" t="s">
-        <v>79</v>
+        <v>35</v>
       </c>
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.35">
@@ -2775,16 +2800,19 @@
         <v>32</v>
       </c>
       <c r="B95" t="s">
-        <v>180</v>
-      </c>
-      <c r="D95" t="s">
-        <v>65</v>
-      </c>
-      <c r="E95" t="s">
-        <v>168</v>
-      </c>
-      <c r="F95" t="s">
-        <v>181</v>
+        <v>90</v>
+      </c>
+      <c r="C95" s="2" t="s">
+        <v>220</v>
+      </c>
+      <c r="D95">
+        <v>1</v>
+      </c>
+      <c r="E95" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="F95" s="2" t="s">
+        <v>222</v>
       </c>
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.35">
@@ -2792,16 +2820,16 @@
         <v>32</v>
       </c>
       <c r="B96" t="s">
-        <v>180</v>
+        <v>78</v>
       </c>
       <c r="D96" t="s">
         <v>65</v>
       </c>
       <c r="E96" t="s">
-        <v>168</v>
+        <v>85</v>
       </c>
       <c r="F96" t="s">
-        <v>177</v>
+        <v>79</v>
       </c>
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.35">
@@ -2809,16 +2837,16 @@
         <v>32</v>
       </c>
       <c r="B97" t="s">
-        <v>19</v>
+        <v>180</v>
       </c>
       <c r="D97" t="s">
-        <v>87</v>
+        <v>65</v>
       </c>
       <c r="E97" t="s">
-        <v>53</v>
+        <v>168</v>
       </c>
       <c r="F97" t="s">
-        <v>46</v>
+        <v>181</v>
       </c>
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.35">
@@ -2826,19 +2854,16 @@
         <v>32</v>
       </c>
       <c r="B98" t="s">
-        <v>19</v>
-      </c>
-      <c r="C98" t="s">
-        <v>20</v>
-      </c>
-      <c r="D98">
-        <v>1</v>
+        <v>180</v>
+      </c>
+      <c r="D98" t="s">
+        <v>65</v>
       </c>
       <c r="E98" t="s">
-        <v>40</v>
+        <v>168</v>
       </c>
       <c r="F98" t="s">
-        <v>43</v>
+        <v>177</v>
       </c>
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.35">
@@ -2848,17 +2873,14 @@
       <c r="B99" t="s">
         <v>19</v>
       </c>
-      <c r="C99" t="s">
-        <v>104</v>
-      </c>
-      <c r="D99">
-        <v>1</v>
+      <c r="D99" t="s">
+        <v>87</v>
       </c>
       <c r="E99" t="s">
-        <v>105</v>
+        <v>53</v>
       </c>
       <c r="F99" t="s">
-        <v>107</v>
+        <v>46</v>
       </c>
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.35">
@@ -2869,16 +2891,16 @@
         <v>19</v>
       </c>
       <c r="C100" t="s">
-        <v>106</v>
+        <v>20</v>
       </c>
       <c r="D100">
         <v>1</v>
       </c>
       <c r="E100" t="s">
-        <v>105</v>
+        <v>40</v>
       </c>
       <c r="F100" t="s">
-        <v>107</v>
+        <v>43</v>
       </c>
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.35">
@@ -2889,16 +2911,16 @@
         <v>19</v>
       </c>
       <c r="C101" t="s">
-        <v>38</v>
+        <v>104</v>
       </c>
       <c r="D101">
         <v>1</v>
       </c>
       <c r="E101" t="s">
-        <v>53</v>
+        <v>105</v>
       </c>
       <c r="F101" t="s">
-        <v>46</v>
+        <v>107</v>
       </c>
     </row>
     <row r="102" spans="1:6" x14ac:dyDescent="0.35">
@@ -2909,16 +2931,16 @@
         <v>19</v>
       </c>
       <c r="C102" t="s">
-        <v>38</v>
+        <v>106</v>
       </c>
       <c r="D102">
         <v>1</v>
       </c>
       <c r="E102" t="s">
-        <v>53</v>
+        <v>105</v>
       </c>
       <c r="F102" t="s">
-        <v>38</v>
+        <v>107</v>
       </c>
     </row>
     <row r="103" spans="1:6" x14ac:dyDescent="0.35">
@@ -2929,13 +2951,16 @@
         <v>19</v>
       </c>
       <c r="C103" t="s">
-        <v>206</v>
+        <v>38</v>
+      </c>
+      <c r="D103">
+        <v>1</v>
       </c>
       <c r="E103" t="s">
-        <v>103</v>
+        <v>53</v>
       </c>
       <c r="F103" t="s">
-        <v>204</v>
+        <v>46</v>
       </c>
     </row>
     <row r="104" spans="1:6" x14ac:dyDescent="0.35">
@@ -2943,16 +2968,19 @@
         <v>32</v>
       </c>
       <c r="B104" t="s">
-        <v>9</v>
-      </c>
-      <c r="D104" t="s">
-        <v>87</v>
+        <v>19</v>
+      </c>
+      <c r="C104" t="s">
+        <v>38</v>
+      </c>
+      <c r="D104">
+        <v>1</v>
       </c>
       <c r="E104" t="s">
-        <v>11</v>
+        <v>53</v>
       </c>
       <c r="F104" t="s">
-        <v>12</v>
+        <v>38</v>
       </c>
     </row>
     <row r="105" spans="1:6" x14ac:dyDescent="0.35">
@@ -2960,19 +2988,16 @@
         <v>32</v>
       </c>
       <c r="B105" t="s">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="C105" t="s">
-        <v>10</v>
-      </c>
-      <c r="D105">
-        <v>1</v>
+        <v>206</v>
       </c>
       <c r="E105" t="s">
-        <v>11</v>
+        <v>103</v>
       </c>
       <c r="F105" t="s">
-        <v>12</v>
+        <v>204</v>
       </c>
     </row>
     <row r="106" spans="1:6" x14ac:dyDescent="0.35">
@@ -2982,17 +3007,14 @@
       <c r="B106" t="s">
         <v>9</v>
       </c>
-      <c r="C106" t="s">
-        <v>16</v>
-      </c>
-      <c r="D106">
-        <v>1</v>
+      <c r="D106" t="s">
+        <v>87</v>
       </c>
       <c r="E106" t="s">
-        <v>40</v>
+        <v>11</v>
       </c>
       <c r="F106" t="s">
-        <v>37</v>
+        <v>12</v>
       </c>
     </row>
     <row r="107" spans="1:6" x14ac:dyDescent="0.35">
@@ -3000,16 +3022,19 @@
         <v>32</v>
       </c>
       <c r="B107" t="s">
-        <v>185</v>
-      </c>
-      <c r="D107" t="s">
-        <v>68</v>
+        <v>9</v>
+      </c>
+      <c r="C107" t="s">
+        <v>10</v>
+      </c>
+      <c r="D107">
+        <v>1</v>
       </c>
       <c r="E107" t="s">
-        <v>105</v>
+        <v>11</v>
       </c>
       <c r="F107" t="s">
-        <v>107</v>
+        <v>12</v>
       </c>
     </row>
     <row r="108" spans="1:6" x14ac:dyDescent="0.35">
@@ -3017,16 +3042,19 @@
         <v>32</v>
       </c>
       <c r="B108" t="s">
-        <v>75</v>
-      </c>
-      <c r="D108" t="s">
-        <v>87</v>
+        <v>9</v>
+      </c>
+      <c r="C108" t="s">
+        <v>16</v>
+      </c>
+      <c r="D108">
+        <v>1</v>
       </c>
       <c r="E108" t="s">
-        <v>11</v>
+        <v>40</v>
       </c>
       <c r="F108" t="s">
-        <v>71</v>
+        <v>37</v>
       </c>
     </row>
     <row r="109" spans="1:6" x14ac:dyDescent="0.35">
@@ -3034,16 +3062,16 @@
         <v>32</v>
       </c>
       <c r="B109" t="s">
-        <v>75</v>
-      </c>
-      <c r="C109" t="s">
-        <v>74</v>
+        <v>185</v>
+      </c>
+      <c r="D109" t="s">
+        <v>68</v>
       </c>
       <c r="E109" t="s">
-        <v>11</v>
+        <v>105</v>
       </c>
       <c r="F109" t="s">
-        <v>71</v>
+        <v>107</v>
       </c>
     </row>
     <row r="110" spans="1:6" x14ac:dyDescent="0.35">
@@ -3051,7 +3079,7 @@
         <v>32</v>
       </c>
       <c r="B110" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="D110" t="s">
         <v>87</v>
@@ -3068,13 +3096,10 @@
         <v>32</v>
       </c>
       <c r="B111" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="C111" t="s">
-        <v>70</v>
-      </c>
-      <c r="D111">
-        <v>2</v>
+        <v>74</v>
       </c>
       <c r="E111" t="s">
         <v>11</v>
@@ -3088,16 +3113,16 @@
         <v>32</v>
       </c>
       <c r="B112" t="s">
-        <v>186</v>
+        <v>72</v>
       </c>
       <c r="D112" t="s">
-        <v>65</v>
+        <v>87</v>
       </c>
       <c r="E112" t="s">
-        <v>85</v>
+        <v>11</v>
       </c>
       <c r="F112" t="s">
-        <v>79</v>
+        <v>71</v>
       </c>
     </row>
     <row r="113" spans="1:6" x14ac:dyDescent="0.35">
@@ -3105,10 +3130,13 @@
         <v>32</v>
       </c>
       <c r="B113" t="s">
-        <v>73</v>
-      </c>
-      <c r="D113" t="s">
-        <v>87</v>
+        <v>72</v>
+      </c>
+      <c r="C113" t="s">
+        <v>70</v>
+      </c>
+      <c r="D113">
+        <v>2</v>
       </c>
       <c r="E113" t="s">
         <v>11</v>
@@ -3122,16 +3150,16 @@
         <v>32</v>
       </c>
       <c r="B114" t="s">
-        <v>73</v>
-      </c>
-      <c r="C114" t="s">
-        <v>74</v>
+        <v>186</v>
+      </c>
+      <c r="D114" t="s">
+        <v>65</v>
       </c>
       <c r="E114" t="s">
-        <v>11</v>
+        <v>85</v>
       </c>
       <c r="F114" t="s">
-        <v>71</v>
+        <v>79</v>
       </c>
     </row>
     <row r="115" spans="1:6" x14ac:dyDescent="0.35">
@@ -3139,7 +3167,7 @@
         <v>32</v>
       </c>
       <c r="B115" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="D115" t="s">
         <v>87</v>
@@ -3156,13 +3184,10 @@
         <v>32</v>
       </c>
       <c r="B116" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="C116" t="s">
-        <v>70</v>
-      </c>
-      <c r="D116">
-        <v>2</v>
+        <v>74</v>
       </c>
       <c r="E116" t="s">
         <v>11</v>
@@ -3176,16 +3201,16 @@
         <v>32</v>
       </c>
       <c r="B117" t="s">
-        <v>92</v>
+        <v>69</v>
       </c>
       <c r="D117" t="s">
         <v>87</v>
       </c>
       <c r="E117" t="s">
-        <v>53</v>
+        <v>11</v>
       </c>
       <c r="F117" t="s">
-        <v>47</v>
+        <v>71</v>
       </c>
     </row>
     <row r="118" spans="1:6" x14ac:dyDescent="0.35">
@@ -3193,16 +3218,19 @@
         <v>32</v>
       </c>
       <c r="B118" t="s">
-        <v>162</v>
-      </c>
-      <c r="D118" t="s">
-        <v>87</v>
+        <v>69</v>
+      </c>
+      <c r="C118" t="s">
+        <v>70</v>
+      </c>
+      <c r="D118">
+        <v>2</v>
       </c>
       <c r="E118" t="s">
-        <v>116</v>
+        <v>11</v>
       </c>
       <c r="F118" t="s">
-        <v>163</v>
+        <v>71</v>
       </c>
     </row>
     <row r="119" spans="1:6" x14ac:dyDescent="0.35">
@@ -3210,19 +3238,16 @@
         <v>32</v>
       </c>
       <c r="B119" t="s">
-        <v>162</v>
-      </c>
-      <c r="C119" t="s">
-        <v>164</v>
-      </c>
-      <c r="D119">
-        <v>1</v>
+        <v>92</v>
+      </c>
+      <c r="D119" t="s">
+        <v>87</v>
       </c>
       <c r="E119" t="s">
-        <v>116</v>
+        <v>53</v>
       </c>
       <c r="F119" t="s">
-        <v>163</v>
+        <v>47</v>
       </c>
     </row>
     <row r="120" spans="1:6" x14ac:dyDescent="0.35">
@@ -3230,16 +3255,19 @@
         <v>32</v>
       </c>
       <c r="B120" t="s">
-        <v>118</v>
-      </c>
-      <c r="D120" t="s">
-        <v>68</v>
-      </c>
-      <c r="E120" t="s">
-        <v>116</v>
-      </c>
-      <c r="F120" t="s">
-        <v>119</v>
+        <v>92</v>
+      </c>
+      <c r="C120" s="2" t="s">
+        <v>220</v>
+      </c>
+      <c r="D120">
+        <v>1</v>
+      </c>
+      <c r="E120" s="2" t="s">
+        <v>219</v>
+      </c>
+      <c r="F120" s="2" t="s">
+        <v>218</v>
       </c>
     </row>
     <row r="121" spans="1:6" x14ac:dyDescent="0.35">
@@ -3247,16 +3275,16 @@
         <v>32</v>
       </c>
       <c r="B121" t="s">
-        <v>118</v>
-      </c>
-      <c r="C121" t="s">
-        <v>124</v>
+        <v>162</v>
+      </c>
+      <c r="D121" t="s">
+        <v>87</v>
       </c>
       <c r="E121" t="s">
         <v>116</v>
       </c>
       <c r="F121" t="s">
-        <v>121</v>
+        <v>163</v>
       </c>
     </row>
     <row r="122" spans="1:6" x14ac:dyDescent="0.35">
@@ -3264,16 +3292,19 @@
         <v>32</v>
       </c>
       <c r="B122" t="s">
-        <v>118</v>
+        <v>162</v>
       </c>
       <c r="C122" t="s">
-        <v>52</v>
+        <v>164</v>
+      </c>
+      <c r="D122">
+        <v>1</v>
       </c>
       <c r="E122" t="s">
         <v>116</v>
       </c>
       <c r="F122" t="s">
-        <v>119</v>
+        <v>163</v>
       </c>
     </row>
     <row r="123" spans="1:6" x14ac:dyDescent="0.35">
@@ -3283,14 +3314,14 @@
       <c r="B123" t="s">
         <v>118</v>
       </c>
-      <c r="C123" t="s">
-        <v>129</v>
+      <c r="D123" t="s">
+        <v>68</v>
       </c>
       <c r="E123" t="s">
         <v>116</v>
       </c>
       <c r="F123" t="s">
-        <v>130</v>
+        <v>119</v>
       </c>
     </row>
     <row r="124" spans="1:6" x14ac:dyDescent="0.35">
@@ -3301,7 +3332,7 @@
         <v>118</v>
       </c>
       <c r="C124" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="E124" t="s">
         <v>116</v>
@@ -3318,13 +3349,13 @@
         <v>118</v>
       </c>
       <c r="C125" t="s">
-        <v>136</v>
+        <v>52</v>
       </c>
       <c r="E125" t="s">
         <v>116</v>
       </c>
       <c r="F125" t="s">
-        <v>137</v>
+        <v>119</v>
       </c>
     </row>
     <row r="126" spans="1:6" x14ac:dyDescent="0.35">
@@ -3335,13 +3366,13 @@
         <v>118</v>
       </c>
       <c r="C126" t="s">
-        <v>146</v>
+        <v>129</v>
       </c>
       <c r="E126" t="s">
         <v>116</v>
       </c>
       <c r="F126" t="s">
-        <v>147</v>
+        <v>130</v>
       </c>
     </row>
     <row r="127" spans="1:6" x14ac:dyDescent="0.35">
@@ -3352,13 +3383,13 @@
         <v>118</v>
       </c>
       <c r="C127" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="E127" t="s">
         <v>116</v>
       </c>
       <c r="F127" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="128" spans="1:6" x14ac:dyDescent="0.35">
@@ -3369,13 +3400,13 @@
         <v>118</v>
       </c>
       <c r="C128" t="s">
-        <v>51</v>
+        <v>136</v>
       </c>
       <c r="E128" t="s">
         <v>116</v>
       </c>
       <c r="F128" t="s">
-        <v>119</v>
+        <v>137</v>
       </c>
     </row>
     <row r="129" spans="1:6" x14ac:dyDescent="0.35">
@@ -3383,16 +3414,16 @@
         <v>32</v>
       </c>
       <c r="B129" t="s">
-        <v>165</v>
-      </c>
-      <c r="D129" t="s">
-        <v>87</v>
+        <v>118</v>
+      </c>
+      <c r="C129" t="s">
+        <v>146</v>
       </c>
       <c r="E129" t="s">
         <v>116</v>
       </c>
       <c r="F129" t="s">
-        <v>163</v>
+        <v>147</v>
       </c>
     </row>
     <row r="130" spans="1:6" x14ac:dyDescent="0.35">
@@ -3400,16 +3431,16 @@
         <v>32</v>
       </c>
       <c r="B130" t="s">
-        <v>165</v>
+        <v>118</v>
       </c>
       <c r="C130" t="s">
-        <v>166</v>
+        <v>120</v>
       </c>
       <c r="E130" t="s">
         <v>116</v>
       </c>
       <c r="F130" t="s">
-        <v>163</v>
+        <v>122</v>
       </c>
     </row>
     <row r="131" spans="1:6" x14ac:dyDescent="0.35">
@@ -3417,16 +3448,16 @@
         <v>32</v>
       </c>
       <c r="B131" t="s">
-        <v>149</v>
-      </c>
-      <c r="D131" t="s">
-        <v>68</v>
+        <v>118</v>
+      </c>
+      <c r="C131" t="s">
+        <v>51</v>
       </c>
       <c r="E131" t="s">
         <v>116</v>
       </c>
       <c r="F131" t="s">
-        <v>147</v>
+        <v>119</v>
       </c>
     </row>
     <row r="132" spans="1:6" x14ac:dyDescent="0.35">
@@ -3434,16 +3465,16 @@
         <v>32</v>
       </c>
       <c r="B132" t="s">
-        <v>149</v>
-      </c>
-      <c r="C132" t="s">
-        <v>151</v>
+        <v>165</v>
+      </c>
+      <c r="D132" t="s">
+        <v>87</v>
       </c>
       <c r="E132" t="s">
         <v>116</v>
       </c>
       <c r="F132" t="s">
-        <v>147</v>
+        <v>163</v>
       </c>
     </row>
     <row r="133" spans="1:6" x14ac:dyDescent="0.35">
@@ -3451,16 +3482,16 @@
         <v>32</v>
       </c>
       <c r="B133" t="s">
-        <v>149</v>
+        <v>165</v>
       </c>
       <c r="C133" t="s">
-        <v>49</v>
+        <v>166</v>
       </c>
       <c r="E133" t="s">
         <v>116</v>
       </c>
       <c r="F133" t="s">
-        <v>147</v>
+        <v>163</v>
       </c>
     </row>
     <row r="134" spans="1:6" x14ac:dyDescent="0.35">
@@ -3470,8 +3501,8 @@
       <c r="B134" t="s">
         <v>149</v>
       </c>
-      <c r="C134" t="s">
-        <v>150</v>
+      <c r="D134" t="s">
+        <v>68</v>
       </c>
       <c r="E134" t="s">
         <v>116</v>
@@ -3488,7 +3519,7 @@
         <v>149</v>
       </c>
       <c r="C135" t="s">
-        <v>50</v>
+        <v>151</v>
       </c>
       <c r="E135" t="s">
         <v>116</v>
@@ -3502,16 +3533,16 @@
         <v>32</v>
       </c>
       <c r="B136" t="s">
-        <v>138</v>
-      </c>
-      <c r="D136" t="s">
-        <v>68</v>
+        <v>149</v>
+      </c>
+      <c r="C136" t="s">
+        <v>49</v>
       </c>
       <c r="E136" t="s">
         <v>116</v>
       </c>
       <c r="F136" t="s">
-        <v>137</v>
+        <v>147</v>
       </c>
     </row>
     <row r="137" spans="1:6" x14ac:dyDescent="0.35">
@@ -3519,10 +3550,10 @@
         <v>32</v>
       </c>
       <c r="B137" t="s">
-        <v>138</v>
+        <v>149</v>
       </c>
       <c r="C137" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="E137" t="s">
         <v>116</v>
@@ -3536,16 +3567,16 @@
         <v>32</v>
       </c>
       <c r="B138" t="s">
-        <v>138</v>
+        <v>149</v>
       </c>
       <c r="C138" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="E138" t="s">
         <v>116</v>
       </c>
       <c r="F138" t="s">
-        <v>137</v>
+        <v>147</v>
       </c>
     </row>
     <row r="139" spans="1:6" x14ac:dyDescent="0.35">
@@ -3555,8 +3586,8 @@
       <c r="B139" t="s">
         <v>138</v>
       </c>
-      <c r="C139" t="s">
-        <v>57</v>
+      <c r="D139" t="s">
+        <v>68</v>
       </c>
       <c r="E139" t="s">
         <v>116</v>
@@ -3573,13 +3604,13 @@
         <v>138</v>
       </c>
       <c r="C140" t="s">
-        <v>156</v>
+        <v>148</v>
       </c>
       <c r="E140" t="s">
         <v>116</v>
       </c>
       <c r="F140" t="s">
-        <v>158</v>
+        <v>147</v>
       </c>
     </row>
     <row r="141" spans="1:6" x14ac:dyDescent="0.35">
@@ -3590,13 +3621,13 @@
         <v>138</v>
       </c>
       <c r="C141" t="s">
-        <v>154</v>
+        <v>58</v>
       </c>
       <c r="E141" t="s">
         <v>116</v>
       </c>
       <c r="F141" t="s">
-        <v>155</v>
+        <v>137</v>
       </c>
     </row>
     <row r="142" spans="1:6" x14ac:dyDescent="0.35">
@@ -3607,13 +3638,13 @@
         <v>138</v>
       </c>
       <c r="C142" t="s">
-        <v>184</v>
+        <v>57</v>
       </c>
       <c r="E142" t="s">
         <v>116</v>
       </c>
       <c r="F142" t="s">
-        <v>183</v>
+        <v>137</v>
       </c>
     </row>
     <row r="143" spans="1:6" x14ac:dyDescent="0.35">
@@ -3624,7 +3655,7 @@
         <v>138</v>
       </c>
       <c r="C143" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="E143" t="s">
         <v>116</v>
@@ -3638,16 +3669,16 @@
         <v>32</v>
       </c>
       <c r="B144" t="s">
-        <v>125</v>
-      </c>
-      <c r="D144" t="s">
-        <v>68</v>
+        <v>138</v>
+      </c>
+      <c r="C144" t="s">
+        <v>154</v>
       </c>
       <c r="E144" t="s">
         <v>116</v>
       </c>
       <c r="F144" t="s">
-        <v>121</v>
+        <v>155</v>
       </c>
     </row>
     <row r="145" spans="1:6" x14ac:dyDescent="0.35">
@@ -3655,16 +3686,16 @@
         <v>32</v>
       </c>
       <c r="B145" t="s">
-        <v>125</v>
+        <v>138</v>
       </c>
       <c r="C145" t="s">
-        <v>127</v>
+        <v>184</v>
       </c>
       <c r="E145" t="s">
         <v>116</v>
       </c>
       <c r="F145" t="s">
-        <v>121</v>
+        <v>183</v>
       </c>
     </row>
     <row r="146" spans="1:6" x14ac:dyDescent="0.35">
@@ -3672,16 +3703,16 @@
         <v>32</v>
       </c>
       <c r="B146" t="s">
-        <v>131</v>
-      </c>
-      <c r="D146" t="s">
-        <v>68</v>
+        <v>138</v>
+      </c>
+      <c r="C146" t="s">
+        <v>157</v>
       </c>
       <c r="E146" t="s">
         <v>116</v>
       </c>
       <c r="F146" t="s">
-        <v>130</v>
+        <v>158</v>
       </c>
     </row>
     <row r="147" spans="1:6" x14ac:dyDescent="0.35">
@@ -3689,16 +3720,16 @@
         <v>32</v>
       </c>
       <c r="B147" t="s">
-        <v>131</v>
-      </c>
-      <c r="C147" t="s">
-        <v>132</v>
+        <v>125</v>
+      </c>
+      <c r="D147" t="s">
+        <v>68</v>
       </c>
       <c r="E147" t="s">
         <v>116</v>
       </c>
       <c r="F147" t="s">
-        <v>130</v>
+        <v>121</v>
       </c>
     </row>
     <row r="148" spans="1:6" x14ac:dyDescent="0.35">
@@ -3706,16 +3737,16 @@
         <v>32</v>
       </c>
       <c r="B148" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
       <c r="C148" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="E148" t="s">
         <v>116</v>
       </c>
       <c r="F148" t="s">
-        <v>130</v>
+        <v>121</v>
       </c>
     </row>
     <row r="149" spans="1:6" x14ac:dyDescent="0.35">
@@ -3725,8 +3756,8 @@
       <c r="B149" t="s">
         <v>131</v>
       </c>
-      <c r="C149" t="s">
-        <v>134</v>
+      <c r="D149" t="s">
+        <v>68</v>
       </c>
       <c r="E149" t="s">
         <v>116</v>
@@ -3743,7 +3774,7 @@
         <v>131</v>
       </c>
       <c r="C150" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="E150" t="s">
         <v>116</v>
@@ -3757,16 +3788,16 @@
         <v>32</v>
       </c>
       <c r="B151" t="s">
-        <v>126</v>
-      </c>
-      <c r="D151" t="s">
-        <v>68</v>
+        <v>131</v>
+      </c>
+      <c r="C151" t="s">
+        <v>133</v>
       </c>
       <c r="E151" t="s">
         <v>116</v>
       </c>
       <c r="F151" t="s">
-        <v>121</v>
+        <v>130</v>
       </c>
     </row>
     <row r="152" spans="1:6" x14ac:dyDescent="0.35">
@@ -3774,16 +3805,16 @@
         <v>32</v>
       </c>
       <c r="B152" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="C152" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="E152" t="s">
         <v>116</v>
       </c>
       <c r="F152" t="s">
-        <v>121</v>
+        <v>130</v>
       </c>
     </row>
     <row r="153" spans="1:6" x14ac:dyDescent="0.35">
@@ -3791,16 +3822,16 @@
         <v>32</v>
       </c>
       <c r="B153" t="s">
-        <v>98</v>
-      </c>
-      <c r="D153" t="s">
-        <v>87</v>
+        <v>131</v>
+      </c>
+      <c r="C153" t="s">
+        <v>135</v>
       </c>
       <c r="E153" t="s">
-        <v>14</v>
+        <v>116</v>
       </c>
       <c r="F153" t="s">
-        <v>99</v>
+        <v>130</v>
       </c>
     </row>
     <row r="154" spans="1:6" x14ac:dyDescent="0.35">
@@ -3808,16 +3839,16 @@
         <v>32</v>
       </c>
       <c r="B154" t="s">
-        <v>13</v>
+        <v>126</v>
       </c>
       <c r="D154" t="s">
-        <v>87</v>
+        <v>68</v>
       </c>
       <c r="E154" t="s">
-        <v>14</v>
+        <v>116</v>
       </c>
       <c r="F154" t="s">
-        <v>17</v>
+        <v>121</v>
       </c>
     </row>
     <row r="155" spans="1:6" x14ac:dyDescent="0.35">
@@ -3825,19 +3856,16 @@
         <v>32</v>
       </c>
       <c r="B155" t="s">
-        <v>13</v>
+        <v>126</v>
       </c>
       <c r="C155" t="s">
-        <v>10</v>
-      </c>
-      <c r="D155">
-        <v>1</v>
+        <v>128</v>
       </c>
       <c r="E155" t="s">
-        <v>14</v>
+        <v>116</v>
       </c>
       <c r="F155" t="s">
-        <v>15</v>
+        <v>121</v>
       </c>
     </row>
     <row r="156" spans="1:6" x14ac:dyDescent="0.35">
@@ -3845,19 +3873,16 @@
         <v>32</v>
       </c>
       <c r="B156" t="s">
-        <v>13</v>
-      </c>
-      <c r="C156" t="s">
-        <v>20</v>
-      </c>
-      <c r="D156">
-        <v>1</v>
+        <v>98</v>
+      </c>
+      <c r="D156" t="s">
+        <v>87</v>
       </c>
       <c r="E156" t="s">
         <v>14</v>
       </c>
       <c r="F156" t="s">
-        <v>23</v>
+        <v>99</v>
       </c>
     </row>
     <row r="157" spans="1:6" x14ac:dyDescent="0.35">
@@ -3867,11 +3892,8 @@
       <c r="B157" t="s">
         <v>13</v>
       </c>
-      <c r="C157" t="s">
-        <v>18</v>
-      </c>
-      <c r="D157">
-        <v>1</v>
+      <c r="D157" t="s">
+        <v>87</v>
       </c>
       <c r="E157" t="s">
         <v>14</v>
@@ -3885,16 +3907,19 @@
         <v>32</v>
       </c>
       <c r="B158" t="s">
-        <v>97</v>
-      </c>
-      <c r="D158" t="s">
-        <v>87</v>
+        <v>13</v>
+      </c>
+      <c r="C158" t="s">
+        <v>10</v>
+      </c>
+      <c r="D158">
+        <v>1</v>
       </c>
       <c r="E158" t="s">
-        <v>54</v>
+        <v>14</v>
       </c>
       <c r="F158" t="s">
-        <v>63</v>
+        <v>15</v>
       </c>
     </row>
     <row r="159" spans="1:6" x14ac:dyDescent="0.35">
@@ -3902,16 +3927,19 @@
         <v>32</v>
       </c>
       <c r="B159" t="s">
-        <v>97</v>
+        <v>13</v>
       </c>
       <c r="C159" t="s">
-        <v>191</v>
+        <v>20</v>
+      </c>
+      <c r="D159">
+        <v>1</v>
       </c>
       <c r="E159" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F159" t="s">
-        <v>89</v>
+        <v>23</v>
       </c>
     </row>
     <row r="160" spans="1:6" x14ac:dyDescent="0.35">
@@ -3919,16 +3947,19 @@
         <v>32</v>
       </c>
       <c r="B160" t="s">
-        <v>33</v>
-      </c>
-      <c r="D160" t="s">
-        <v>87</v>
+        <v>13</v>
+      </c>
+      <c r="C160" t="s">
+        <v>18</v>
+      </c>
+      <c r="D160">
+        <v>1</v>
       </c>
       <c r="E160" t="s">
-        <v>54</v>
+        <v>14</v>
       </c>
       <c r="F160" t="s">
-        <v>56</v>
+        <v>17</v>
       </c>
     </row>
     <row r="161" spans="1:6" x14ac:dyDescent="0.35">
@@ -3936,13 +3967,10 @@
         <v>32</v>
       </c>
       <c r="B161" t="s">
-        <v>33</v>
-      </c>
-      <c r="C161" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="D161">
-        <v>1</v>
+        <v>97</v>
+      </c>
+      <c r="D161" t="s">
+        <v>87</v>
       </c>
       <c r="E161" t="s">
         <v>54</v>
@@ -3956,10 +3984,10 @@
         <v>32</v>
       </c>
       <c r="B162" t="s">
-        <v>33</v>
-      </c>
-      <c r="C162" s="1" t="s">
-        <v>39</v>
+        <v>97</v>
+      </c>
+      <c r="C162" s="2" t="s">
+        <v>216</v>
       </c>
       <c r="D162">
         <v>1</v>
@@ -3967,8 +3995,8 @@
       <c r="E162" t="s">
         <v>54</v>
       </c>
-      <c r="F162" t="s">
-        <v>55</v>
+      <c r="F162" s="2" t="s">
+        <v>193</v>
       </c>
     </row>
     <row r="163" spans="1:6" x14ac:dyDescent="0.35">
@@ -3976,16 +4004,16 @@
         <v>32</v>
       </c>
       <c r="B163" t="s">
-        <v>33</v>
-      </c>
-      <c r="C163" s="1" t="s">
-        <v>57</v>
+        <v>97</v>
+      </c>
+      <c r="C163" t="s">
+        <v>191</v>
       </c>
       <c r="E163" t="s">
-        <v>54</v>
+        <v>24</v>
       </c>
       <c r="F163" t="s">
-        <v>56</v>
+        <v>89</v>
       </c>
     </row>
     <row r="164" spans="1:6" x14ac:dyDescent="0.35">
@@ -3995,14 +4023,14 @@
       <c r="B164" t="s">
         <v>33</v>
       </c>
-      <c r="C164" s="1" t="s">
-        <v>195</v>
+      <c r="D164" t="s">
+        <v>87</v>
       </c>
       <c r="E164" t="s">
         <v>54</v>
       </c>
       <c r="F164" t="s">
-        <v>193</v>
+        <v>56</v>
       </c>
     </row>
     <row r="165" spans="1:6" x14ac:dyDescent="0.35">
@@ -4010,17 +4038,19 @@
         <v>32</v>
       </c>
       <c r="B165" t="s">
-        <v>182</v>
-      </c>
-      <c r="C165" s="1"/>
-      <c r="D165" t="s">
-        <v>68</v>
+        <v>33</v>
+      </c>
+      <c r="C165" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="D165">
+        <v>1</v>
       </c>
       <c r="E165" t="s">
-        <v>116</v>
+        <v>54</v>
       </c>
       <c r="F165" t="s">
-        <v>183</v>
+        <v>193</v>
       </c>
     </row>
     <row r="166" spans="1:6" x14ac:dyDescent="0.35">
@@ -4028,15 +4058,107 @@
         <v>32</v>
       </c>
       <c r="B166" t="s">
+        <v>33</v>
+      </c>
+      <c r="C166" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D166">
+        <v>1</v>
+      </c>
+      <c r="E166" t="s">
+        <v>54</v>
+      </c>
+      <c r="F166" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="167" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A167" t="s">
+        <v>32</v>
+      </c>
+      <c r="B167" t="s">
+        <v>33</v>
+      </c>
+      <c r="C167" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D167">
+        <v>1</v>
+      </c>
+      <c r="E167" t="s">
+        <v>54</v>
+      </c>
+      <c r="F167" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="168" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A168" t="s">
+        <v>32</v>
+      </c>
+      <c r="B168" t="s">
+        <v>33</v>
+      </c>
+      <c r="C168" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="E168" t="s">
+        <v>54</v>
+      </c>
+      <c r="F168" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="169" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A169" t="s">
+        <v>32</v>
+      </c>
+      <c r="B169" t="s">
+        <v>33</v>
+      </c>
+      <c r="C169" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="E169" t="s">
+        <v>54</v>
+      </c>
+      <c r="F169" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="170" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A170" t="s">
+        <v>32</v>
+      </c>
+      <c r="B170" t="s">
+        <v>182</v>
+      </c>
+      <c r="C170" s="1"/>
+      <c r="D170" t="s">
+        <v>68</v>
+      </c>
+      <c r="E170" t="s">
+        <v>116</v>
+      </c>
+      <c r="F170" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="171" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A171" t="s">
+        <v>32</v>
+      </c>
+      <c r="B171" t="s">
         <v>88</v>
       </c>
-      <c r="D166" t="s">
+      <c r="D171" t="s">
         <v>65</v>
       </c>
-      <c r="E166" t="s">
+      <c r="E171" t="s">
         <v>24</v>
       </c>
-      <c r="F166" t="s">
+      <c r="F171" t="s">
         <v>89</v>
       </c>
     </row>

</xml_diff>

<commit_message>
[PowerPoint] (ThemeColorScheme) Add snippet
</commit_message>
<xml_diff>
--- a/snippet-extractor-metadata/powerpoint.xlsx
+++ b/snippet-extractor-metadata/powerpoint.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A2CA723-45CB-4135-8A1A-0329A73196F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D0F7BFA-D1AA-43BE-B4C8-CBE72F79E65D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25180" windowHeight="16140" xr2:uid="{CB5595D7-4492-4192-A1C1-2583BA1957AA}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="856" uniqueCount="223">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="871" uniqueCount="230">
   <si>
     <t>Class</t>
   </si>
@@ -689,6 +689,27 @@
   </si>
   <si>
     <t>getShapeById</t>
+  </si>
+  <si>
+    <t>themeColorScheme</t>
+  </si>
+  <si>
+    <t>getThemeColors</t>
+  </si>
+  <si>
+    <t>powerpoint-slide-management-get-set-theme-color-scheme</t>
+  </si>
+  <si>
+    <t>ThemeColor</t>
+  </si>
+  <si>
+    <t>setThemeColors</t>
+  </si>
+  <si>
+    <t>ThemeColorScheme</t>
+  </si>
+  <si>
+    <t>resetThemeColors</t>
   </si>
 </sst>
 </file>
@@ -769,10 +790,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{78C585A5-D505-49C6-9CA1-8E6558948317}" name="Snippets" displayName="Snippets" ref="A1:F171" totalsRowShown="0" headerRowDxfId="4">
-  <autoFilter ref="A1:F171" xr:uid="{EAC65D03-FDD2-4352-A5F3-1CDEDE6251B2}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F167">
-    <sortCondition ref="B1:B167"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{78C585A5-D505-49C6-9CA1-8E6558948317}" name="Snippets" displayName="Snippets" ref="A1:F174" totalsRowShown="0" headerRowDxfId="4">
+  <autoFilter ref="A1:F174" xr:uid="{EAC65D03-FDD2-4352-A5F3-1CDEDE6251B2}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F168">
+    <sortCondition ref="B1:B168"/>
   </sortState>
   <tableColumns count="6">
     <tableColumn id="6" xr3:uid="{408888B8-C1DD-4B51-B1EB-5663F091D142}" name="Package"/>
@@ -1083,7 +1104,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{809930CD-A227-47DC-AAA4-BB816AEDEB59}">
-  <dimension ref="A1:F171"/>
+  <dimension ref="A1:F174"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="11.453125" bestFit="1" customWidth="1"/>
@@ -2006,16 +2027,16 @@
       <c r="B51" t="s">
         <v>45</v>
       </c>
-      <c r="C51" s="2" t="s">
+      <c r="C51" t="s">
         <v>217</v>
       </c>
       <c r="D51">
         <v>1</v>
       </c>
-      <c r="E51" s="2" t="s">
+      <c r="E51" t="s">
         <v>54</v>
       </c>
-      <c r="F51" s="2" t="s">
+      <c r="F51" t="s">
         <v>193</v>
       </c>
     </row>
@@ -2802,16 +2823,16 @@
       <c r="B95" t="s">
         <v>90</v>
       </c>
-      <c r="C95" s="2" t="s">
+      <c r="C95" t="s">
         <v>220</v>
       </c>
       <c r="D95">
         <v>1</v>
       </c>
-      <c r="E95" s="2" t="s">
+      <c r="E95" t="s">
         <v>221</v>
       </c>
-      <c r="F95" s="2" t="s">
+      <c r="F95" t="s">
         <v>222</v>
       </c>
     </row>
@@ -3005,16 +3026,16 @@
         <v>32</v>
       </c>
       <c r="B106" t="s">
-        <v>9</v>
-      </c>
-      <c r="D106" t="s">
-        <v>87</v>
-      </c>
-      <c r="E106" t="s">
-        <v>11</v>
-      </c>
-      <c r="F106" t="s">
-        <v>12</v>
+        <v>19</v>
+      </c>
+      <c r="C106" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="E106" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="F106" s="2" t="s">
+        <v>224</v>
       </c>
     </row>
     <row r="107" spans="1:6" x14ac:dyDescent="0.35">
@@ -3024,11 +3045,8 @@
       <c r="B107" t="s">
         <v>9</v>
       </c>
-      <c r="C107" t="s">
-        <v>10</v>
-      </c>
-      <c r="D107">
-        <v>1</v>
+      <c r="D107" t="s">
+        <v>87</v>
       </c>
       <c r="E107" t="s">
         <v>11</v>
@@ -3045,16 +3063,16 @@
         <v>9</v>
       </c>
       <c r="C108" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="D108">
         <v>1</v>
       </c>
       <c r="E108" t="s">
-        <v>40</v>
+        <v>11</v>
       </c>
       <c r="F108" t="s">
-        <v>37</v>
+        <v>12</v>
       </c>
     </row>
     <row r="109" spans="1:6" x14ac:dyDescent="0.35">
@@ -3062,16 +3080,19 @@
         <v>32</v>
       </c>
       <c r="B109" t="s">
-        <v>185</v>
-      </c>
-      <c r="D109" t="s">
-        <v>68</v>
+        <v>9</v>
+      </c>
+      <c r="C109" t="s">
+        <v>16</v>
+      </c>
+      <c r="D109">
+        <v>1</v>
       </c>
       <c r="E109" t="s">
-        <v>105</v>
+        <v>40</v>
       </c>
       <c r="F109" t="s">
-        <v>107</v>
+        <v>37</v>
       </c>
     </row>
     <row r="110" spans="1:6" x14ac:dyDescent="0.35">
@@ -3079,16 +3100,16 @@
         <v>32</v>
       </c>
       <c r="B110" t="s">
-        <v>75</v>
+        <v>185</v>
       </c>
       <c r="D110" t="s">
-        <v>87</v>
+        <v>68</v>
       </c>
       <c r="E110" t="s">
-        <v>11</v>
+        <v>105</v>
       </c>
       <c r="F110" t="s">
-        <v>71</v>
+        <v>107</v>
       </c>
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.35">
@@ -3098,8 +3119,8 @@
       <c r="B111" t="s">
         <v>75</v>
       </c>
-      <c r="C111" t="s">
-        <v>74</v>
+      <c r="D111" t="s">
+        <v>87</v>
       </c>
       <c r="E111" t="s">
         <v>11</v>
@@ -3113,10 +3134,10 @@
         <v>32</v>
       </c>
       <c r="B112" t="s">
-        <v>72</v>
-      </c>
-      <c r="D112" t="s">
-        <v>87</v>
+        <v>75</v>
+      </c>
+      <c r="C112" t="s">
+        <v>74</v>
       </c>
       <c r="E112" t="s">
         <v>11</v>
@@ -3132,11 +3153,8 @@
       <c r="B113" t="s">
         <v>72</v>
       </c>
-      <c r="C113" t="s">
-        <v>70</v>
-      </c>
-      <c r="D113">
-        <v>2</v>
+      <c r="D113" t="s">
+        <v>87</v>
       </c>
       <c r="E113" t="s">
         <v>11</v>
@@ -3150,16 +3168,19 @@
         <v>32</v>
       </c>
       <c r="B114" t="s">
-        <v>186</v>
-      </c>
-      <c r="D114" t="s">
-        <v>65</v>
+        <v>72</v>
+      </c>
+      <c r="C114" t="s">
+        <v>70</v>
+      </c>
+      <c r="D114">
+        <v>2</v>
       </c>
       <c r="E114" t="s">
-        <v>85</v>
+        <v>11</v>
       </c>
       <c r="F114" t="s">
-        <v>79</v>
+        <v>71</v>
       </c>
     </row>
     <row r="115" spans="1:6" x14ac:dyDescent="0.35">
@@ -3167,16 +3188,16 @@
         <v>32</v>
       </c>
       <c r="B115" t="s">
-        <v>73</v>
+        <v>186</v>
       </c>
       <c r="D115" t="s">
-        <v>87</v>
+        <v>65</v>
       </c>
       <c r="E115" t="s">
-        <v>11</v>
+        <v>85</v>
       </c>
       <c r="F115" t="s">
-        <v>71</v>
+        <v>79</v>
       </c>
     </row>
     <row r="116" spans="1:6" x14ac:dyDescent="0.35">
@@ -3186,8 +3207,8 @@
       <c r="B116" t="s">
         <v>73</v>
       </c>
-      <c r="C116" t="s">
-        <v>74</v>
+      <c r="D116" t="s">
+        <v>87</v>
       </c>
       <c r="E116" t="s">
         <v>11</v>
@@ -3201,10 +3222,10 @@
         <v>32</v>
       </c>
       <c r="B117" t="s">
-        <v>69</v>
-      </c>
-      <c r="D117" t="s">
-        <v>87</v>
+        <v>73</v>
+      </c>
+      <c r="C117" t="s">
+        <v>74</v>
       </c>
       <c r="E117" t="s">
         <v>11</v>
@@ -3220,11 +3241,8 @@
       <c r="B118" t="s">
         <v>69</v>
       </c>
-      <c r="C118" t="s">
-        <v>70</v>
-      </c>
-      <c r="D118">
-        <v>2</v>
+      <c r="D118" t="s">
+        <v>87</v>
       </c>
       <c r="E118" t="s">
         <v>11</v>
@@ -3238,16 +3256,19 @@
         <v>32</v>
       </c>
       <c r="B119" t="s">
-        <v>92</v>
-      </c>
-      <c r="D119" t="s">
-        <v>87</v>
+        <v>69</v>
+      </c>
+      <c r="C119" t="s">
+        <v>70</v>
+      </c>
+      <c r="D119">
+        <v>2</v>
       </c>
       <c r="E119" t="s">
-        <v>53</v>
+        <v>11</v>
       </c>
       <c r="F119" t="s">
-        <v>47</v>
+        <v>71</v>
       </c>
     </row>
     <row r="120" spans="1:6" x14ac:dyDescent="0.35">
@@ -3257,17 +3278,14 @@
       <c r="B120" t="s">
         <v>92</v>
       </c>
-      <c r="C120" s="2" t="s">
-        <v>220</v>
-      </c>
-      <c r="D120">
-        <v>1</v>
-      </c>
-      <c r="E120" s="2" t="s">
-        <v>219</v>
-      </c>
-      <c r="F120" s="2" t="s">
-        <v>218</v>
+      <c r="D120" t="s">
+        <v>87</v>
+      </c>
+      <c r="E120" t="s">
+        <v>53</v>
+      </c>
+      <c r="F120" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="121" spans="1:6" x14ac:dyDescent="0.35">
@@ -3275,16 +3293,19 @@
         <v>32</v>
       </c>
       <c r="B121" t="s">
-        <v>162</v>
-      </c>
-      <c r="D121" t="s">
-        <v>87</v>
+        <v>92</v>
+      </c>
+      <c r="C121" t="s">
+        <v>220</v>
+      </c>
+      <c r="D121">
+        <v>1</v>
       </c>
       <c r="E121" t="s">
-        <v>116</v>
+        <v>219</v>
       </c>
       <c r="F121" t="s">
-        <v>163</v>
+        <v>218</v>
       </c>
     </row>
     <row r="122" spans="1:6" x14ac:dyDescent="0.35">
@@ -3294,11 +3315,8 @@
       <c r="B122" t="s">
         <v>162</v>
       </c>
-      <c r="C122" t="s">
-        <v>164</v>
-      </c>
-      <c r="D122">
-        <v>1</v>
+      <c r="D122" t="s">
+        <v>87</v>
       </c>
       <c r="E122" t="s">
         <v>116</v>
@@ -3312,16 +3330,19 @@
         <v>32</v>
       </c>
       <c r="B123" t="s">
-        <v>118</v>
-      </c>
-      <c r="D123" t="s">
-        <v>68</v>
+        <v>162</v>
+      </c>
+      <c r="C123" t="s">
+        <v>164</v>
+      </c>
+      <c r="D123">
+        <v>1</v>
       </c>
       <c r="E123" t="s">
         <v>116</v>
       </c>
       <c r="F123" t="s">
-        <v>119</v>
+        <v>163</v>
       </c>
     </row>
     <row r="124" spans="1:6" x14ac:dyDescent="0.35">
@@ -3331,14 +3352,14 @@
       <c r="B124" t="s">
         <v>118</v>
       </c>
-      <c r="C124" t="s">
-        <v>124</v>
+      <c r="D124" t="s">
+        <v>68</v>
       </c>
       <c r="E124" t="s">
         <v>116</v>
       </c>
       <c r="F124" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
     <row r="125" spans="1:6" x14ac:dyDescent="0.35">
@@ -3349,13 +3370,13 @@
         <v>118</v>
       </c>
       <c r="C125" t="s">
-        <v>52</v>
+        <v>124</v>
       </c>
       <c r="E125" t="s">
         <v>116</v>
       </c>
       <c r="F125" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
     </row>
     <row r="126" spans="1:6" x14ac:dyDescent="0.35">
@@ -3366,13 +3387,13 @@
         <v>118</v>
       </c>
       <c r="C126" t="s">
-        <v>129</v>
+        <v>52</v>
       </c>
       <c r="E126" t="s">
         <v>116</v>
       </c>
       <c r="F126" t="s">
-        <v>130</v>
+        <v>119</v>
       </c>
     </row>
     <row r="127" spans="1:6" x14ac:dyDescent="0.35">
@@ -3383,13 +3404,13 @@
         <v>118</v>
       </c>
       <c r="C127" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="E127" t="s">
         <v>116</v>
       </c>
       <c r="F127" t="s">
-        <v>121</v>
+        <v>130</v>
       </c>
     </row>
     <row r="128" spans="1:6" x14ac:dyDescent="0.35">
@@ -3400,13 +3421,13 @@
         <v>118</v>
       </c>
       <c r="C128" t="s">
-        <v>136</v>
+        <v>123</v>
       </c>
       <c r="E128" t="s">
         <v>116</v>
       </c>
       <c r="F128" t="s">
-        <v>137</v>
+        <v>121</v>
       </c>
     </row>
     <row r="129" spans="1:6" x14ac:dyDescent="0.35">
@@ -3417,13 +3438,13 @@
         <v>118</v>
       </c>
       <c r="C129" t="s">
-        <v>146</v>
+        <v>136</v>
       </c>
       <c r="E129" t="s">
         <v>116</v>
       </c>
       <c r="F129" t="s">
-        <v>147</v>
+        <v>137</v>
       </c>
     </row>
     <row r="130" spans="1:6" x14ac:dyDescent="0.35">
@@ -3434,13 +3455,13 @@
         <v>118</v>
       </c>
       <c r="C130" t="s">
-        <v>120</v>
+        <v>146</v>
       </c>
       <c r="E130" t="s">
         <v>116</v>
       </c>
       <c r="F130" t="s">
-        <v>122</v>
+        <v>147</v>
       </c>
     </row>
     <row r="131" spans="1:6" x14ac:dyDescent="0.35">
@@ -3451,13 +3472,13 @@
         <v>118</v>
       </c>
       <c r="C131" t="s">
-        <v>51</v>
+        <v>120</v>
       </c>
       <c r="E131" t="s">
         <v>116</v>
       </c>
       <c r="F131" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
     </row>
     <row r="132" spans="1:6" x14ac:dyDescent="0.35">
@@ -3465,16 +3486,16 @@
         <v>32</v>
       </c>
       <c r="B132" t="s">
-        <v>165</v>
-      </c>
-      <c r="D132" t="s">
-        <v>87</v>
+        <v>118</v>
+      </c>
+      <c r="C132" t="s">
+        <v>51</v>
       </c>
       <c r="E132" t="s">
         <v>116</v>
       </c>
       <c r="F132" t="s">
-        <v>163</v>
+        <v>119</v>
       </c>
     </row>
     <row r="133" spans="1:6" x14ac:dyDescent="0.35">
@@ -3484,8 +3505,8 @@
       <c r="B133" t="s">
         <v>165</v>
       </c>
-      <c r="C133" t="s">
-        <v>166</v>
+      <c r="D133" t="s">
+        <v>87</v>
       </c>
       <c r="E133" t="s">
         <v>116</v>
@@ -3499,16 +3520,16 @@
         <v>32</v>
       </c>
       <c r="B134" t="s">
-        <v>149</v>
-      </c>
-      <c r="D134" t="s">
-        <v>68</v>
+        <v>165</v>
+      </c>
+      <c r="C134" t="s">
+        <v>166</v>
       </c>
       <c r="E134" t="s">
         <v>116</v>
       </c>
       <c r="F134" t="s">
-        <v>147</v>
+        <v>163</v>
       </c>
     </row>
     <row r="135" spans="1:6" x14ac:dyDescent="0.35">
@@ -3518,8 +3539,8 @@
       <c r="B135" t="s">
         <v>149</v>
       </c>
-      <c r="C135" t="s">
-        <v>151</v>
+      <c r="D135" t="s">
+        <v>68</v>
       </c>
       <c r="E135" t="s">
         <v>116</v>
@@ -3536,7 +3557,7 @@
         <v>149</v>
       </c>
       <c r="C136" t="s">
-        <v>49</v>
+        <v>151</v>
       </c>
       <c r="E136" t="s">
         <v>116</v>
@@ -3553,7 +3574,7 @@
         <v>149</v>
       </c>
       <c r="C137" t="s">
-        <v>150</v>
+        <v>49</v>
       </c>
       <c r="E137" t="s">
         <v>116</v>
@@ -3570,7 +3591,7 @@
         <v>149</v>
       </c>
       <c r="C138" t="s">
-        <v>50</v>
+        <v>150</v>
       </c>
       <c r="E138" t="s">
         <v>116</v>
@@ -3584,16 +3605,16 @@
         <v>32</v>
       </c>
       <c r="B139" t="s">
-        <v>138</v>
-      </c>
-      <c r="D139" t="s">
-        <v>68</v>
+        <v>149</v>
+      </c>
+      <c r="C139" t="s">
+        <v>50</v>
       </c>
       <c r="E139" t="s">
         <v>116</v>
       </c>
       <c r="F139" t="s">
-        <v>137</v>
+        <v>147</v>
       </c>
     </row>
     <row r="140" spans="1:6" x14ac:dyDescent="0.35">
@@ -3603,14 +3624,14 @@
       <c r="B140" t="s">
         <v>138</v>
       </c>
-      <c r="C140" t="s">
-        <v>148</v>
+      <c r="D140" t="s">
+        <v>68</v>
       </c>
       <c r="E140" t="s">
         <v>116</v>
       </c>
       <c r="F140" t="s">
-        <v>147</v>
+        <v>137</v>
       </c>
     </row>
     <row r="141" spans="1:6" x14ac:dyDescent="0.35">
@@ -3621,13 +3642,13 @@
         <v>138</v>
       </c>
       <c r="C141" t="s">
-        <v>58</v>
+        <v>148</v>
       </c>
       <c r="E141" t="s">
         <v>116</v>
       </c>
       <c r="F141" t="s">
-        <v>137</v>
+        <v>147</v>
       </c>
     </row>
     <row r="142" spans="1:6" x14ac:dyDescent="0.35">
@@ -3638,7 +3659,7 @@
         <v>138</v>
       </c>
       <c r="C142" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E142" t="s">
         <v>116</v>
@@ -3655,13 +3676,13 @@
         <v>138</v>
       </c>
       <c r="C143" t="s">
-        <v>156</v>
+        <v>57</v>
       </c>
       <c r="E143" t="s">
         <v>116</v>
       </c>
       <c r="F143" t="s">
-        <v>158</v>
+        <v>137</v>
       </c>
     </row>
     <row r="144" spans="1:6" x14ac:dyDescent="0.35">
@@ -3672,13 +3693,13 @@
         <v>138</v>
       </c>
       <c r="C144" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="E144" t="s">
         <v>116</v>
       </c>
       <c r="F144" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
     </row>
     <row r="145" spans="1:6" x14ac:dyDescent="0.35">
@@ -3689,13 +3710,13 @@
         <v>138</v>
       </c>
       <c r="C145" t="s">
-        <v>184</v>
+        <v>154</v>
       </c>
       <c r="E145" t="s">
         <v>116</v>
       </c>
       <c r="F145" t="s">
-        <v>183</v>
+        <v>155</v>
       </c>
     </row>
     <row r="146" spans="1:6" x14ac:dyDescent="0.35">
@@ -3706,13 +3727,13 @@
         <v>138</v>
       </c>
       <c r="C146" t="s">
-        <v>157</v>
+        <v>184</v>
       </c>
       <c r="E146" t="s">
         <v>116</v>
       </c>
       <c r="F146" t="s">
-        <v>158</v>
+        <v>183</v>
       </c>
     </row>
     <row r="147" spans="1:6" x14ac:dyDescent="0.35">
@@ -3720,16 +3741,16 @@
         <v>32</v>
       </c>
       <c r="B147" t="s">
-        <v>125</v>
-      </c>
-      <c r="D147" t="s">
-        <v>68</v>
+        <v>138</v>
+      </c>
+      <c r="C147" t="s">
+        <v>157</v>
       </c>
       <c r="E147" t="s">
         <v>116</v>
       </c>
       <c r="F147" t="s">
-        <v>121</v>
+        <v>158</v>
       </c>
     </row>
     <row r="148" spans="1:6" x14ac:dyDescent="0.35">
@@ -3739,8 +3760,8 @@
       <c r="B148" t="s">
         <v>125</v>
       </c>
-      <c r="C148" t="s">
-        <v>127</v>
+      <c r="D148" t="s">
+        <v>68</v>
       </c>
       <c r="E148" t="s">
         <v>116</v>
@@ -3754,16 +3775,16 @@
         <v>32</v>
       </c>
       <c r="B149" t="s">
-        <v>131</v>
-      </c>
-      <c r="D149" t="s">
-        <v>68</v>
+        <v>125</v>
+      </c>
+      <c r="C149" t="s">
+        <v>127</v>
       </c>
       <c r="E149" t="s">
         <v>116</v>
       </c>
       <c r="F149" t="s">
-        <v>130</v>
+        <v>121</v>
       </c>
     </row>
     <row r="150" spans="1:6" x14ac:dyDescent="0.35">
@@ -3773,8 +3794,8 @@
       <c r="B150" t="s">
         <v>131</v>
       </c>
-      <c r="C150" t="s">
-        <v>132</v>
+      <c r="D150" t="s">
+        <v>68</v>
       </c>
       <c r="E150" t="s">
         <v>116</v>
@@ -3791,7 +3812,7 @@
         <v>131</v>
       </c>
       <c r="C151" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="E151" t="s">
         <v>116</v>
@@ -3808,7 +3829,7 @@
         <v>131</v>
       </c>
       <c r="C152" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="E152" t="s">
         <v>116</v>
@@ -3825,7 +3846,7 @@
         <v>131</v>
       </c>
       <c r="C153" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E153" t="s">
         <v>116</v>
@@ -3839,16 +3860,16 @@
         <v>32</v>
       </c>
       <c r="B154" t="s">
-        <v>126</v>
-      </c>
-      <c r="D154" t="s">
-        <v>68</v>
+        <v>131</v>
+      </c>
+      <c r="C154" t="s">
+        <v>135</v>
       </c>
       <c r="E154" t="s">
         <v>116</v>
       </c>
       <c r="F154" t="s">
-        <v>121</v>
+        <v>130</v>
       </c>
     </row>
     <row r="155" spans="1:6" x14ac:dyDescent="0.35">
@@ -3858,8 +3879,8 @@
       <c r="B155" t="s">
         <v>126</v>
       </c>
-      <c r="C155" t="s">
-        <v>128</v>
+      <c r="D155" t="s">
+        <v>68</v>
       </c>
       <c r="E155" t="s">
         <v>116</v>
@@ -3873,16 +3894,16 @@
         <v>32</v>
       </c>
       <c r="B156" t="s">
-        <v>98</v>
-      </c>
-      <c r="D156" t="s">
-        <v>87</v>
+        <v>126</v>
+      </c>
+      <c r="C156" t="s">
+        <v>128</v>
       </c>
       <c r="E156" t="s">
-        <v>14</v>
+        <v>116</v>
       </c>
       <c r="F156" t="s">
-        <v>99</v>
+        <v>121</v>
       </c>
     </row>
     <row r="157" spans="1:6" x14ac:dyDescent="0.35">
@@ -3890,7 +3911,7 @@
         <v>32</v>
       </c>
       <c r="B157" t="s">
-        <v>13</v>
+        <v>98</v>
       </c>
       <c r="D157" t="s">
         <v>87</v>
@@ -3899,7 +3920,7 @@
         <v>14</v>
       </c>
       <c r="F157" t="s">
-        <v>17</v>
+        <v>99</v>
       </c>
     </row>
     <row r="158" spans="1:6" x14ac:dyDescent="0.35">
@@ -3909,17 +3930,14 @@
       <c r="B158" t="s">
         <v>13</v>
       </c>
-      <c r="C158" t="s">
-        <v>10</v>
-      </c>
-      <c r="D158">
-        <v>1</v>
+      <c r="D158" t="s">
+        <v>87</v>
       </c>
       <c r="E158" t="s">
         <v>14</v>
       </c>
       <c r="F158" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="159" spans="1:6" x14ac:dyDescent="0.35">
@@ -3930,7 +3948,7 @@
         <v>13</v>
       </c>
       <c r="C159" t="s">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="D159">
         <v>1</v>
@@ -3939,7 +3957,7 @@
         <v>14</v>
       </c>
       <c r="F159" t="s">
-        <v>23</v>
+        <v>15</v>
       </c>
     </row>
     <row r="160" spans="1:6" x14ac:dyDescent="0.35">
@@ -3950,7 +3968,7 @@
         <v>13</v>
       </c>
       <c r="C160" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D160">
         <v>1</v>
@@ -3959,7 +3977,7 @@
         <v>14</v>
       </c>
       <c r="F160" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
     </row>
     <row r="161" spans="1:6" x14ac:dyDescent="0.35">
@@ -3967,16 +3985,19 @@
         <v>32</v>
       </c>
       <c r="B161" t="s">
-        <v>97</v>
-      </c>
-      <c r="D161" t="s">
-        <v>87</v>
+        <v>13</v>
+      </c>
+      <c r="C161" t="s">
+        <v>18</v>
+      </c>
+      <c r="D161">
+        <v>1</v>
       </c>
       <c r="E161" t="s">
-        <v>54</v>
+        <v>14</v>
       </c>
       <c r="F161" t="s">
-        <v>63</v>
+        <v>17</v>
       </c>
     </row>
     <row r="162" spans="1:6" x14ac:dyDescent="0.35">
@@ -3986,17 +4007,14 @@
       <c r="B162" t="s">
         <v>97</v>
       </c>
-      <c r="C162" s="2" t="s">
-        <v>216</v>
-      </c>
-      <c r="D162">
-        <v>1</v>
+      <c r="D162" t="s">
+        <v>87</v>
       </c>
       <c r="E162" t="s">
         <v>54</v>
       </c>
-      <c r="F162" s="2" t="s">
-        <v>193</v>
+      <c r="F162" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="163" spans="1:6" x14ac:dyDescent="0.35">
@@ -4007,13 +4025,16 @@
         <v>97</v>
       </c>
       <c r="C163" t="s">
-        <v>191</v>
+        <v>216</v>
+      </c>
+      <c r="D163">
+        <v>1</v>
       </c>
       <c r="E163" t="s">
-        <v>24</v>
+        <v>54</v>
       </c>
       <c r="F163" t="s">
-        <v>89</v>
+        <v>193</v>
       </c>
     </row>
     <row r="164" spans="1:6" x14ac:dyDescent="0.35">
@@ -4021,16 +4042,16 @@
         <v>32</v>
       </c>
       <c r="B164" t="s">
-        <v>33</v>
-      </c>
-      <c r="D164" t="s">
-        <v>87</v>
+        <v>97</v>
+      </c>
+      <c r="C164" t="s">
+        <v>191</v>
       </c>
       <c r="E164" t="s">
-        <v>54</v>
+        <v>24</v>
       </c>
       <c r="F164" t="s">
-        <v>56</v>
+        <v>89</v>
       </c>
     </row>
     <row r="165" spans="1:6" x14ac:dyDescent="0.35">
@@ -4040,17 +4061,14 @@
       <c r="B165" t="s">
         <v>33</v>
       </c>
-      <c r="C165" s="2" t="s">
-        <v>215</v>
-      </c>
-      <c r="D165">
-        <v>1</v>
+      <c r="D165" t="s">
+        <v>87</v>
       </c>
       <c r="E165" t="s">
         <v>54</v>
       </c>
       <c r="F165" t="s">
-        <v>193</v>
+        <v>56</v>
       </c>
     </row>
     <row r="166" spans="1:6" x14ac:dyDescent="0.35">
@@ -4060,8 +4078,8 @@
       <c r="B166" t="s">
         <v>33</v>
       </c>
-      <c r="C166" s="1" t="s">
-        <v>39</v>
+      <c r="C166" t="s">
+        <v>215</v>
       </c>
       <c r="D166">
         <v>1</v>
@@ -4070,7 +4088,7 @@
         <v>54</v>
       </c>
       <c r="F166" t="s">
-        <v>63</v>
+        <v>193</v>
       </c>
     </row>
     <row r="167" spans="1:6" x14ac:dyDescent="0.35">
@@ -4090,7 +4108,7 @@
         <v>54</v>
       </c>
       <c r="F167" t="s">
-        <v>55</v>
+        <v>63</v>
       </c>
     </row>
     <row r="168" spans="1:6" x14ac:dyDescent="0.35">
@@ -4101,13 +4119,16 @@
         <v>33</v>
       </c>
       <c r="C168" s="1" t="s">
-        <v>57</v>
+        <v>39</v>
+      </c>
+      <c r="D168">
+        <v>1</v>
       </c>
       <c r="E168" t="s">
         <v>54</v>
       </c>
       <c r="F168" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="169" spans="1:6" x14ac:dyDescent="0.35">
@@ -4118,13 +4139,13 @@
         <v>33</v>
       </c>
       <c r="C169" s="1" t="s">
-        <v>195</v>
+        <v>57</v>
       </c>
       <c r="E169" t="s">
         <v>54</v>
       </c>
       <c r="F169" t="s">
-        <v>193</v>
+        <v>56</v>
       </c>
     </row>
     <row r="170" spans="1:6" x14ac:dyDescent="0.35">
@@ -4132,17 +4153,16 @@
         <v>32</v>
       </c>
       <c r="B170" t="s">
-        <v>182</v>
-      </c>
-      <c r="C170" s="1"/>
-      <c r="D170" t="s">
-        <v>68</v>
+        <v>33</v>
+      </c>
+      <c r="C170" s="1" t="s">
+        <v>195</v>
       </c>
       <c r="E170" t="s">
-        <v>116</v>
+        <v>54</v>
       </c>
       <c r="F170" t="s">
-        <v>183</v>
+        <v>193</v>
       </c>
     </row>
     <row r="171" spans="1:6" x14ac:dyDescent="0.35">
@@ -4150,16 +4170,70 @@
         <v>32</v>
       </c>
       <c r="B171" t="s">
+        <v>182</v>
+      </c>
+      <c r="C171" s="1"/>
+      <c r="D171" t="s">
+        <v>68</v>
+      </c>
+      <c r="E171" t="s">
+        <v>116</v>
+      </c>
+      <c r="F171" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="172" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A172" t="s">
+        <v>32</v>
+      </c>
+      <c r="B172" t="s">
         <v>88</v>
       </c>
-      <c r="D171" t="s">
+      <c r="D172" t="s">
         <v>65</v>
       </c>
-      <c r="E171" t="s">
+      <c r="E172" t="s">
         <v>24</v>
       </c>
-      <c r="F171" t="s">
+      <c r="F172" t="s">
         <v>89</v>
+      </c>
+    </row>
+    <row r="173" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A173" t="s">
+        <v>32</v>
+      </c>
+      <c r="B173" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="C173" s="2"/>
+      <c r="D173" t="s">
+        <v>65</v>
+      </c>
+      <c r="E173" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="F173" s="2" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="174" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A174" t="s">
+        <v>32</v>
+      </c>
+      <c r="B174" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="C174" s="2"/>
+      <c r="D174" t="s">
+        <v>87</v>
+      </c>
+      <c r="E174" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="F174" s="2" t="s">
+        <v>229</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
[PowerPoint] (ThemeColorScheme) Add snippet (#1077)
* [PowerPoint] (ThemeColorScheme) Add snippet

* Fix failing test
</commit_message>
<xml_diff>
--- a/snippet-extractor-metadata/powerpoint.xlsx
+++ b/snippet-extractor-metadata/powerpoint.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A2CA723-45CB-4135-8A1A-0329A73196F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D0F7BFA-D1AA-43BE-B4C8-CBE72F79E65D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25180" windowHeight="16140" xr2:uid="{CB5595D7-4492-4192-A1C1-2583BA1957AA}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="856" uniqueCount="223">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="871" uniqueCount="230">
   <si>
     <t>Class</t>
   </si>
@@ -689,6 +689,27 @@
   </si>
   <si>
     <t>getShapeById</t>
+  </si>
+  <si>
+    <t>themeColorScheme</t>
+  </si>
+  <si>
+    <t>getThemeColors</t>
+  </si>
+  <si>
+    <t>powerpoint-slide-management-get-set-theme-color-scheme</t>
+  </si>
+  <si>
+    <t>ThemeColor</t>
+  </si>
+  <si>
+    <t>setThemeColors</t>
+  </si>
+  <si>
+    <t>ThemeColorScheme</t>
+  </si>
+  <si>
+    <t>resetThemeColors</t>
   </si>
 </sst>
 </file>
@@ -769,10 +790,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{78C585A5-D505-49C6-9CA1-8E6558948317}" name="Snippets" displayName="Snippets" ref="A1:F171" totalsRowShown="0" headerRowDxfId="4">
-  <autoFilter ref="A1:F171" xr:uid="{EAC65D03-FDD2-4352-A5F3-1CDEDE6251B2}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F167">
-    <sortCondition ref="B1:B167"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{78C585A5-D505-49C6-9CA1-8E6558948317}" name="Snippets" displayName="Snippets" ref="A1:F174" totalsRowShown="0" headerRowDxfId="4">
+  <autoFilter ref="A1:F174" xr:uid="{EAC65D03-FDD2-4352-A5F3-1CDEDE6251B2}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F168">
+    <sortCondition ref="B1:B168"/>
   </sortState>
   <tableColumns count="6">
     <tableColumn id="6" xr3:uid="{408888B8-C1DD-4B51-B1EB-5663F091D142}" name="Package"/>
@@ -1083,7 +1104,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{809930CD-A227-47DC-AAA4-BB816AEDEB59}">
-  <dimension ref="A1:F171"/>
+  <dimension ref="A1:F174"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="11.453125" bestFit="1" customWidth="1"/>
@@ -2006,16 +2027,16 @@
       <c r="B51" t="s">
         <v>45</v>
       </c>
-      <c r="C51" s="2" t="s">
+      <c r="C51" t="s">
         <v>217</v>
       </c>
       <c r="D51">
         <v>1</v>
       </c>
-      <c r="E51" s="2" t="s">
+      <c r="E51" t="s">
         <v>54</v>
       </c>
-      <c r="F51" s="2" t="s">
+      <c r="F51" t="s">
         <v>193</v>
       </c>
     </row>
@@ -2802,16 +2823,16 @@
       <c r="B95" t="s">
         <v>90</v>
       </c>
-      <c r="C95" s="2" t="s">
+      <c r="C95" t="s">
         <v>220</v>
       </c>
       <c r="D95">
         <v>1</v>
       </c>
-      <c r="E95" s="2" t="s">
+      <c r="E95" t="s">
         <v>221</v>
       </c>
-      <c r="F95" s="2" t="s">
+      <c r="F95" t="s">
         <v>222</v>
       </c>
     </row>
@@ -3005,16 +3026,16 @@
         <v>32</v>
       </c>
       <c r="B106" t="s">
-        <v>9</v>
-      </c>
-      <c r="D106" t="s">
-        <v>87</v>
-      </c>
-      <c r="E106" t="s">
-        <v>11</v>
-      </c>
-      <c r="F106" t="s">
-        <v>12</v>
+        <v>19</v>
+      </c>
+      <c r="C106" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="E106" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="F106" s="2" t="s">
+        <v>224</v>
       </c>
     </row>
     <row r="107" spans="1:6" x14ac:dyDescent="0.35">
@@ -3024,11 +3045,8 @@
       <c r="B107" t="s">
         <v>9</v>
       </c>
-      <c r="C107" t="s">
-        <v>10</v>
-      </c>
-      <c r="D107">
-        <v>1</v>
+      <c r="D107" t="s">
+        <v>87</v>
       </c>
       <c r="E107" t="s">
         <v>11</v>
@@ -3045,16 +3063,16 @@
         <v>9</v>
       </c>
       <c r="C108" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="D108">
         <v>1</v>
       </c>
       <c r="E108" t="s">
-        <v>40</v>
+        <v>11</v>
       </c>
       <c r="F108" t="s">
-        <v>37</v>
+        <v>12</v>
       </c>
     </row>
     <row r="109" spans="1:6" x14ac:dyDescent="0.35">
@@ -3062,16 +3080,19 @@
         <v>32</v>
       </c>
       <c r="B109" t="s">
-        <v>185</v>
-      </c>
-      <c r="D109" t="s">
-        <v>68</v>
+        <v>9</v>
+      </c>
+      <c r="C109" t="s">
+        <v>16</v>
+      </c>
+      <c r="D109">
+        <v>1</v>
       </c>
       <c r="E109" t="s">
-        <v>105</v>
+        <v>40</v>
       </c>
       <c r="F109" t="s">
-        <v>107</v>
+        <v>37</v>
       </c>
     </row>
     <row r="110" spans="1:6" x14ac:dyDescent="0.35">
@@ -3079,16 +3100,16 @@
         <v>32</v>
       </c>
       <c r="B110" t="s">
-        <v>75</v>
+        <v>185</v>
       </c>
       <c r="D110" t="s">
-        <v>87</v>
+        <v>68</v>
       </c>
       <c r="E110" t="s">
-        <v>11</v>
+        <v>105</v>
       </c>
       <c r="F110" t="s">
-        <v>71</v>
+        <v>107</v>
       </c>
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.35">
@@ -3098,8 +3119,8 @@
       <c r="B111" t="s">
         <v>75</v>
       </c>
-      <c r="C111" t="s">
-        <v>74</v>
+      <c r="D111" t="s">
+        <v>87</v>
       </c>
       <c r="E111" t="s">
         <v>11</v>
@@ -3113,10 +3134,10 @@
         <v>32</v>
       </c>
       <c r="B112" t="s">
-        <v>72</v>
-      </c>
-      <c r="D112" t="s">
-        <v>87</v>
+        <v>75</v>
+      </c>
+      <c r="C112" t="s">
+        <v>74</v>
       </c>
       <c r="E112" t="s">
         <v>11</v>
@@ -3132,11 +3153,8 @@
       <c r="B113" t="s">
         <v>72</v>
       </c>
-      <c r="C113" t="s">
-        <v>70</v>
-      </c>
-      <c r="D113">
-        <v>2</v>
+      <c r="D113" t="s">
+        <v>87</v>
       </c>
       <c r="E113" t="s">
         <v>11</v>
@@ -3150,16 +3168,19 @@
         <v>32</v>
       </c>
       <c r="B114" t="s">
-        <v>186</v>
-      </c>
-      <c r="D114" t="s">
-        <v>65</v>
+        <v>72</v>
+      </c>
+      <c r="C114" t="s">
+        <v>70</v>
+      </c>
+      <c r="D114">
+        <v>2</v>
       </c>
       <c r="E114" t="s">
-        <v>85</v>
+        <v>11</v>
       </c>
       <c r="F114" t="s">
-        <v>79</v>
+        <v>71</v>
       </c>
     </row>
     <row r="115" spans="1:6" x14ac:dyDescent="0.35">
@@ -3167,16 +3188,16 @@
         <v>32</v>
       </c>
       <c r="B115" t="s">
-        <v>73</v>
+        <v>186</v>
       </c>
       <c r="D115" t="s">
-        <v>87</v>
+        <v>65</v>
       </c>
       <c r="E115" t="s">
-        <v>11</v>
+        <v>85</v>
       </c>
       <c r="F115" t="s">
-        <v>71</v>
+        <v>79</v>
       </c>
     </row>
     <row r="116" spans="1:6" x14ac:dyDescent="0.35">
@@ -3186,8 +3207,8 @@
       <c r="B116" t="s">
         <v>73</v>
       </c>
-      <c r="C116" t="s">
-        <v>74</v>
+      <c r="D116" t="s">
+        <v>87</v>
       </c>
       <c r="E116" t="s">
         <v>11</v>
@@ -3201,10 +3222,10 @@
         <v>32</v>
       </c>
       <c r="B117" t="s">
-        <v>69</v>
-      </c>
-      <c r="D117" t="s">
-        <v>87</v>
+        <v>73</v>
+      </c>
+      <c r="C117" t="s">
+        <v>74</v>
       </c>
       <c r="E117" t="s">
         <v>11</v>
@@ -3220,11 +3241,8 @@
       <c r="B118" t="s">
         <v>69</v>
       </c>
-      <c r="C118" t="s">
-        <v>70</v>
-      </c>
-      <c r="D118">
-        <v>2</v>
+      <c r="D118" t="s">
+        <v>87</v>
       </c>
       <c r="E118" t="s">
         <v>11</v>
@@ -3238,16 +3256,19 @@
         <v>32</v>
       </c>
       <c r="B119" t="s">
-        <v>92</v>
-      </c>
-      <c r="D119" t="s">
-        <v>87</v>
+        <v>69</v>
+      </c>
+      <c r="C119" t="s">
+        <v>70</v>
+      </c>
+      <c r="D119">
+        <v>2</v>
       </c>
       <c r="E119" t="s">
-        <v>53</v>
+        <v>11</v>
       </c>
       <c r="F119" t="s">
-        <v>47</v>
+        <v>71</v>
       </c>
     </row>
     <row r="120" spans="1:6" x14ac:dyDescent="0.35">
@@ -3257,17 +3278,14 @@
       <c r="B120" t="s">
         <v>92</v>
       </c>
-      <c r="C120" s="2" t="s">
-        <v>220</v>
-      </c>
-      <c r="D120">
-        <v>1</v>
-      </c>
-      <c r="E120" s="2" t="s">
-        <v>219</v>
-      </c>
-      <c r="F120" s="2" t="s">
-        <v>218</v>
+      <c r="D120" t="s">
+        <v>87</v>
+      </c>
+      <c r="E120" t="s">
+        <v>53</v>
+      </c>
+      <c r="F120" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="121" spans="1:6" x14ac:dyDescent="0.35">
@@ -3275,16 +3293,19 @@
         <v>32</v>
       </c>
       <c r="B121" t="s">
-        <v>162</v>
-      </c>
-      <c r="D121" t="s">
-        <v>87</v>
+        <v>92</v>
+      </c>
+      <c r="C121" t="s">
+        <v>220</v>
+      </c>
+      <c r="D121">
+        <v>1</v>
       </c>
       <c r="E121" t="s">
-        <v>116</v>
+        <v>219</v>
       </c>
       <c r="F121" t="s">
-        <v>163</v>
+        <v>218</v>
       </c>
     </row>
     <row r="122" spans="1:6" x14ac:dyDescent="0.35">
@@ -3294,11 +3315,8 @@
       <c r="B122" t="s">
         <v>162</v>
       </c>
-      <c r="C122" t="s">
-        <v>164</v>
-      </c>
-      <c r="D122">
-        <v>1</v>
+      <c r="D122" t="s">
+        <v>87</v>
       </c>
       <c r="E122" t="s">
         <v>116</v>
@@ -3312,16 +3330,19 @@
         <v>32</v>
       </c>
       <c r="B123" t="s">
-        <v>118</v>
-      </c>
-      <c r="D123" t="s">
-        <v>68</v>
+        <v>162</v>
+      </c>
+      <c r="C123" t="s">
+        <v>164</v>
+      </c>
+      <c r="D123">
+        <v>1</v>
       </c>
       <c r="E123" t="s">
         <v>116</v>
       </c>
       <c r="F123" t="s">
-        <v>119</v>
+        <v>163</v>
       </c>
     </row>
     <row r="124" spans="1:6" x14ac:dyDescent="0.35">
@@ -3331,14 +3352,14 @@
       <c r="B124" t="s">
         <v>118</v>
       </c>
-      <c r="C124" t="s">
-        <v>124</v>
+      <c r="D124" t="s">
+        <v>68</v>
       </c>
       <c r="E124" t="s">
         <v>116</v>
       </c>
       <c r="F124" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
     <row r="125" spans="1:6" x14ac:dyDescent="0.35">
@@ -3349,13 +3370,13 @@
         <v>118</v>
       </c>
       <c r="C125" t="s">
-        <v>52</v>
+        <v>124</v>
       </c>
       <c r="E125" t="s">
         <v>116</v>
       </c>
       <c r="F125" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
     </row>
     <row r="126" spans="1:6" x14ac:dyDescent="0.35">
@@ -3366,13 +3387,13 @@
         <v>118</v>
       </c>
       <c r="C126" t="s">
-        <v>129</v>
+        <v>52</v>
       </c>
       <c r="E126" t="s">
         <v>116</v>
       </c>
       <c r="F126" t="s">
-        <v>130</v>
+        <v>119</v>
       </c>
     </row>
     <row r="127" spans="1:6" x14ac:dyDescent="0.35">
@@ -3383,13 +3404,13 @@
         <v>118</v>
       </c>
       <c r="C127" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="E127" t="s">
         <v>116</v>
       </c>
       <c r="F127" t="s">
-        <v>121</v>
+        <v>130</v>
       </c>
     </row>
     <row r="128" spans="1:6" x14ac:dyDescent="0.35">
@@ -3400,13 +3421,13 @@
         <v>118</v>
       </c>
       <c r="C128" t="s">
-        <v>136</v>
+        <v>123</v>
       </c>
       <c r="E128" t="s">
         <v>116</v>
       </c>
       <c r="F128" t="s">
-        <v>137</v>
+        <v>121</v>
       </c>
     </row>
     <row r="129" spans="1:6" x14ac:dyDescent="0.35">
@@ -3417,13 +3438,13 @@
         <v>118</v>
       </c>
       <c r="C129" t="s">
-        <v>146</v>
+        <v>136</v>
       </c>
       <c r="E129" t="s">
         <v>116</v>
       </c>
       <c r="F129" t="s">
-        <v>147</v>
+        <v>137</v>
       </c>
     </row>
     <row r="130" spans="1:6" x14ac:dyDescent="0.35">
@@ -3434,13 +3455,13 @@
         <v>118</v>
       </c>
       <c r="C130" t="s">
-        <v>120</v>
+        <v>146</v>
       </c>
       <c r="E130" t="s">
         <v>116</v>
       </c>
       <c r="F130" t="s">
-        <v>122</v>
+        <v>147</v>
       </c>
     </row>
     <row r="131" spans="1:6" x14ac:dyDescent="0.35">
@@ -3451,13 +3472,13 @@
         <v>118</v>
       </c>
       <c r="C131" t="s">
-        <v>51</v>
+        <v>120</v>
       </c>
       <c r="E131" t="s">
         <v>116</v>
       </c>
       <c r="F131" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
     </row>
     <row r="132" spans="1:6" x14ac:dyDescent="0.35">
@@ -3465,16 +3486,16 @@
         <v>32</v>
       </c>
       <c r="B132" t="s">
-        <v>165</v>
-      </c>
-      <c r="D132" t="s">
-        <v>87</v>
+        <v>118</v>
+      </c>
+      <c r="C132" t="s">
+        <v>51</v>
       </c>
       <c r="E132" t="s">
         <v>116</v>
       </c>
       <c r="F132" t="s">
-        <v>163</v>
+        <v>119</v>
       </c>
     </row>
     <row r="133" spans="1:6" x14ac:dyDescent="0.35">
@@ -3484,8 +3505,8 @@
       <c r="B133" t="s">
         <v>165</v>
       </c>
-      <c r="C133" t="s">
-        <v>166</v>
+      <c r="D133" t="s">
+        <v>87</v>
       </c>
       <c r="E133" t="s">
         <v>116</v>
@@ -3499,16 +3520,16 @@
         <v>32</v>
       </c>
       <c r="B134" t="s">
-        <v>149</v>
-      </c>
-      <c r="D134" t="s">
-        <v>68</v>
+        <v>165</v>
+      </c>
+      <c r="C134" t="s">
+        <v>166</v>
       </c>
       <c r="E134" t="s">
         <v>116</v>
       </c>
       <c r="F134" t="s">
-        <v>147</v>
+        <v>163</v>
       </c>
     </row>
     <row r="135" spans="1:6" x14ac:dyDescent="0.35">
@@ -3518,8 +3539,8 @@
       <c r="B135" t="s">
         <v>149</v>
       </c>
-      <c r="C135" t="s">
-        <v>151</v>
+      <c r="D135" t="s">
+        <v>68</v>
       </c>
       <c r="E135" t="s">
         <v>116</v>
@@ -3536,7 +3557,7 @@
         <v>149</v>
       </c>
       <c r="C136" t="s">
-        <v>49</v>
+        <v>151</v>
       </c>
       <c r="E136" t="s">
         <v>116</v>
@@ -3553,7 +3574,7 @@
         <v>149</v>
       </c>
       <c r="C137" t="s">
-        <v>150</v>
+        <v>49</v>
       </c>
       <c r="E137" t="s">
         <v>116</v>
@@ -3570,7 +3591,7 @@
         <v>149</v>
       </c>
       <c r="C138" t="s">
-        <v>50</v>
+        <v>150</v>
       </c>
       <c r="E138" t="s">
         <v>116</v>
@@ -3584,16 +3605,16 @@
         <v>32</v>
       </c>
       <c r="B139" t="s">
-        <v>138</v>
-      </c>
-      <c r="D139" t="s">
-        <v>68</v>
+        <v>149</v>
+      </c>
+      <c r="C139" t="s">
+        <v>50</v>
       </c>
       <c r="E139" t="s">
         <v>116</v>
       </c>
       <c r="F139" t="s">
-        <v>137</v>
+        <v>147</v>
       </c>
     </row>
     <row r="140" spans="1:6" x14ac:dyDescent="0.35">
@@ -3603,14 +3624,14 @@
       <c r="B140" t="s">
         <v>138</v>
       </c>
-      <c r="C140" t="s">
-        <v>148</v>
+      <c r="D140" t="s">
+        <v>68</v>
       </c>
       <c r="E140" t="s">
         <v>116</v>
       </c>
       <c r="F140" t="s">
-        <v>147</v>
+        <v>137</v>
       </c>
     </row>
     <row r="141" spans="1:6" x14ac:dyDescent="0.35">
@@ -3621,13 +3642,13 @@
         <v>138</v>
       </c>
       <c r="C141" t="s">
-        <v>58</v>
+        <v>148</v>
       </c>
       <c r="E141" t="s">
         <v>116</v>
       </c>
       <c r="F141" t="s">
-        <v>137</v>
+        <v>147</v>
       </c>
     </row>
     <row r="142" spans="1:6" x14ac:dyDescent="0.35">
@@ -3638,7 +3659,7 @@
         <v>138</v>
       </c>
       <c r="C142" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E142" t="s">
         <v>116</v>
@@ -3655,13 +3676,13 @@
         <v>138</v>
       </c>
       <c r="C143" t="s">
-        <v>156</v>
+        <v>57</v>
       </c>
       <c r="E143" t="s">
         <v>116</v>
       </c>
       <c r="F143" t="s">
-        <v>158</v>
+        <v>137</v>
       </c>
     </row>
     <row r="144" spans="1:6" x14ac:dyDescent="0.35">
@@ -3672,13 +3693,13 @@
         <v>138</v>
       </c>
       <c r="C144" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="E144" t="s">
         <v>116</v>
       </c>
       <c r="F144" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
     </row>
     <row r="145" spans="1:6" x14ac:dyDescent="0.35">
@@ -3689,13 +3710,13 @@
         <v>138</v>
       </c>
       <c r="C145" t="s">
-        <v>184</v>
+        <v>154</v>
       </c>
       <c r="E145" t="s">
         <v>116</v>
       </c>
       <c r="F145" t="s">
-        <v>183</v>
+        <v>155</v>
       </c>
     </row>
     <row r="146" spans="1:6" x14ac:dyDescent="0.35">
@@ -3706,13 +3727,13 @@
         <v>138</v>
       </c>
       <c r="C146" t="s">
-        <v>157</v>
+        <v>184</v>
       </c>
       <c r="E146" t="s">
         <v>116</v>
       </c>
       <c r="F146" t="s">
-        <v>158</v>
+        <v>183</v>
       </c>
     </row>
     <row r="147" spans="1:6" x14ac:dyDescent="0.35">
@@ -3720,16 +3741,16 @@
         <v>32</v>
       </c>
       <c r="B147" t="s">
-        <v>125</v>
-      </c>
-      <c r="D147" t="s">
-        <v>68</v>
+        <v>138</v>
+      </c>
+      <c r="C147" t="s">
+        <v>157</v>
       </c>
       <c r="E147" t="s">
         <v>116</v>
       </c>
       <c r="F147" t="s">
-        <v>121</v>
+        <v>158</v>
       </c>
     </row>
     <row r="148" spans="1:6" x14ac:dyDescent="0.35">
@@ -3739,8 +3760,8 @@
       <c r="B148" t="s">
         <v>125</v>
       </c>
-      <c r="C148" t="s">
-        <v>127</v>
+      <c r="D148" t="s">
+        <v>68</v>
       </c>
       <c r="E148" t="s">
         <v>116</v>
@@ -3754,16 +3775,16 @@
         <v>32</v>
       </c>
       <c r="B149" t="s">
-        <v>131</v>
-      </c>
-      <c r="D149" t="s">
-        <v>68</v>
+        <v>125</v>
+      </c>
+      <c r="C149" t="s">
+        <v>127</v>
       </c>
       <c r="E149" t="s">
         <v>116</v>
       </c>
       <c r="F149" t="s">
-        <v>130</v>
+        <v>121</v>
       </c>
     </row>
     <row r="150" spans="1:6" x14ac:dyDescent="0.35">
@@ -3773,8 +3794,8 @@
       <c r="B150" t="s">
         <v>131</v>
       </c>
-      <c r="C150" t="s">
-        <v>132</v>
+      <c r="D150" t="s">
+        <v>68</v>
       </c>
       <c r="E150" t="s">
         <v>116</v>
@@ -3791,7 +3812,7 @@
         <v>131</v>
       </c>
       <c r="C151" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="E151" t="s">
         <v>116</v>
@@ -3808,7 +3829,7 @@
         <v>131</v>
       </c>
       <c r="C152" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="E152" t="s">
         <v>116</v>
@@ -3825,7 +3846,7 @@
         <v>131</v>
       </c>
       <c r="C153" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E153" t="s">
         <v>116</v>
@@ -3839,16 +3860,16 @@
         <v>32</v>
       </c>
       <c r="B154" t="s">
-        <v>126</v>
-      </c>
-      <c r="D154" t="s">
-        <v>68</v>
+        <v>131</v>
+      </c>
+      <c r="C154" t="s">
+        <v>135</v>
       </c>
       <c r="E154" t="s">
         <v>116</v>
       </c>
       <c r="F154" t="s">
-        <v>121</v>
+        <v>130</v>
       </c>
     </row>
     <row r="155" spans="1:6" x14ac:dyDescent="0.35">
@@ -3858,8 +3879,8 @@
       <c r="B155" t="s">
         <v>126</v>
       </c>
-      <c r="C155" t="s">
-        <v>128</v>
+      <c r="D155" t="s">
+        <v>68</v>
       </c>
       <c r="E155" t="s">
         <v>116</v>
@@ -3873,16 +3894,16 @@
         <v>32</v>
       </c>
       <c r="B156" t="s">
-        <v>98</v>
-      </c>
-      <c r="D156" t="s">
-        <v>87</v>
+        <v>126</v>
+      </c>
+      <c r="C156" t="s">
+        <v>128</v>
       </c>
       <c r="E156" t="s">
-        <v>14</v>
+        <v>116</v>
       </c>
       <c r="F156" t="s">
-        <v>99</v>
+        <v>121</v>
       </c>
     </row>
     <row r="157" spans="1:6" x14ac:dyDescent="0.35">
@@ -3890,7 +3911,7 @@
         <v>32</v>
       </c>
       <c r="B157" t="s">
-        <v>13</v>
+        <v>98</v>
       </c>
       <c r="D157" t="s">
         <v>87</v>
@@ -3899,7 +3920,7 @@
         <v>14</v>
       </c>
       <c r="F157" t="s">
-        <v>17</v>
+        <v>99</v>
       </c>
     </row>
     <row r="158" spans="1:6" x14ac:dyDescent="0.35">
@@ -3909,17 +3930,14 @@
       <c r="B158" t="s">
         <v>13</v>
       </c>
-      <c r="C158" t="s">
-        <v>10</v>
-      </c>
-      <c r="D158">
-        <v>1</v>
+      <c r="D158" t="s">
+        <v>87</v>
       </c>
       <c r="E158" t="s">
         <v>14</v>
       </c>
       <c r="F158" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="159" spans="1:6" x14ac:dyDescent="0.35">
@@ -3930,7 +3948,7 @@
         <v>13</v>
       </c>
       <c r="C159" t="s">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="D159">
         <v>1</v>
@@ -3939,7 +3957,7 @@
         <v>14</v>
       </c>
       <c r="F159" t="s">
-        <v>23</v>
+        <v>15</v>
       </c>
     </row>
     <row r="160" spans="1:6" x14ac:dyDescent="0.35">
@@ -3950,7 +3968,7 @@
         <v>13</v>
       </c>
       <c r="C160" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D160">
         <v>1</v>
@@ -3959,7 +3977,7 @@
         <v>14</v>
       </c>
       <c r="F160" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
     </row>
     <row r="161" spans="1:6" x14ac:dyDescent="0.35">
@@ -3967,16 +3985,19 @@
         <v>32</v>
       </c>
       <c r="B161" t="s">
-        <v>97</v>
-      </c>
-      <c r="D161" t="s">
-        <v>87</v>
+        <v>13</v>
+      </c>
+      <c r="C161" t="s">
+        <v>18</v>
+      </c>
+      <c r="D161">
+        <v>1</v>
       </c>
       <c r="E161" t="s">
-        <v>54</v>
+        <v>14</v>
       </c>
       <c r="F161" t="s">
-        <v>63</v>
+        <v>17</v>
       </c>
     </row>
     <row r="162" spans="1:6" x14ac:dyDescent="0.35">
@@ -3986,17 +4007,14 @@
       <c r="B162" t="s">
         <v>97</v>
       </c>
-      <c r="C162" s="2" t="s">
-        <v>216</v>
-      </c>
-      <c r="D162">
-        <v>1</v>
+      <c r="D162" t="s">
+        <v>87</v>
       </c>
       <c r="E162" t="s">
         <v>54</v>
       </c>
-      <c r="F162" s="2" t="s">
-        <v>193</v>
+      <c r="F162" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="163" spans="1:6" x14ac:dyDescent="0.35">
@@ -4007,13 +4025,16 @@
         <v>97</v>
       </c>
       <c r="C163" t="s">
-        <v>191</v>
+        <v>216</v>
+      </c>
+      <c r="D163">
+        <v>1</v>
       </c>
       <c r="E163" t="s">
-        <v>24</v>
+        <v>54</v>
       </c>
       <c r="F163" t="s">
-        <v>89</v>
+        <v>193</v>
       </c>
     </row>
     <row r="164" spans="1:6" x14ac:dyDescent="0.35">
@@ -4021,16 +4042,16 @@
         <v>32</v>
       </c>
       <c r="B164" t="s">
-        <v>33</v>
-      </c>
-      <c r="D164" t="s">
-        <v>87</v>
+        <v>97</v>
+      </c>
+      <c r="C164" t="s">
+        <v>191</v>
       </c>
       <c r="E164" t="s">
-        <v>54</v>
+        <v>24</v>
       </c>
       <c r="F164" t="s">
-        <v>56</v>
+        <v>89</v>
       </c>
     </row>
     <row r="165" spans="1:6" x14ac:dyDescent="0.35">
@@ -4040,17 +4061,14 @@
       <c r="B165" t="s">
         <v>33</v>
       </c>
-      <c r="C165" s="2" t="s">
-        <v>215</v>
-      </c>
-      <c r="D165">
-        <v>1</v>
+      <c r="D165" t="s">
+        <v>87</v>
       </c>
       <c r="E165" t="s">
         <v>54</v>
       </c>
       <c r="F165" t="s">
-        <v>193</v>
+        <v>56</v>
       </c>
     </row>
     <row r="166" spans="1:6" x14ac:dyDescent="0.35">
@@ -4060,8 +4078,8 @@
       <c r="B166" t="s">
         <v>33</v>
       </c>
-      <c r="C166" s="1" t="s">
-        <v>39</v>
+      <c r="C166" t="s">
+        <v>215</v>
       </c>
       <c r="D166">
         <v>1</v>
@@ -4070,7 +4088,7 @@
         <v>54</v>
       </c>
       <c r="F166" t="s">
-        <v>63</v>
+        <v>193</v>
       </c>
     </row>
     <row r="167" spans="1:6" x14ac:dyDescent="0.35">
@@ -4090,7 +4108,7 @@
         <v>54</v>
       </c>
       <c r="F167" t="s">
-        <v>55</v>
+        <v>63</v>
       </c>
     </row>
     <row r="168" spans="1:6" x14ac:dyDescent="0.35">
@@ -4101,13 +4119,16 @@
         <v>33</v>
       </c>
       <c r="C168" s="1" t="s">
-        <v>57</v>
+        <v>39</v>
+      </c>
+      <c r="D168">
+        <v>1</v>
       </c>
       <c r="E168" t="s">
         <v>54</v>
       </c>
       <c r="F168" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="169" spans="1:6" x14ac:dyDescent="0.35">
@@ -4118,13 +4139,13 @@
         <v>33</v>
       </c>
       <c r="C169" s="1" t="s">
-        <v>195</v>
+        <v>57</v>
       </c>
       <c r="E169" t="s">
         <v>54</v>
       </c>
       <c r="F169" t="s">
-        <v>193</v>
+        <v>56</v>
       </c>
     </row>
     <row r="170" spans="1:6" x14ac:dyDescent="0.35">
@@ -4132,17 +4153,16 @@
         <v>32</v>
       </c>
       <c r="B170" t="s">
-        <v>182</v>
-      </c>
-      <c r="C170" s="1"/>
-      <c r="D170" t="s">
-        <v>68</v>
+        <v>33</v>
+      </c>
+      <c r="C170" s="1" t="s">
+        <v>195</v>
       </c>
       <c r="E170" t="s">
-        <v>116</v>
+        <v>54</v>
       </c>
       <c r="F170" t="s">
-        <v>183</v>
+        <v>193</v>
       </c>
     </row>
     <row r="171" spans="1:6" x14ac:dyDescent="0.35">
@@ -4150,16 +4170,70 @@
         <v>32</v>
       </c>
       <c r="B171" t="s">
+        <v>182</v>
+      </c>
+      <c r="C171" s="1"/>
+      <c r="D171" t="s">
+        <v>68</v>
+      </c>
+      <c r="E171" t="s">
+        <v>116</v>
+      </c>
+      <c r="F171" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="172" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A172" t="s">
+        <v>32</v>
+      </c>
+      <c r="B172" t="s">
         <v>88</v>
       </c>
-      <c r="D171" t="s">
+      <c r="D172" t="s">
         <v>65</v>
       </c>
-      <c r="E171" t="s">
+      <c r="E172" t="s">
         <v>24</v>
       </c>
-      <c r="F171" t="s">
+      <c r="F172" t="s">
         <v>89</v>
+      </c>
+    </row>
+    <row r="173" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A173" t="s">
+        <v>32</v>
+      </c>
+      <c r="B173" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="C173" s="2"/>
+      <c r="D173" t="s">
+        <v>65</v>
+      </c>
+      <c r="E173" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="F173" s="2" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="174" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A174" t="s">
+        <v>32</v>
+      </c>
+      <c r="B174" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="C174" s="2"/>
+      <c r="D174" t="s">
+        <v>87</v>
+      </c>
+      <c r="E174" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="F174" s="2" t="s">
+        <v>229</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
[PowerPoint] (Slide) Add snippet for background fill (#1080)
* [PowerPoint] (Slide) Add snippet for background fill

* Add gets

* Fixes

* Updates based on feedback
</commit_message>
<xml_diff>
--- a/snippet-extractor-metadata/powerpoint.xlsx
+++ b/snippet-extractor-metadata/powerpoint.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D0F7BFA-D1AA-43BE-B4C8-CBE72F79E65D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A9BEA72-B956-4608-AB68-9EF73CDABC17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25180" windowHeight="16140" xr2:uid="{CB5595D7-4492-4192-A1C1-2583BA1957AA}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="871" uniqueCount="230">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="986" uniqueCount="259">
   <si>
     <t>Class</t>
   </si>
@@ -710,6 +710,93 @@
   </si>
   <si>
     <t>resetThemeColors</t>
+  </si>
+  <si>
+    <t>background</t>
+  </si>
+  <si>
+    <t>powerpoint-slide-management-get-set-background-fill</t>
+  </si>
+  <si>
+    <t>getBackgroundFill</t>
+  </si>
+  <si>
+    <t>SlideBackground</t>
+  </si>
+  <si>
+    <t>SlideBackgroundFill</t>
+  </si>
+  <si>
+    <t>setGradientFill</t>
+  </si>
+  <si>
+    <t>setPatternFill</t>
+  </si>
+  <si>
+    <t>setPictureOrTextureFill</t>
+  </si>
+  <si>
+    <t>setSolidFill</t>
+  </si>
+  <si>
+    <t>setPictureFill</t>
+  </si>
+  <si>
+    <t>SlideBackgroundSolidFillOptions</t>
+  </si>
+  <si>
+    <t>SlideBackgroundGradientFillType</t>
+  </si>
+  <si>
+    <t>SlideBackgroundGradientFillOptions</t>
+  </si>
+  <si>
+    <t>SlideBackgroundPatternFillType</t>
+  </si>
+  <si>
+    <t>SlideBackgroundPatternFillOptions</t>
+  </si>
+  <si>
+    <t>SlideBackgroundPictureOrTextureFillOptions</t>
+  </si>
+  <si>
+    <t>SlideBackgroundFillType</t>
+  </si>
+  <si>
+    <t>SlideBackgroundSolidFill</t>
+  </si>
+  <si>
+    <t>getSolidFill</t>
+  </si>
+  <si>
+    <t>SlideBackgroundGradientFill</t>
+  </si>
+  <si>
+    <t>getGradientFill</t>
+  </si>
+  <si>
+    <t>SlideBackgroundPatternFill</t>
+  </si>
+  <si>
+    <t>getPatternFill</t>
+  </si>
+  <si>
+    <t>SlideBackgroundPictureOrTextureFill</t>
+  </si>
+  <si>
+    <t>getPictureFill</t>
+  </si>
+  <si>
+    <t>getSolidFillOrNullObject</t>
+  </si>
+  <si>
+    <t>getGradientFillOrNullObject</t>
+  </si>
+  <si>
+    <t>getPatternFillOrNullObject</t>
+  </si>
+  <si>
+    <t>getPictureOrTextureFillOrNullObject</t>
   </si>
 </sst>
 </file>
@@ -790,10 +877,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{78C585A5-D505-49C6-9CA1-8E6558948317}" name="Snippets" displayName="Snippets" ref="A1:F174" totalsRowShown="0" headerRowDxfId="4">
-  <autoFilter ref="A1:F174" xr:uid="{EAC65D03-FDD2-4352-A5F3-1CDEDE6251B2}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F168">
-    <sortCondition ref="B1:B168"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{78C585A5-D505-49C6-9CA1-8E6558948317}" name="Snippets" displayName="Snippets" ref="A1:F197" totalsRowShown="0" headerRowDxfId="4">
+  <autoFilter ref="A1:F197" xr:uid="{EAC65D03-FDD2-4352-A5F3-1CDEDE6251B2}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F191">
+    <sortCondition ref="B1:B191"/>
   </sortState>
   <tableColumns count="6">
     <tableColumn id="6" xr3:uid="{408888B8-C1DD-4B51-B1EB-5663F091D142}" name="Package"/>
@@ -1104,7 +1191,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{809930CD-A227-47DC-AAA4-BB816AEDEB59}">
-  <dimension ref="A1:F174"/>
+  <dimension ref="A1:F197"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="11.453125" bestFit="1" customWidth="1"/>
@@ -3011,14 +3098,14 @@
       <c r="B105" t="s">
         <v>19</v>
       </c>
-      <c r="C105" t="s">
-        <v>206</v>
-      </c>
-      <c r="E105" t="s">
-        <v>103</v>
-      </c>
-      <c r="F105" t="s">
-        <v>204</v>
+      <c r="C105" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="E105" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="F105" s="2" t="s">
+        <v>232</v>
       </c>
     </row>
     <row r="106" spans="1:6" x14ac:dyDescent="0.35">
@@ -3028,14 +3115,14 @@
       <c r="B106" t="s">
         <v>19</v>
       </c>
-      <c r="C106" s="2" t="s">
-        <v>223</v>
-      </c>
-      <c r="E106" s="2" t="s">
-        <v>225</v>
-      </c>
-      <c r="F106" s="2" t="s">
-        <v>224</v>
+      <c r="C106" t="s">
+        <v>206</v>
+      </c>
+      <c r="E106" t="s">
+        <v>103</v>
+      </c>
+      <c r="F106" t="s">
+        <v>204</v>
       </c>
     </row>
     <row r="107" spans="1:6" x14ac:dyDescent="0.35">
@@ -3043,408 +3130,427 @@
         <v>32</v>
       </c>
       <c r="B107" t="s">
-        <v>9</v>
-      </c>
-      <c r="D107" t="s">
-        <v>87</v>
+        <v>19</v>
+      </c>
+      <c r="C107" t="s">
+        <v>223</v>
       </c>
       <c r="E107" t="s">
-        <v>11</v>
+        <v>225</v>
       </c>
       <c r="F107" t="s">
-        <v>12</v>
+        <v>224</v>
       </c>
     </row>
     <row r="108" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A108" t="s">
         <v>32</v>
       </c>
-      <c r="B108" t="s">
-        <v>9</v>
-      </c>
-      <c r="C108" t="s">
-        <v>10</v>
-      </c>
-      <c r="D108">
-        <v>1</v>
-      </c>
-      <c r="E108" t="s">
-        <v>11</v>
-      </c>
-      <c r="F108" t="s">
-        <v>12</v>
+      <c r="B108" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="C108" s="2"/>
+      <c r="D108" t="s">
+        <v>87</v>
+      </c>
+      <c r="E108" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="F108" s="2" t="s">
+        <v>232</v>
       </c>
     </row>
     <row r="109" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A109" t="s">
         <v>32</v>
       </c>
-      <c r="B109" t="s">
-        <v>9</v>
-      </c>
-      <c r="C109" t="s">
-        <v>16</v>
-      </c>
-      <c r="D109">
-        <v>1</v>
-      </c>
-      <c r="E109" t="s">
-        <v>40</v>
-      </c>
-      <c r="F109" t="s">
-        <v>37</v>
+      <c r="B109" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="C109" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E109" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="F109" s="2" t="s">
+        <v>232</v>
       </c>
     </row>
     <row r="110" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A110" t="s">
         <v>32</v>
       </c>
-      <c r="B110" t="s">
-        <v>185</v>
-      </c>
+      <c r="B110" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="C110" s="2"/>
       <c r="D110" t="s">
-        <v>68</v>
-      </c>
-      <c r="E110" t="s">
-        <v>105</v>
-      </c>
-      <c r="F110" t="s">
-        <v>107</v>
+        <v>87</v>
+      </c>
+      <c r="E110" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="F110" s="2" t="s">
+        <v>232</v>
       </c>
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A111" t="s">
         <v>32</v>
       </c>
-      <c r="B111" t="s">
-        <v>75</v>
-      </c>
-      <c r="D111" t="s">
-        <v>87</v>
-      </c>
-      <c r="E111" t="s">
-        <v>11</v>
-      </c>
-      <c r="F111" t="s">
-        <v>71</v>
+      <c r="B111" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="C111" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="D111">
+        <v>1</v>
+      </c>
+      <c r="E111" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="F111" s="2" t="s">
+        <v>250</v>
       </c>
     </row>
     <row r="112" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A112" t="s">
         <v>32</v>
       </c>
-      <c r="B112" t="s">
-        <v>75</v>
-      </c>
-      <c r="C112" t="s">
-        <v>74</v>
-      </c>
-      <c r="E112" t="s">
-        <v>11</v>
-      </c>
-      <c r="F112" t="s">
-        <v>71</v>
+      <c r="B112" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="C112" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="D112">
+        <v>1</v>
+      </c>
+      <c r="E112" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="F112" s="2" t="s">
+        <v>252</v>
       </c>
     </row>
     <row r="113" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A113" t="s">
         <v>32</v>
       </c>
-      <c r="B113" t="s">
-        <v>72</v>
-      </c>
-      <c r="D113" t="s">
-        <v>87</v>
-      </c>
-      <c r="E113" t="s">
-        <v>11</v>
-      </c>
-      <c r="F113" t="s">
-        <v>71</v>
+      <c r="B113" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="C113" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="D113">
+        <v>1</v>
+      </c>
+      <c r="E113" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="F113" s="2" t="s">
+        <v>254</v>
       </c>
     </row>
     <row r="114" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A114" t="s">
         <v>32</v>
       </c>
-      <c r="B114" t="s">
-        <v>72</v>
-      </c>
-      <c r="C114" t="s">
-        <v>70</v>
+      <c r="B114" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="C114" s="2" t="s">
+        <v>255</v>
       </c>
       <c r="D114">
-        <v>2</v>
-      </c>
-      <c r="E114" t="s">
-        <v>11</v>
-      </c>
-      <c r="F114" t="s">
-        <v>71</v>
+        <v>1</v>
+      </c>
+      <c r="E114" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="F114" s="2" t="s">
+        <v>248</v>
       </c>
     </row>
     <row r="115" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A115" t="s">
         <v>32</v>
       </c>
-      <c r="B115" t="s">
-        <v>186</v>
-      </c>
-      <c r="D115" t="s">
-        <v>65</v>
-      </c>
-      <c r="E115" t="s">
-        <v>85</v>
-      </c>
-      <c r="F115" t="s">
-        <v>79</v>
+      <c r="B115" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="C115" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="D115">
+        <v>1</v>
+      </c>
+      <c r="E115" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="F115" s="2" t="s">
+        <v>235</v>
       </c>
     </row>
     <row r="116" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A116" t="s">
         <v>32</v>
       </c>
-      <c r="B116" t="s">
-        <v>73</v>
-      </c>
-      <c r="D116" t="s">
-        <v>87</v>
-      </c>
-      <c r="E116" t="s">
-        <v>11</v>
-      </c>
-      <c r="F116" t="s">
-        <v>71</v>
+      <c r="B116" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="C116" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="D116">
+        <v>1</v>
+      </c>
+      <c r="E116" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="F116" s="2" t="s">
+        <v>236</v>
       </c>
     </row>
     <row r="117" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A117" t="s">
         <v>32</v>
       </c>
-      <c r="B117" t="s">
-        <v>73</v>
-      </c>
-      <c r="C117" t="s">
-        <v>74</v>
-      </c>
-      <c r="E117" t="s">
-        <v>11</v>
-      </c>
-      <c r="F117" t="s">
-        <v>71</v>
+      <c r="B117" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="C117" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="D117">
+        <v>1</v>
+      </c>
+      <c r="E117" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="F117" s="2" t="s">
+        <v>239</v>
       </c>
     </row>
     <row r="118" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A118" t="s">
         <v>32</v>
       </c>
-      <c r="B118" t="s">
-        <v>69</v>
-      </c>
-      <c r="D118" t="s">
-        <v>87</v>
-      </c>
-      <c r="E118" t="s">
-        <v>11</v>
-      </c>
-      <c r="F118" t="s">
-        <v>71</v>
+      <c r="B118" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="C118" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="D118">
+        <v>1</v>
+      </c>
+      <c r="E118" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="F118" s="2" t="s">
+        <v>238</v>
       </c>
     </row>
     <row r="119" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A119" t="s">
         <v>32</v>
       </c>
-      <c r="B119" t="s">
-        <v>69</v>
-      </c>
-      <c r="C119" t="s">
-        <v>70</v>
-      </c>
-      <c r="D119">
-        <v>2</v>
-      </c>
-      <c r="E119" t="s">
-        <v>11</v>
-      </c>
-      <c r="F119" t="s">
-        <v>71</v>
+      <c r="B119" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="C119" s="2"/>
+      <c r="D119" t="s">
+        <v>65</v>
+      </c>
+      <c r="E119" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="F119" s="2" t="s">
+        <v>232</v>
       </c>
     </row>
     <row r="120" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A120" t="s">
         <v>32</v>
       </c>
-      <c r="B120" t="s">
-        <v>92</v>
-      </c>
+      <c r="B120" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="C120" s="2"/>
       <c r="D120" t="s">
         <v>87</v>
       </c>
-      <c r="E120" t="s">
-        <v>53</v>
-      </c>
-      <c r="F120" t="s">
-        <v>47</v>
+      <c r="E120" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="F120" s="2" t="s">
+        <v>250</v>
       </c>
     </row>
     <row r="121" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A121" t="s">
         <v>32</v>
       </c>
-      <c r="B121" t="s">
-        <v>92</v>
-      </c>
-      <c r="C121" t="s">
-        <v>220</v>
-      </c>
-      <c r="D121">
-        <v>1</v>
-      </c>
-      <c r="E121" t="s">
-        <v>219</v>
-      </c>
-      <c r="F121" t="s">
-        <v>218</v>
+      <c r="B121" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="C121" s="2"/>
+      <c r="D121" t="s">
+        <v>68</v>
+      </c>
+      <c r="E121" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="F121" s="2" t="s">
+        <v>235</v>
       </c>
     </row>
     <row r="122" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A122" t="s">
         <v>32</v>
       </c>
-      <c r="B122" t="s">
-        <v>162</v>
-      </c>
+      <c r="B122" s="2" t="s">
+        <v>241</v>
+      </c>
+      <c r="C122" s="2"/>
       <c r="D122" t="s">
-        <v>87</v>
-      </c>
-      <c r="E122" t="s">
-        <v>116</v>
-      </c>
-      <c r="F122" t="s">
-        <v>163</v>
+        <v>65</v>
+      </c>
+      <c r="E122" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="F122" s="2" t="s">
+        <v>235</v>
       </c>
     </row>
     <row r="123" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A123" t="s">
         <v>32</v>
       </c>
-      <c r="B123" t="s">
-        <v>162</v>
-      </c>
-      <c r="C123" t="s">
-        <v>164</v>
-      </c>
-      <c r="D123">
-        <v>1</v>
-      </c>
-      <c r="E123" t="s">
-        <v>116</v>
-      </c>
-      <c r="F123" t="s">
-        <v>163</v>
+      <c r="B123" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="C123" s="2"/>
+      <c r="D123" t="s">
+        <v>87</v>
+      </c>
+      <c r="E123" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="F123" s="2" t="s">
+        <v>252</v>
       </c>
     </row>
     <row r="124" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A124" t="s">
         <v>32</v>
       </c>
-      <c r="B124" t="s">
-        <v>118</v>
-      </c>
+      <c r="B124" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="C124" s="2"/>
       <c r="D124" t="s">
         <v>68</v>
       </c>
-      <c r="E124" t="s">
-        <v>116</v>
-      </c>
-      <c r="F124" t="s">
-        <v>119</v>
+      <c r="E124" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="F124" s="2" t="s">
+        <v>236</v>
       </c>
     </row>
     <row r="125" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A125" t="s">
         <v>32</v>
       </c>
-      <c r="B125" t="s">
-        <v>118</v>
-      </c>
-      <c r="C125" t="s">
-        <v>124</v>
-      </c>
-      <c r="E125" t="s">
-        <v>116</v>
-      </c>
-      <c r="F125" t="s">
-        <v>121</v>
+      <c r="B125" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="C125" s="2"/>
+      <c r="D125" t="s">
+        <v>65</v>
+      </c>
+      <c r="E125" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="F125" s="2" t="s">
+        <v>236</v>
       </c>
     </row>
     <row r="126" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A126" t="s">
         <v>32</v>
       </c>
-      <c r="B126" t="s">
-        <v>118</v>
-      </c>
-      <c r="C126" t="s">
-        <v>52</v>
-      </c>
-      <c r="E126" t="s">
-        <v>116</v>
-      </c>
-      <c r="F126" t="s">
-        <v>119</v>
+      <c r="B126" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="C126" s="2"/>
+      <c r="D126" t="s">
+        <v>87</v>
+      </c>
+      <c r="E126" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="F126" s="2" t="s">
+        <v>254</v>
       </c>
     </row>
     <row r="127" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A127" t="s">
         <v>32</v>
       </c>
-      <c r="B127" t="s">
-        <v>118</v>
-      </c>
-      <c r="C127" t="s">
-        <v>129</v>
-      </c>
-      <c r="E127" t="s">
-        <v>116</v>
-      </c>
-      <c r="F127" t="s">
-        <v>130</v>
+      <c r="B127" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="C127" s="2"/>
+      <c r="D127" t="s">
+        <v>68</v>
+      </c>
+      <c r="E127" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="F127" s="2" t="s">
+        <v>239</v>
       </c>
     </row>
     <row r="128" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A128" t="s">
         <v>32</v>
       </c>
-      <c r="B128" t="s">
-        <v>118</v>
-      </c>
-      <c r="C128" t="s">
-        <v>123</v>
-      </c>
-      <c r="E128" t="s">
-        <v>116</v>
-      </c>
-      <c r="F128" t="s">
-        <v>121</v>
+      <c r="B128" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="C128" s="2"/>
+      <c r="D128" t="s">
+        <v>87</v>
+      </c>
+      <c r="E128" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="F128" s="2" t="s">
+        <v>248</v>
       </c>
     </row>
     <row r="129" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A129" t="s">
         <v>32</v>
       </c>
-      <c r="B129" t="s">
-        <v>118</v>
-      </c>
-      <c r="C129" t="s">
-        <v>136</v>
-      </c>
-      <c r="E129" t="s">
-        <v>116</v>
-      </c>
-      <c r="F129" t="s">
-        <v>137</v>
+      <c r="B129" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="C129" s="2"/>
+      <c r="D129" t="s">
+        <v>68</v>
+      </c>
+      <c r="E129" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="F129" s="2" t="s">
+        <v>238</v>
       </c>
     </row>
     <row r="130" spans="1:6" x14ac:dyDescent="0.35">
@@ -3452,16 +3558,16 @@
         <v>32</v>
       </c>
       <c r="B130" t="s">
-        <v>118</v>
-      </c>
-      <c r="C130" t="s">
-        <v>146</v>
+        <v>9</v>
+      </c>
+      <c r="D130" t="s">
+        <v>87</v>
       </c>
       <c r="E130" t="s">
-        <v>116</v>
+        <v>11</v>
       </c>
       <c r="F130" t="s">
-        <v>147</v>
+        <v>12</v>
       </c>
     </row>
     <row r="131" spans="1:6" x14ac:dyDescent="0.35">
@@ -3469,16 +3575,19 @@
         <v>32</v>
       </c>
       <c r="B131" t="s">
-        <v>118</v>
+        <v>9</v>
       </c>
       <c r="C131" t="s">
-        <v>120</v>
+        <v>10</v>
+      </c>
+      <c r="D131">
+        <v>1</v>
       </c>
       <c r="E131" t="s">
-        <v>116</v>
+        <v>11</v>
       </c>
       <c r="F131" t="s">
-        <v>122</v>
+        <v>12</v>
       </c>
     </row>
     <row r="132" spans="1:6" x14ac:dyDescent="0.35">
@@ -3486,16 +3595,19 @@
         <v>32</v>
       </c>
       <c r="B132" t="s">
-        <v>118</v>
+        <v>9</v>
       </c>
       <c r="C132" t="s">
-        <v>51</v>
+        <v>16</v>
+      </c>
+      <c r="D132">
+        <v>1</v>
       </c>
       <c r="E132" t="s">
-        <v>116</v>
+        <v>40</v>
       </c>
       <c r="F132" t="s">
-        <v>119</v>
+        <v>37</v>
       </c>
     </row>
     <row r="133" spans="1:6" x14ac:dyDescent="0.35">
@@ -3503,16 +3615,16 @@
         <v>32</v>
       </c>
       <c r="B133" t="s">
-        <v>165</v>
+        <v>185</v>
       </c>
       <c r="D133" t="s">
-        <v>87</v>
+        <v>68</v>
       </c>
       <c r="E133" t="s">
-        <v>116</v>
+        <v>105</v>
       </c>
       <c r="F133" t="s">
-        <v>163</v>
+        <v>107</v>
       </c>
     </row>
     <row r="134" spans="1:6" x14ac:dyDescent="0.35">
@@ -3520,16 +3632,16 @@
         <v>32</v>
       </c>
       <c r="B134" t="s">
-        <v>165</v>
-      </c>
-      <c r="C134" t="s">
-        <v>166</v>
+        <v>75</v>
+      </c>
+      <c r="D134" t="s">
+        <v>87</v>
       </c>
       <c r="E134" t="s">
-        <v>116</v>
+        <v>11</v>
       </c>
       <c r="F134" t="s">
-        <v>163</v>
+        <v>71</v>
       </c>
     </row>
     <row r="135" spans="1:6" x14ac:dyDescent="0.35">
@@ -3537,16 +3649,16 @@
         <v>32</v>
       </c>
       <c r="B135" t="s">
-        <v>149</v>
-      </c>
-      <c r="D135" t="s">
-        <v>68</v>
+        <v>75</v>
+      </c>
+      <c r="C135" t="s">
+        <v>74</v>
       </c>
       <c r="E135" t="s">
-        <v>116</v>
+        <v>11</v>
       </c>
       <c r="F135" t="s">
-        <v>147</v>
+        <v>71</v>
       </c>
     </row>
     <row r="136" spans="1:6" x14ac:dyDescent="0.35">
@@ -3554,16 +3666,16 @@
         <v>32</v>
       </c>
       <c r="B136" t="s">
-        <v>149</v>
-      </c>
-      <c r="C136" t="s">
-        <v>151</v>
+        <v>72</v>
+      </c>
+      <c r="D136" t="s">
+        <v>87</v>
       </c>
       <c r="E136" t="s">
-        <v>116</v>
+        <v>11</v>
       </c>
       <c r="F136" t="s">
-        <v>147</v>
+        <v>71</v>
       </c>
     </row>
     <row r="137" spans="1:6" x14ac:dyDescent="0.35">
@@ -3571,16 +3683,19 @@
         <v>32</v>
       </c>
       <c r="B137" t="s">
-        <v>149</v>
+        <v>72</v>
       </c>
       <c r="C137" t="s">
-        <v>49</v>
+        <v>70</v>
+      </c>
+      <c r="D137">
+        <v>2</v>
       </c>
       <c r="E137" t="s">
-        <v>116</v>
+        <v>11</v>
       </c>
       <c r="F137" t="s">
-        <v>147</v>
+        <v>71</v>
       </c>
     </row>
     <row r="138" spans="1:6" x14ac:dyDescent="0.35">
@@ -3588,16 +3703,16 @@
         <v>32</v>
       </c>
       <c r="B138" t="s">
-        <v>149</v>
-      </c>
-      <c r="C138" t="s">
-        <v>150</v>
+        <v>186</v>
+      </c>
+      <c r="D138" t="s">
+        <v>65</v>
       </c>
       <c r="E138" t="s">
-        <v>116</v>
+        <v>85</v>
       </c>
       <c r="F138" t="s">
-        <v>147</v>
+        <v>79</v>
       </c>
     </row>
     <row r="139" spans="1:6" x14ac:dyDescent="0.35">
@@ -3605,16 +3720,16 @@
         <v>32</v>
       </c>
       <c r="B139" t="s">
-        <v>149</v>
-      </c>
-      <c r="C139" t="s">
-        <v>50</v>
+        <v>73</v>
+      </c>
+      <c r="D139" t="s">
+        <v>87</v>
       </c>
       <c r="E139" t="s">
-        <v>116</v>
+        <v>11</v>
       </c>
       <c r="F139" t="s">
-        <v>147</v>
+        <v>71</v>
       </c>
     </row>
     <row r="140" spans="1:6" x14ac:dyDescent="0.35">
@@ -3622,16 +3737,16 @@
         <v>32</v>
       </c>
       <c r="B140" t="s">
-        <v>138</v>
-      </c>
-      <c r="D140" t="s">
-        <v>68</v>
+        <v>73</v>
+      </c>
+      <c r="C140" t="s">
+        <v>74</v>
       </c>
       <c r="E140" t="s">
-        <v>116</v>
+        <v>11</v>
       </c>
       <c r="F140" t="s">
-        <v>137</v>
+        <v>71</v>
       </c>
     </row>
     <row r="141" spans="1:6" x14ac:dyDescent="0.35">
@@ -3639,16 +3754,16 @@
         <v>32</v>
       </c>
       <c r="B141" t="s">
-        <v>138</v>
-      </c>
-      <c r="C141" t="s">
-        <v>148</v>
+        <v>69</v>
+      </c>
+      <c r="D141" t="s">
+        <v>87</v>
       </c>
       <c r="E141" t="s">
-        <v>116</v>
+        <v>11</v>
       </c>
       <c r="F141" t="s">
-        <v>147</v>
+        <v>71</v>
       </c>
     </row>
     <row r="142" spans="1:6" x14ac:dyDescent="0.35">
@@ -3656,16 +3771,19 @@
         <v>32</v>
       </c>
       <c r="B142" t="s">
-        <v>138</v>
+        <v>69</v>
       </c>
       <c r="C142" t="s">
-        <v>58</v>
+        <v>70</v>
+      </c>
+      <c r="D142">
+        <v>2</v>
       </c>
       <c r="E142" t="s">
-        <v>116</v>
+        <v>11</v>
       </c>
       <c r="F142" t="s">
-        <v>137</v>
+        <v>71</v>
       </c>
     </row>
     <row r="143" spans="1:6" x14ac:dyDescent="0.35">
@@ -3673,16 +3791,16 @@
         <v>32</v>
       </c>
       <c r="B143" t="s">
-        <v>138</v>
-      </c>
-      <c r="C143" t="s">
-        <v>57</v>
+        <v>92</v>
+      </c>
+      <c r="D143" t="s">
+        <v>87</v>
       </c>
       <c r="E143" t="s">
-        <v>116</v>
+        <v>53</v>
       </c>
       <c r="F143" t="s">
-        <v>137</v>
+        <v>47</v>
       </c>
     </row>
     <row r="144" spans="1:6" x14ac:dyDescent="0.35">
@@ -3690,16 +3808,19 @@
         <v>32</v>
       </c>
       <c r="B144" t="s">
-        <v>138</v>
+        <v>92</v>
       </c>
       <c r="C144" t="s">
-        <v>156</v>
+        <v>220</v>
+      </c>
+      <c r="D144">
+        <v>1</v>
       </c>
       <c r="E144" t="s">
-        <v>116</v>
+        <v>219</v>
       </c>
       <c r="F144" t="s">
-        <v>158</v>
+        <v>218</v>
       </c>
     </row>
     <row r="145" spans="1:6" x14ac:dyDescent="0.35">
@@ -3707,16 +3828,16 @@
         <v>32</v>
       </c>
       <c r="B145" t="s">
-        <v>138</v>
-      </c>
-      <c r="C145" t="s">
-        <v>154</v>
+        <v>162</v>
+      </c>
+      <c r="D145" t="s">
+        <v>87</v>
       </c>
       <c r="E145" t="s">
         <v>116</v>
       </c>
       <c r="F145" t="s">
-        <v>155</v>
+        <v>163</v>
       </c>
     </row>
     <row r="146" spans="1:6" x14ac:dyDescent="0.35">
@@ -3724,16 +3845,19 @@
         <v>32</v>
       </c>
       <c r="B146" t="s">
-        <v>138</v>
+        <v>162</v>
       </c>
       <c r="C146" t="s">
-        <v>184</v>
+        <v>164</v>
+      </c>
+      <c r="D146">
+        <v>1</v>
       </c>
       <c r="E146" t="s">
         <v>116</v>
       </c>
       <c r="F146" t="s">
-        <v>183</v>
+        <v>163</v>
       </c>
     </row>
     <row r="147" spans="1:6" x14ac:dyDescent="0.35">
@@ -3741,16 +3865,16 @@
         <v>32</v>
       </c>
       <c r="B147" t="s">
-        <v>138</v>
-      </c>
-      <c r="C147" t="s">
-        <v>157</v>
+        <v>118</v>
+      </c>
+      <c r="D147" t="s">
+        <v>68</v>
       </c>
       <c r="E147" t="s">
         <v>116</v>
       </c>
       <c r="F147" t="s">
-        <v>158</v>
+        <v>119</v>
       </c>
     </row>
     <row r="148" spans="1:6" x14ac:dyDescent="0.35">
@@ -3758,10 +3882,10 @@
         <v>32</v>
       </c>
       <c r="B148" t="s">
-        <v>125</v>
-      </c>
-      <c r="D148" t="s">
-        <v>68</v>
+        <v>118</v>
+      </c>
+      <c r="C148" t="s">
+        <v>124</v>
       </c>
       <c r="E148" t="s">
         <v>116</v>
@@ -3775,16 +3899,16 @@
         <v>32</v>
       </c>
       <c r="B149" t="s">
-        <v>125</v>
+        <v>118</v>
       </c>
       <c r="C149" t="s">
-        <v>127</v>
+        <v>52</v>
       </c>
       <c r="E149" t="s">
         <v>116</v>
       </c>
       <c r="F149" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
     <row r="150" spans="1:6" x14ac:dyDescent="0.35">
@@ -3792,10 +3916,10 @@
         <v>32</v>
       </c>
       <c r="B150" t="s">
-        <v>131</v>
-      </c>
-      <c r="D150" t="s">
-        <v>68</v>
+        <v>118</v>
+      </c>
+      <c r="C150" t="s">
+        <v>129</v>
       </c>
       <c r="E150" t="s">
         <v>116</v>
@@ -3809,16 +3933,16 @@
         <v>32</v>
       </c>
       <c r="B151" t="s">
-        <v>131</v>
+        <v>118</v>
       </c>
       <c r="C151" t="s">
-        <v>132</v>
+        <v>123</v>
       </c>
       <c r="E151" t="s">
         <v>116</v>
       </c>
       <c r="F151" t="s">
-        <v>130</v>
+        <v>121</v>
       </c>
     </row>
     <row r="152" spans="1:6" x14ac:dyDescent="0.35">
@@ -3826,16 +3950,16 @@
         <v>32</v>
       </c>
       <c r="B152" t="s">
-        <v>131</v>
+        <v>118</v>
       </c>
       <c r="C152" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="E152" t="s">
         <v>116</v>
       </c>
       <c r="F152" t="s">
-        <v>130</v>
+        <v>137</v>
       </c>
     </row>
     <row r="153" spans="1:6" x14ac:dyDescent="0.35">
@@ -3843,16 +3967,16 @@
         <v>32</v>
       </c>
       <c r="B153" t="s">
-        <v>131</v>
+        <v>118</v>
       </c>
       <c r="C153" t="s">
-        <v>134</v>
+        <v>146</v>
       </c>
       <c r="E153" t="s">
         <v>116</v>
       </c>
       <c r="F153" t="s">
-        <v>130</v>
+        <v>147</v>
       </c>
     </row>
     <row r="154" spans="1:6" x14ac:dyDescent="0.35">
@@ -3860,16 +3984,16 @@
         <v>32</v>
       </c>
       <c r="B154" t="s">
-        <v>131</v>
+        <v>118</v>
       </c>
       <c r="C154" t="s">
-        <v>135</v>
+        <v>120</v>
       </c>
       <c r="E154" t="s">
         <v>116</v>
       </c>
       <c r="F154" t="s">
-        <v>130</v>
+        <v>122</v>
       </c>
     </row>
     <row r="155" spans="1:6" x14ac:dyDescent="0.35">
@@ -3877,16 +4001,16 @@
         <v>32</v>
       </c>
       <c r="B155" t="s">
-        <v>126</v>
-      </c>
-      <c r="D155" t="s">
-        <v>68</v>
+        <v>118</v>
+      </c>
+      <c r="C155" t="s">
+        <v>51</v>
       </c>
       <c r="E155" t="s">
         <v>116</v>
       </c>
       <c r="F155" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
     <row r="156" spans="1:6" x14ac:dyDescent="0.35">
@@ -3894,16 +4018,16 @@
         <v>32</v>
       </c>
       <c r="B156" t="s">
-        <v>126</v>
-      </c>
-      <c r="C156" t="s">
-        <v>128</v>
+        <v>165</v>
+      </c>
+      <c r="D156" t="s">
+        <v>87</v>
       </c>
       <c r="E156" t="s">
         <v>116</v>
       </c>
       <c r="F156" t="s">
-        <v>121</v>
+        <v>163</v>
       </c>
     </row>
     <row r="157" spans="1:6" x14ac:dyDescent="0.35">
@@ -3911,16 +4035,16 @@
         <v>32</v>
       </c>
       <c r="B157" t="s">
-        <v>98</v>
-      </c>
-      <c r="D157" t="s">
-        <v>87</v>
+        <v>165</v>
+      </c>
+      <c r="C157" t="s">
+        <v>166</v>
       </c>
       <c r="E157" t="s">
-        <v>14</v>
+        <v>116</v>
       </c>
       <c r="F157" t="s">
-        <v>99</v>
+        <v>163</v>
       </c>
     </row>
     <row r="158" spans="1:6" x14ac:dyDescent="0.35">
@@ -3928,16 +4052,16 @@
         <v>32</v>
       </c>
       <c r="B158" t="s">
-        <v>13</v>
+        <v>149</v>
       </c>
       <c r="D158" t="s">
-        <v>87</v>
+        <v>68</v>
       </c>
       <c r="E158" t="s">
-        <v>14</v>
+        <v>116</v>
       </c>
       <c r="F158" t="s">
-        <v>17</v>
+        <v>147</v>
       </c>
     </row>
     <row r="159" spans="1:6" x14ac:dyDescent="0.35">
@@ -3945,19 +4069,16 @@
         <v>32</v>
       </c>
       <c r="B159" t="s">
-        <v>13</v>
+        <v>149</v>
       </c>
       <c r="C159" t="s">
-        <v>10</v>
-      </c>
-      <c r="D159">
-        <v>1</v>
+        <v>151</v>
       </c>
       <c r="E159" t="s">
-        <v>14</v>
+        <v>116</v>
       </c>
       <c r="F159" t="s">
-        <v>15</v>
+        <v>147</v>
       </c>
     </row>
     <row r="160" spans="1:6" x14ac:dyDescent="0.35">
@@ -3965,19 +4086,16 @@
         <v>32</v>
       </c>
       <c r="B160" t="s">
-        <v>13</v>
+        <v>149</v>
       </c>
       <c r="C160" t="s">
-        <v>20</v>
-      </c>
-      <c r="D160">
-        <v>1</v>
+        <v>49</v>
       </c>
       <c r="E160" t="s">
-        <v>14</v>
+        <v>116</v>
       </c>
       <c r="F160" t="s">
-        <v>23</v>
+        <v>147</v>
       </c>
     </row>
     <row r="161" spans="1:6" x14ac:dyDescent="0.35">
@@ -3985,19 +4103,16 @@
         <v>32</v>
       </c>
       <c r="B161" t="s">
-        <v>13</v>
+        <v>149</v>
       </c>
       <c r="C161" t="s">
-        <v>18</v>
-      </c>
-      <c r="D161">
-        <v>1</v>
+        <v>150</v>
       </c>
       <c r="E161" t="s">
-        <v>14</v>
+        <v>116</v>
       </c>
       <c r="F161" t="s">
-        <v>17</v>
+        <v>147</v>
       </c>
     </row>
     <row r="162" spans="1:6" x14ac:dyDescent="0.35">
@@ -4005,16 +4120,16 @@
         <v>32</v>
       </c>
       <c r="B162" t="s">
-        <v>97</v>
-      </c>
-      <c r="D162" t="s">
-        <v>87</v>
+        <v>149</v>
+      </c>
+      <c r="C162" t="s">
+        <v>50</v>
       </c>
       <c r="E162" t="s">
-        <v>54</v>
+        <v>116</v>
       </c>
       <c r="F162" t="s">
-        <v>63</v>
+        <v>147</v>
       </c>
     </row>
     <row r="163" spans="1:6" x14ac:dyDescent="0.35">
@@ -4022,19 +4137,16 @@
         <v>32</v>
       </c>
       <c r="B163" t="s">
-        <v>97</v>
-      </c>
-      <c r="C163" t="s">
-        <v>216</v>
-      </c>
-      <c r="D163">
-        <v>1</v>
+        <v>138</v>
+      </c>
+      <c r="D163" t="s">
+        <v>68</v>
       </c>
       <c r="E163" t="s">
-        <v>54</v>
+        <v>116</v>
       </c>
       <c r="F163" t="s">
-        <v>193</v>
+        <v>137</v>
       </c>
     </row>
     <row r="164" spans="1:6" x14ac:dyDescent="0.35">
@@ -4042,16 +4154,16 @@
         <v>32</v>
       </c>
       <c r="B164" t="s">
-        <v>97</v>
+        <v>138</v>
       </c>
       <c r="C164" t="s">
-        <v>191</v>
+        <v>148</v>
       </c>
       <c r="E164" t="s">
-        <v>24</v>
+        <v>116</v>
       </c>
       <c r="F164" t="s">
-        <v>89</v>
+        <v>147</v>
       </c>
     </row>
     <row r="165" spans="1:6" x14ac:dyDescent="0.35">
@@ -4059,16 +4171,16 @@
         <v>32</v>
       </c>
       <c r="B165" t="s">
-        <v>33</v>
-      </c>
-      <c r="D165" t="s">
-        <v>87</v>
+        <v>138</v>
+      </c>
+      <c r="C165" t="s">
+        <v>58</v>
       </c>
       <c r="E165" t="s">
-        <v>54</v>
+        <v>116</v>
       </c>
       <c r="F165" t="s">
-        <v>56</v>
+        <v>137</v>
       </c>
     </row>
     <row r="166" spans="1:6" x14ac:dyDescent="0.35">
@@ -4076,19 +4188,16 @@
         <v>32</v>
       </c>
       <c r="B166" t="s">
-        <v>33</v>
+        <v>138</v>
       </c>
       <c r="C166" t="s">
-        <v>215</v>
-      </c>
-      <c r="D166">
-        <v>1</v>
+        <v>57</v>
       </c>
       <c r="E166" t="s">
-        <v>54</v>
+        <v>116</v>
       </c>
       <c r="F166" t="s">
-        <v>193</v>
+        <v>137</v>
       </c>
     </row>
     <row r="167" spans="1:6" x14ac:dyDescent="0.35">
@@ -4096,19 +4205,16 @@
         <v>32</v>
       </c>
       <c r="B167" t="s">
-        <v>33</v>
-      </c>
-      <c r="C167" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="D167">
-        <v>1</v>
+        <v>138</v>
+      </c>
+      <c r="C167" t="s">
+        <v>156</v>
       </c>
       <c r="E167" t="s">
-        <v>54</v>
+        <v>116</v>
       </c>
       <c r="F167" t="s">
-        <v>63</v>
+        <v>158</v>
       </c>
     </row>
     <row r="168" spans="1:6" x14ac:dyDescent="0.35">
@@ -4116,19 +4222,16 @@
         <v>32</v>
       </c>
       <c r="B168" t="s">
-        <v>33</v>
-      </c>
-      <c r="C168" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="D168">
-        <v>1</v>
+        <v>138</v>
+      </c>
+      <c r="C168" t="s">
+        <v>154</v>
       </c>
       <c r="E168" t="s">
-        <v>54</v>
+        <v>116</v>
       </c>
       <c r="F168" t="s">
-        <v>55</v>
+        <v>155</v>
       </c>
     </row>
     <row r="169" spans="1:6" x14ac:dyDescent="0.35">
@@ -4136,16 +4239,16 @@
         <v>32</v>
       </c>
       <c r="B169" t="s">
-        <v>33</v>
-      </c>
-      <c r="C169" s="1" t="s">
-        <v>57</v>
+        <v>138</v>
+      </c>
+      <c r="C169" t="s">
+        <v>184</v>
       </c>
       <c r="E169" t="s">
-        <v>54</v>
+        <v>116</v>
       </c>
       <c r="F169" t="s">
-        <v>56</v>
+        <v>183</v>
       </c>
     </row>
     <row r="170" spans="1:6" x14ac:dyDescent="0.35">
@@ -4153,16 +4256,16 @@
         <v>32</v>
       </c>
       <c r="B170" t="s">
-        <v>33</v>
-      </c>
-      <c r="C170" s="1" t="s">
-        <v>195</v>
+        <v>138</v>
+      </c>
+      <c r="C170" t="s">
+        <v>157</v>
       </c>
       <c r="E170" t="s">
-        <v>54</v>
+        <v>116</v>
       </c>
       <c r="F170" t="s">
-        <v>193</v>
+        <v>158</v>
       </c>
     </row>
     <row r="171" spans="1:6" x14ac:dyDescent="0.35">
@@ -4170,9 +4273,8 @@
         <v>32</v>
       </c>
       <c r="B171" t="s">
-        <v>182</v>
-      </c>
-      <c r="C171" s="1"/>
+        <v>125</v>
+      </c>
       <c r="D171" t="s">
         <v>68</v>
       </c>
@@ -4180,7 +4282,7 @@
         <v>116</v>
       </c>
       <c r="F171" t="s">
-        <v>183</v>
+        <v>121</v>
       </c>
     </row>
     <row r="172" spans="1:6" x14ac:dyDescent="0.35">
@@ -4188,51 +4290,462 @@
         <v>32</v>
       </c>
       <c r="B172" t="s">
-        <v>88</v>
-      </c>
-      <c r="D172" t="s">
-        <v>65</v>
+        <v>125</v>
+      </c>
+      <c r="C172" t="s">
+        <v>127</v>
       </c>
       <c r="E172" t="s">
-        <v>24</v>
+        <v>116</v>
       </c>
       <c r="F172" t="s">
-        <v>89</v>
+        <v>121</v>
       </c>
     </row>
     <row r="173" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A173" t="s">
         <v>32</v>
       </c>
-      <c r="B173" s="2" t="s">
-        <v>226</v>
-      </c>
-      <c r="C173" s="2"/>
+      <c r="B173" t="s">
+        <v>131</v>
+      </c>
       <c r="D173" t="s">
-        <v>65</v>
-      </c>
-      <c r="E173" s="2" t="s">
-        <v>225</v>
-      </c>
-      <c r="F173" s="2" t="s">
-        <v>227</v>
+        <v>68</v>
+      </c>
+      <c r="E173" t="s">
+        <v>116</v>
+      </c>
+      <c r="F173" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="174" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A174" t="s">
         <v>32</v>
       </c>
-      <c r="B174" s="2" t="s">
+      <c r="B174" t="s">
+        <v>131</v>
+      </c>
+      <c r="C174" t="s">
+        <v>132</v>
+      </c>
+      <c r="E174" t="s">
+        <v>116</v>
+      </c>
+      <c r="F174" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="175" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A175" t="s">
+        <v>32</v>
+      </c>
+      <c r="B175" t="s">
+        <v>131</v>
+      </c>
+      <c r="C175" t="s">
+        <v>133</v>
+      </c>
+      <c r="E175" t="s">
+        <v>116</v>
+      </c>
+      <c r="F175" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="176" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A176" t="s">
+        <v>32</v>
+      </c>
+      <c r="B176" t="s">
+        <v>131</v>
+      </c>
+      <c r="C176" t="s">
+        <v>134</v>
+      </c>
+      <c r="E176" t="s">
+        <v>116</v>
+      </c>
+      <c r="F176" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="177" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A177" t="s">
+        <v>32</v>
+      </c>
+      <c r="B177" t="s">
+        <v>131</v>
+      </c>
+      <c r="C177" t="s">
+        <v>135</v>
+      </c>
+      <c r="E177" t="s">
+        <v>116</v>
+      </c>
+      <c r="F177" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="178" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A178" t="s">
+        <v>32</v>
+      </c>
+      <c r="B178" t="s">
+        <v>126</v>
+      </c>
+      <c r="D178" t="s">
+        <v>68</v>
+      </c>
+      <c r="E178" t="s">
+        <v>116</v>
+      </c>
+      <c r="F178" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="179" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A179" t="s">
+        <v>32</v>
+      </c>
+      <c r="B179" t="s">
+        <v>126</v>
+      </c>
+      <c r="C179" t="s">
+        <v>128</v>
+      </c>
+      <c r="E179" t="s">
+        <v>116</v>
+      </c>
+      <c r="F179" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="180" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A180" t="s">
+        <v>32</v>
+      </c>
+      <c r="B180" t="s">
+        <v>98</v>
+      </c>
+      <c r="D180" t="s">
+        <v>87</v>
+      </c>
+      <c r="E180" t="s">
+        <v>14</v>
+      </c>
+      <c r="F180" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="181" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A181" t="s">
+        <v>32</v>
+      </c>
+      <c r="B181" t="s">
+        <v>13</v>
+      </c>
+      <c r="D181" t="s">
+        <v>87</v>
+      </c>
+      <c r="E181" t="s">
+        <v>14</v>
+      </c>
+      <c r="F181" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="182" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A182" t="s">
+        <v>32</v>
+      </c>
+      <c r="B182" t="s">
+        <v>13</v>
+      </c>
+      <c r="C182" t="s">
+        <v>10</v>
+      </c>
+      <c r="D182">
+        <v>1</v>
+      </c>
+      <c r="E182" t="s">
+        <v>14</v>
+      </c>
+      <c r="F182" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="183" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A183" t="s">
+        <v>32</v>
+      </c>
+      <c r="B183" t="s">
+        <v>13</v>
+      </c>
+      <c r="C183" t="s">
+        <v>20</v>
+      </c>
+      <c r="D183">
+        <v>1</v>
+      </c>
+      <c r="E183" t="s">
+        <v>14</v>
+      </c>
+      <c r="F183" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="184" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A184" t="s">
+        <v>32</v>
+      </c>
+      <c r="B184" t="s">
+        <v>13</v>
+      </c>
+      <c r="C184" t="s">
+        <v>18</v>
+      </c>
+      <c r="D184">
+        <v>1</v>
+      </c>
+      <c r="E184" t="s">
+        <v>14</v>
+      </c>
+      <c r="F184" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="185" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A185" t="s">
+        <v>32</v>
+      </c>
+      <c r="B185" t="s">
+        <v>97</v>
+      </c>
+      <c r="D185" t="s">
+        <v>87</v>
+      </c>
+      <c r="E185" t="s">
+        <v>54</v>
+      </c>
+      <c r="F185" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="186" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A186" t="s">
+        <v>32</v>
+      </c>
+      <c r="B186" t="s">
+        <v>97</v>
+      </c>
+      <c r="C186" t="s">
+        <v>216</v>
+      </c>
+      <c r="D186">
+        <v>1</v>
+      </c>
+      <c r="E186" t="s">
+        <v>54</v>
+      </c>
+      <c r="F186" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="187" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A187" t="s">
+        <v>32</v>
+      </c>
+      <c r="B187" t="s">
+        <v>97</v>
+      </c>
+      <c r="C187" t="s">
+        <v>191</v>
+      </c>
+      <c r="E187" t="s">
+        <v>24</v>
+      </c>
+      <c r="F187" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="188" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A188" t="s">
+        <v>32</v>
+      </c>
+      <c r="B188" t="s">
+        <v>33</v>
+      </c>
+      <c r="D188" t="s">
+        <v>87</v>
+      </c>
+      <c r="E188" t="s">
+        <v>54</v>
+      </c>
+      <c r="F188" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="189" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A189" t="s">
+        <v>32</v>
+      </c>
+      <c r="B189" t="s">
+        <v>33</v>
+      </c>
+      <c r="C189" t="s">
+        <v>215</v>
+      </c>
+      <c r="D189">
+        <v>1</v>
+      </c>
+      <c r="E189" t="s">
+        <v>54</v>
+      </c>
+      <c r="F189" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="190" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A190" t="s">
+        <v>32</v>
+      </c>
+      <c r="B190" t="s">
+        <v>33</v>
+      </c>
+      <c r="C190" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D190">
+        <v>1</v>
+      </c>
+      <c r="E190" t="s">
+        <v>54</v>
+      </c>
+      <c r="F190" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="191" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A191" t="s">
+        <v>32</v>
+      </c>
+      <c r="B191" t="s">
+        <v>33</v>
+      </c>
+      <c r="C191" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D191">
+        <v>1</v>
+      </c>
+      <c r="E191" t="s">
+        <v>54</v>
+      </c>
+      <c r="F191" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="192" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A192" t="s">
+        <v>32</v>
+      </c>
+      <c r="B192" t="s">
+        <v>33</v>
+      </c>
+      <c r="C192" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="E192" t="s">
+        <v>54</v>
+      </c>
+      <c r="F192" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="193" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A193" t="s">
+        <v>32</v>
+      </c>
+      <c r="B193" t="s">
+        <v>33</v>
+      </c>
+      <c r="C193" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="E193" t="s">
+        <v>54</v>
+      </c>
+      <c r="F193" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="194" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A194" t="s">
+        <v>32</v>
+      </c>
+      <c r="B194" t="s">
+        <v>182</v>
+      </c>
+      <c r="C194" s="1"/>
+      <c r="D194" t="s">
+        <v>68</v>
+      </c>
+      <c r="E194" t="s">
+        <v>116</v>
+      </c>
+      <c r="F194" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="195" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A195" t="s">
+        <v>32</v>
+      </c>
+      <c r="B195" t="s">
+        <v>88</v>
+      </c>
+      <c r="D195" t="s">
+        <v>65</v>
+      </c>
+      <c r="E195" t="s">
+        <v>24</v>
+      </c>
+      <c r="F195" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="196" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A196" t="s">
+        <v>32</v>
+      </c>
+      <c r="B196" t="s">
+        <v>226</v>
+      </c>
+      <c r="D196" t="s">
+        <v>65</v>
+      </c>
+      <c r="E196" t="s">
+        <v>225</v>
+      </c>
+      <c r="F196" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="197" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A197" t="s">
+        <v>32</v>
+      </c>
+      <c r="B197" t="s">
         <v>228</v>
       </c>
-      <c r="C174" s="2"/>
-      <c r="D174" t="s">
+      <c r="D197" t="s">
         <v>87</v>
       </c>
-      <c r="E174" s="2" t="s">
+      <c r="E197" t="s">
         <v>225</v>
       </c>
-      <c r="F174" s="2" t="s">
+      <c r="F197" t="s">
         <v>229</v>
       </c>
     </row>

</xml_diff>